<commit_message>
Atualizações nas pontuações da Anran, Emre, Domina, Mizuki e Jetpack Cat
</commit_message>
<xml_diff>
--- a/dist/OWPick/_internal/heroes ally.xlsx
+++ b/dist/OWPick/_internal/heroes ally.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DAVI\Projeto\Overwatch\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F2D71AF-FB3C-4331-8FAB-EF4A36D19420}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FEDA322-9302-4352-A258-94E05081D888}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="51">
   <si>
     <t>Hero</t>
   </si>
@@ -166,34 +166,7 @@
     <t>Emre</t>
   </si>
   <si>
-    <t>0.5</t>
-  </si>
-  <si>
-    <t>-0.5</t>
-  </si>
-  <si>
-    <t>1.5</t>
-  </si>
-  <si>
     <t>Mizuki</t>
-  </si>
-  <si>
-    <t>0.25</t>
-  </si>
-  <si>
-    <t>-0.75</t>
-  </si>
-  <si>
-    <t>-0.25</t>
-  </si>
-  <si>
-    <t>1.25</t>
-  </si>
-  <si>
-    <t>0.75</t>
-  </si>
-  <si>
-    <t>1.75</t>
   </si>
   <si>
     <t>Jetpack Cat</t>
@@ -530,7 +503,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>59</v>
+        <v>50</v>
       </c>
       <c r="K1" s="1" t="s">
         <v>9</v>
@@ -557,7 +530,7 @@
         <v>15</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>58</v>
+        <v>49</v>
       </c>
       <c r="T1" s="1" t="s">
         <v>16</v>
@@ -587,7 +560,7 @@
         <v>24</v>
       </c>
       <c r="AC1" s="1" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="AD1" s="1" t="s">
         <v>25</v>
@@ -741,8 +714,8 @@
       <c r="AB2" s="3">
         <v>1</v>
       </c>
-      <c r="AC2" s="3" t="s">
-        <v>52</v>
+      <c r="AC2" s="3">
+        <v>1</v>
       </c>
       <c r="AD2" s="3">
         <v>-1</v>
@@ -839,8 +812,8 @@
       <c r="I3" s="3">
         <v>1</v>
       </c>
-      <c r="J3" s="3" t="s">
-        <v>49</v>
+      <c r="J3" s="3">
+        <v>-1</v>
       </c>
       <c r="K3" s="3">
         <v>1</v>
@@ -849,7 +822,7 @@
         <v>1</v>
       </c>
       <c r="M3" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="N3" s="3">
         <v>0</v>
@@ -897,7 +870,7 @@
         <v>-1</v>
       </c>
       <c r="AC3" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AD3" s="3">
         <v>1</v>
@@ -974,7 +947,7 @@
         <v>-1</v>
       </c>
       <c r="C4" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="D4" s="3">
         <v>-11</v>
@@ -995,7 +968,7 @@
         <v>0</v>
       </c>
       <c r="J4" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K4" s="3">
         <v>-1</v>
@@ -1022,7 +995,7 @@
         <v>0</v>
       </c>
       <c r="S4" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="T4" s="3">
         <v>-1</v>
@@ -1052,7 +1025,7 @@
         <v>1</v>
       </c>
       <c r="AC4" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AD4" s="3">
         <v>-1</v>
@@ -1129,7 +1102,7 @@
         <v>1</v>
       </c>
       <c r="C5" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="D5" s="3">
         <v>0</v>
@@ -1149,8 +1122,8 @@
       <c r="I5" s="3">
         <v>0</v>
       </c>
-      <c r="J5" s="3" t="s">
-        <v>48</v>
+      <c r="J5" s="3">
+        <v>1</v>
       </c>
       <c r="K5" s="3">
         <v>-1</v>
@@ -1159,7 +1132,7 @@
         <v>-1</v>
       </c>
       <c r="M5" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N5" s="3">
         <v>0</v>
@@ -1206,8 +1179,8 @@
       <c r="AB5" s="3">
         <v>1</v>
       </c>
-      <c r="AC5" s="3" t="s">
-        <v>54</v>
+      <c r="AC5" s="3">
+        <v>-1</v>
       </c>
       <c r="AD5" s="3">
         <v>-1</v>
@@ -1284,7 +1257,7 @@
         <v>1</v>
       </c>
       <c r="C6" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="D6" s="3">
         <v>0</v>
@@ -1332,7 +1305,7 @@
         <v>1</v>
       </c>
       <c r="S6" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T6" s="3">
         <v>0</v>
@@ -1361,8 +1334,8 @@
       <c r="AB6" s="3">
         <v>1</v>
       </c>
-      <c r="AC6" s="3" t="s">
-        <v>56</v>
+      <c r="AC6" s="3">
+        <v>-1</v>
       </c>
       <c r="AD6" s="3">
         <v>0</v>
@@ -1459,8 +1432,8 @@
       <c r="I7" s="3">
         <v>0</v>
       </c>
-      <c r="J7" s="3" t="s">
-        <v>48</v>
+      <c r="J7" s="3">
+        <v>0</v>
       </c>
       <c r="K7" s="3">
         <v>1</v>
@@ -1469,7 +1442,7 @@
         <v>0</v>
       </c>
       <c r="M7" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="N7" s="3">
         <v>1</v>
@@ -1487,7 +1460,7 @@
         <v>0</v>
       </c>
       <c r="S7" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="T7" s="3">
         <v>-1</v>
@@ -1516,8 +1489,8 @@
       <c r="AB7" s="3">
         <v>-1</v>
       </c>
-      <c r="AC7" s="3" t="s">
-        <v>54</v>
+      <c r="AC7" s="3">
+        <v>-1</v>
       </c>
       <c r="AD7" s="3">
         <v>-1</v>
@@ -1594,7 +1567,7 @@
         <v>1</v>
       </c>
       <c r="C8" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="D8" s="3">
         <v>0</v>
@@ -1624,7 +1597,7 @@
         <v>-1</v>
       </c>
       <c r="M8" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N8" s="3">
         <v>-1</v>
@@ -1642,7 +1615,7 @@
         <v>1</v>
       </c>
       <c r="S8" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T8" s="3">
         <v>0</v>
@@ -1671,8 +1644,8 @@
       <c r="AB8" s="3">
         <v>1</v>
       </c>
-      <c r="AC8" s="3" t="s">
-        <v>54</v>
+      <c r="AC8" s="3">
+        <v>1</v>
       </c>
       <c r="AD8" s="3">
         <v>-1</v>
@@ -1749,7 +1722,7 @@
         <v>1</v>
       </c>
       <c r="C9" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D9" s="3">
         <v>0</v>
@@ -1827,7 +1800,7 @@
         <v>1</v>
       </c>
       <c r="AC9" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AD9" s="3">
         <v>1</v>
@@ -1898,28 +1871,28 @@
     </row>
     <row r="10" spans="1:51" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>59</v>
+        <v>50</v>
       </c>
       <c r="B10" s="3">
         <v>0</v>
       </c>
       <c r="C10" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="D10" s="3">
-        <v>0</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>48</v>
+        <v>1</v>
+      </c>
+      <c r="E10" s="3">
+        <v>1</v>
       </c>
       <c r="F10" s="3">
         <v>1</v>
       </c>
-      <c r="G10" s="3" t="s">
-        <v>48</v>
+      <c r="G10" s="3">
+        <v>0</v>
       </c>
       <c r="H10" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I10" s="3">
         <v>0</v>
@@ -1927,41 +1900,41 @@
       <c r="J10" s="3">
         <v>-11</v>
       </c>
-      <c r="K10" s="3" t="s">
-        <v>48</v>
+      <c r="K10" s="3">
+        <v>0</v>
       </c>
       <c r="L10" s="3">
         <v>1</v>
       </c>
-      <c r="M10" s="3" t="s">
-        <v>49</v>
+      <c r="M10" s="3">
+        <v>1</v>
       </c>
       <c r="N10" s="3">
         <v>0</v>
       </c>
       <c r="O10" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="P10" s="3">
         <v>1</v>
       </c>
-      <c r="Q10" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="R10" s="3" t="s">
-        <v>48</v>
+      <c r="Q10" s="3">
+        <v>-1</v>
+      </c>
+      <c r="R10" s="3">
+        <v>1</v>
       </c>
       <c r="S10" s="3">
-        <v>0</v>
-      </c>
-      <c r="T10" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="U10" s="3" t="s">
-        <v>48</v>
+        <v>-1</v>
+      </c>
+      <c r="T10" s="3">
+        <v>1</v>
+      </c>
+      <c r="U10" s="3">
+        <v>1</v>
       </c>
       <c r="V10" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="W10" s="3">
         <v>-1</v>
@@ -1972,26 +1945,26 @@
       <c r="Y10" s="3">
         <v>1</v>
       </c>
-      <c r="Z10" s="3" t="s">
-        <v>50</v>
+      <c r="Z10" s="3">
+        <v>1</v>
       </c>
       <c r="AA10" s="3">
         <v>1</v>
       </c>
-      <c r="AB10" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="AC10" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="AD10" s="3" t="s">
-        <v>49</v>
+      <c r="AB10" s="3">
+        <v>1</v>
+      </c>
+      <c r="AC10" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD10" s="3">
+        <v>-1</v>
       </c>
       <c r="AE10" s="3">
         <v>1</v>
       </c>
-      <c r="AF10" s="3" t="s">
-        <v>48</v>
+      <c r="AF10" s="3">
+        <v>0</v>
       </c>
       <c r="AG10" s="3">
         <v>1</v>
@@ -1999,23 +1972,23 @@
       <c r="AH10" s="3">
         <v>1</v>
       </c>
-      <c r="AI10" s="3" t="s">
-        <v>50</v>
+      <c r="AI10" s="3">
+        <v>1</v>
       </c>
       <c r="AJ10" s="3">
         <v>1</v>
       </c>
       <c r="AK10" s="3">
-        <v>1</v>
-      </c>
-      <c r="AL10" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="AM10" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="AN10" s="3" t="s">
-        <v>48</v>
+        <v>-1</v>
+      </c>
+      <c r="AL10" s="3">
+        <v>1</v>
+      </c>
+      <c r="AM10" s="3">
+        <v>0</v>
+      </c>
+      <c r="AN10" s="3">
+        <v>0</v>
       </c>
       <c r="AO10" s="3">
         <v>1</v>
@@ -2023,20 +1996,20 @@
       <c r="AP10" s="3">
         <v>1</v>
       </c>
-      <c r="AQ10" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="AR10" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="AS10" s="3" t="s">
-        <v>48</v>
+      <c r="AQ10" s="3">
+        <v>-1</v>
+      </c>
+      <c r="AR10" s="3">
+        <v>0</v>
+      </c>
+      <c r="AS10" s="3">
+        <v>-1</v>
       </c>
       <c r="AT10" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU10" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AV10" s="3">
         <v>1</v>
@@ -2047,8 +2020,8 @@
       <c r="AX10" s="3">
         <v>1</v>
       </c>
-      <c r="AY10" s="3" t="s">
-        <v>48</v>
+      <c r="AY10" s="3">
+        <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:51" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -2059,7 +2032,7 @@
         <v>1</v>
       </c>
       <c r="C11" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D11" s="3">
         <v>-1</v>
@@ -2079,8 +2052,8 @@
       <c r="I11" s="3">
         <v>1</v>
       </c>
-      <c r="J11" s="3" t="s">
-        <v>48</v>
+      <c r="J11" s="3">
+        <v>0</v>
       </c>
       <c r="K11" s="3">
         <v>-11</v>
@@ -2089,7 +2062,7 @@
         <v>1</v>
       </c>
       <c r="M11" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="N11" s="3">
         <v>1</v>
@@ -2214,7 +2187,7 @@
         <v>0</v>
       </c>
       <c r="C12" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D12" s="3">
         <v>-1</v>
@@ -2234,8 +2207,8 @@
       <c r="I12" s="3">
         <v>1</v>
       </c>
-      <c r="J12" s="3" t="s">
-        <v>48</v>
+      <c r="J12" s="3">
+        <v>0</v>
       </c>
       <c r="K12" s="3">
         <v>1</v>
@@ -2244,7 +2217,7 @@
         <v>-11</v>
       </c>
       <c r="M12" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="N12" s="3">
         <v>1</v>
@@ -2291,8 +2264,8 @@
       <c r="AB12" s="3">
         <v>1</v>
       </c>
-      <c r="AC12" s="3" t="s">
-        <v>53</v>
+      <c r="AC12" s="3">
+        <v>0</v>
       </c>
       <c r="AD12" s="3">
         <v>-1</v>
@@ -2366,154 +2339,154 @@
         <v>47</v>
       </c>
       <c r="B13" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C13" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="D13" s="3">
         <v>0</v>
       </c>
       <c r="E13" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F13" s="3">
         <v>-1</v>
       </c>
       <c r="G13" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H13" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="I13" s="3">
-        <v>1</v>
-      </c>
-      <c r="J13" s="3" t="s">
-        <v>49</v>
+        <v>0</v>
+      </c>
+      <c r="J13" s="3">
+        <v>1</v>
       </c>
       <c r="K13" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="L13" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="M13" s="3">
         <v>-11</v>
       </c>
       <c r="N13" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="O13" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="P13" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="Q13" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="R13" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="S13" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T13" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="U13" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="V13" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W13" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X13" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y13" s="3">
         <v>1</v>
       </c>
       <c r="Z13" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA13" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AB13" s="3">
         <v>1</v>
       </c>
       <c r="AC13" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AD13" s="3">
         <v>0</v>
       </c>
       <c r="AE13" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AF13" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AG13" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH13" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AI13" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AJ13" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AK13" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AL13" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AM13" s="3">
-        <v>-11</v>
+        <v>-1</v>
       </c>
       <c r="AN13" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AO13" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AP13" s="3">
         <v>-1</v>
       </c>
       <c r="AQ13" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AR13" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AS13" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AT13" s="3">
         <v>0</v>
       </c>
       <c r="AU13" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AV13" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AW13" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AX13" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AY13" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="14" spans="1:51" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -2554,7 +2527,7 @@
         <v>-1</v>
       </c>
       <c r="M14" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="N14" s="3">
         <v>-11</v>
@@ -2601,8 +2574,8 @@
       <c r="AB14" s="3">
         <v>1</v>
       </c>
-      <c r="AC14" s="3" t="s">
-        <v>53</v>
+      <c r="AC14" s="3">
+        <v>1</v>
       </c>
       <c r="AD14" s="3">
         <v>-1</v>
@@ -2679,7 +2652,7 @@
         <v>1</v>
       </c>
       <c r="C15" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D15" s="3">
         <v>-1</v>
@@ -2699,8 +2672,8 @@
       <c r="I15" s="3">
         <v>1</v>
       </c>
-      <c r="J15" s="3" t="s">
-        <v>49</v>
+      <c r="J15" s="3">
+        <v>-1</v>
       </c>
       <c r="K15" s="3">
         <v>2</v>
@@ -2709,7 +2682,7 @@
         <v>0</v>
       </c>
       <c r="M15" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="N15" s="3">
         <v>0</v>
@@ -2756,8 +2729,8 @@
       <c r="AB15" s="3">
         <v>-1</v>
       </c>
-      <c r="AC15" s="3" t="s">
-        <v>56</v>
+      <c r="AC15" s="3">
+        <v>1</v>
       </c>
       <c r="AD15" s="3">
         <v>0</v>
@@ -2834,7 +2807,7 @@
         <v>-1</v>
       </c>
       <c r="C16" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="D16" s="3">
         <v>1</v>
@@ -2854,8 +2827,8 @@
       <c r="I16" s="3">
         <v>1</v>
       </c>
-      <c r="J16" s="3" t="s">
-        <v>50</v>
+      <c r="J16" s="3">
+        <v>1</v>
       </c>
       <c r="K16" s="3">
         <v>-1</v>
@@ -2882,7 +2855,7 @@
         <v>1</v>
       </c>
       <c r="S16" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="T16" s="3">
         <v>0</v>
@@ -2911,8 +2884,8 @@
       <c r="AB16" s="3">
         <v>1</v>
       </c>
-      <c r="AC16" s="3" t="s">
-        <v>53</v>
+      <c r="AC16" s="3">
+        <v>1</v>
       </c>
       <c r="AD16" s="3">
         <v>-1</v>
@@ -2989,7 +2962,7 @@
         <v>1</v>
       </c>
       <c r="C17" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D17" s="3">
         <v>-1</v>
@@ -3010,7 +2983,7 @@
         <v>1</v>
       </c>
       <c r="J17" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="K17" s="3">
         <v>1</v>
@@ -3037,7 +3010,7 @@
         <v>-1</v>
       </c>
       <c r="S17" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T17" s="3">
         <v>0</v>
@@ -3067,7 +3040,7 @@
         <v>0</v>
       </c>
       <c r="AC17" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AD17" s="3">
         <v>0</v>
@@ -3144,7 +3117,7 @@
         <v>1</v>
       </c>
       <c r="C18" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="D18" s="3">
         <v>0</v>
@@ -3174,7 +3147,7 @@
         <v>-1</v>
       </c>
       <c r="M18" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="N18" s="3">
         <v>-1</v>
@@ -3192,7 +3165,7 @@
         <v>-11</v>
       </c>
       <c r="S18" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="T18" s="3">
         <v>0</v>
@@ -3221,8 +3194,8 @@
       <c r="AB18" s="3">
         <v>1</v>
       </c>
-      <c r="AC18" s="3" t="s">
-        <v>53</v>
+      <c r="AC18" s="3">
+        <v>0</v>
       </c>
       <c r="AD18" s="3">
         <v>0</v>
@@ -3293,34 +3266,34 @@
     </row>
     <row r="19" spans="1:51" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>58</v>
+        <v>49</v>
       </c>
       <c r="B19" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C19" s="3">
         <v>0</v>
       </c>
       <c r="D19" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="E19" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F19" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G19" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H19" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I19" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J19" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="K19" s="3">
         <v>0</v>
@@ -3329,7 +3302,7 @@
         <v>0</v>
       </c>
       <c r="M19" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N19" s="3">
         <v>0</v>
@@ -3338,25 +3311,25 @@
         <v>0</v>
       </c>
       <c r="P19" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="Q19" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R19" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="S19" s="3">
         <v>-11</v>
       </c>
       <c r="T19" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="U19" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="V19" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="W19" s="3">
         <v>0</v>
@@ -3368,40 +3341,40 @@
         <v>0</v>
       </c>
       <c r="Z19" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA19" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AB19" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AC19" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AD19" s="3">
         <v>0</v>
       </c>
       <c r="AE19" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF19" s="3">
         <v>0</v>
       </c>
       <c r="AG19" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH19" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI19" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AJ19" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AK19" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AL19" s="3">
         <v>0</v>
@@ -3413,22 +3386,22 @@
         <v>0</v>
       </c>
       <c r="AO19" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AP19" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AQ19" s="3">
         <v>0</v>
       </c>
       <c r="AR19" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS19" s="3">
         <v>0</v>
       </c>
       <c r="AT19" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AU19" s="3">
         <v>0</v>
@@ -3440,10 +3413,10 @@
         <v>0</v>
       </c>
       <c r="AX19" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AY19" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20" spans="1:51" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3484,7 +3457,7 @@
         <v>-1</v>
       </c>
       <c r="M20" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="N20" s="3">
         <v>0</v>
@@ -3502,7 +3475,7 @@
         <v>0</v>
       </c>
       <c r="S20" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T20" s="3">
         <v>-11</v>
@@ -3531,8 +3504,8 @@
       <c r="AB20" s="3">
         <v>0</v>
       </c>
-      <c r="AC20" s="3" t="s">
-        <v>56</v>
+      <c r="AC20" s="3">
+        <v>-1</v>
       </c>
       <c r="AD20" s="3">
         <v>0</v>
@@ -3609,7 +3582,7 @@
         <v>-1</v>
       </c>
       <c r="C21" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="D21" s="3">
         <v>1</v>
@@ -3629,8 +3602,8 @@
       <c r="I21" s="3">
         <v>0</v>
       </c>
-      <c r="J21" s="3" t="s">
-        <v>48</v>
+      <c r="J21" s="3">
+        <v>1</v>
       </c>
       <c r="K21" s="3">
         <v>-1</v>
@@ -3639,7 +3612,7 @@
         <v>-1</v>
       </c>
       <c r="M21" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="N21" s="3">
         <v>-1</v>
@@ -3657,7 +3630,7 @@
         <v>1</v>
       </c>
       <c r="S21" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="T21" s="3">
         <v>0</v>
@@ -3686,8 +3659,8 @@
       <c r="AB21" s="3">
         <v>1</v>
       </c>
-      <c r="AC21" s="3" t="s">
-        <v>53</v>
+      <c r="AC21" s="3">
+        <v>0</v>
       </c>
       <c r="AD21" s="3">
         <v>0</v>
@@ -3784,8 +3757,8 @@
       <c r="I22" s="3">
         <v>1</v>
       </c>
-      <c r="J22" s="3" t="s">
-        <v>48</v>
+      <c r="J22" s="3">
+        <v>-1</v>
       </c>
       <c r="K22" s="3">
         <v>0</v>
@@ -3794,7 +3767,7 @@
         <v>0</v>
       </c>
       <c r="M22" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N22" s="3">
         <v>0</v>
@@ -3812,7 +3785,7 @@
         <v>-1</v>
       </c>
       <c r="S22" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="T22" s="3">
         <v>2</v>
@@ -3842,7 +3815,7 @@
         <v>-1</v>
       </c>
       <c r="AC22" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AD22" s="3">
         <v>0</v>
@@ -3919,7 +3892,7 @@
         <v>1</v>
       </c>
       <c r="C23" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D23" s="3">
         <v>-1</v>
@@ -3949,7 +3922,7 @@
         <v>0</v>
       </c>
       <c r="M23" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N23" s="3">
         <v>1</v>
@@ -3967,7 +3940,7 @@
         <v>0</v>
       </c>
       <c r="S23" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T23" s="3">
         <v>0</v>
@@ -3997,7 +3970,7 @@
         <v>0</v>
       </c>
       <c r="AC23" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AD23" s="3">
         <v>0</v>
@@ -4074,7 +4047,7 @@
         <v>1</v>
       </c>
       <c r="C24" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="D24" s="3">
         <v>0</v>
@@ -4094,8 +4067,8 @@
       <c r="I24" s="3">
         <v>-1</v>
       </c>
-      <c r="J24" s="3" t="s">
-        <v>48</v>
+      <c r="J24" s="3">
+        <v>1</v>
       </c>
       <c r="K24" s="3">
         <v>-1</v>
@@ -4104,7 +4077,7 @@
         <v>-1</v>
       </c>
       <c r="M24" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N24" s="3">
         <v>0</v>
@@ -4229,7 +4202,7 @@
         <v>0</v>
       </c>
       <c r="C25" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D25" s="3">
         <v>-1</v>
@@ -4259,7 +4232,7 @@
         <v>0</v>
       </c>
       <c r="M25" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="N25" s="3">
         <v>0</v>
@@ -4307,7 +4280,7 @@
         <v>-1</v>
       </c>
       <c r="AC25" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AD25" s="3">
         <v>1</v>
@@ -4384,7 +4357,7 @@
         <v>1</v>
       </c>
       <c r="C26" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D26" s="3">
         <v>0</v>
@@ -4432,7 +4405,7 @@
         <v>0</v>
       </c>
       <c r="S26" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T26" s="3">
         <v>0</v>
@@ -4461,8 +4434,8 @@
       <c r="AB26" s="3">
         <v>0</v>
       </c>
-      <c r="AC26" s="3" t="s">
-        <v>56</v>
+      <c r="AC26" s="3">
+        <v>-1</v>
       </c>
       <c r="AD26" s="3">
         <v>0</v>
@@ -4539,7 +4512,7 @@
         <v>0</v>
       </c>
       <c r="C27" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="D27" s="3">
         <v>0</v>
@@ -4569,7 +4542,7 @@
         <v>-1</v>
       </c>
       <c r="M27" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="N27" s="3">
         <v>-1</v>
@@ -4587,7 +4560,7 @@
         <v>1</v>
       </c>
       <c r="S27" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T27" s="3">
         <v>1</v>
@@ -4616,8 +4589,8 @@
       <c r="AB27" s="3">
         <v>0</v>
       </c>
-      <c r="AC27" s="3" t="s">
-        <v>48</v>
+      <c r="AC27" s="3">
+        <v>0</v>
       </c>
       <c r="AD27" s="3">
         <v>1</v>
@@ -4694,7 +4667,7 @@
         <v>1</v>
       </c>
       <c r="C28" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="D28" s="3">
         <v>2</v>
@@ -4742,7 +4715,7 @@
         <v>1</v>
       </c>
       <c r="S28" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T28" s="3">
         <v>0</v>
@@ -4771,8 +4744,8 @@
       <c r="AB28" s="3">
         <v>-11</v>
       </c>
-      <c r="AC28" s="3" t="s">
-        <v>53</v>
+      <c r="AC28" s="3">
+        <v>-1</v>
       </c>
       <c r="AD28" s="3">
         <v>-1</v>
@@ -4843,34 +4816,34 @@
     </row>
     <row r="29" spans="1:51" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="B29" s="3" t="s">
-        <v>52</v>
+        <v>48</v>
+      </c>
+      <c r="B29" s="3">
+        <v>1</v>
       </c>
       <c r="C29" s="3">
         <v>0</v>
       </c>
       <c r="D29" s="3">
-        <v>-1</v>
-      </c>
-      <c r="E29" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="F29" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="G29" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="H29" s="3" t="s">
-        <v>48</v>
+        <v>1</v>
+      </c>
+      <c r="E29" s="3">
+        <v>-1</v>
+      </c>
+      <c r="F29" s="3">
+        <v>-1</v>
+      </c>
+      <c r="G29" s="3">
+        <v>-1</v>
+      </c>
+      <c r="H29" s="3">
+        <v>-1</v>
       </c>
       <c r="I29" s="3">
-        <v>1</v>
-      </c>
-      <c r="J29" s="3" t="s">
-        <v>48</v>
+        <v>0</v>
+      </c>
+      <c r="J29" s="3">
+        <v>0</v>
       </c>
       <c r="K29" s="3">
         <v>1</v>
@@ -4879,106 +4852,106 @@
         <v>0</v>
       </c>
       <c r="M29" s="3">
-        <v>1</v>
-      </c>
-      <c r="N29" s="3" t="s">
-        <v>52</v>
+        <v>-1</v>
+      </c>
+      <c r="N29" s="3">
+        <v>1</v>
       </c>
       <c r="O29" s="3">
         <v>1</v>
       </c>
-      <c r="P29" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="Q29" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="R29" s="3" t="s">
-        <v>53</v>
+      <c r="P29" s="3">
+        <v>1</v>
+      </c>
+      <c r="Q29" s="3">
+        <v>0</v>
+      </c>
+      <c r="R29" s="3">
+        <v>0</v>
       </c>
       <c r="S29" s="3">
-        <v>0</v>
-      </c>
-      <c r="T29" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="U29" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="V29" s="3" t="s">
-        <v>52</v>
+        <v>2</v>
+      </c>
+      <c r="T29" s="3">
+        <v>-1</v>
+      </c>
+      <c r="U29" s="3">
+        <v>0</v>
+      </c>
+      <c r="V29" s="3">
+        <v>2</v>
       </c>
       <c r="W29" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="X29" s="3">
         <v>-1</v>
       </c>
       <c r="Y29" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z29" s="3">
-        <v>1</v>
-      </c>
-      <c r="AA29" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="AB29" s="3" t="s">
-        <v>53</v>
+        <v>-1</v>
+      </c>
+      <c r="AA29" s="3">
+        <v>0</v>
+      </c>
+      <c r="AB29" s="3">
+        <v>-1</v>
       </c>
       <c r="AC29" s="3">
         <v>-11</v>
       </c>
-      <c r="AD29" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="AE29" s="3" t="s">
-        <v>56</v>
+      <c r="AD29" s="3">
+        <v>-1</v>
+      </c>
+      <c r="AE29" s="3">
+        <v>-1</v>
       </c>
       <c r="AF29" s="3">
         <v>0</v>
       </c>
-      <c r="AG29" s="3" t="s">
-        <v>57</v>
+      <c r="AG29" s="3">
+        <v>-1</v>
       </c>
       <c r="AH29" s="3">
-        <v>1</v>
-      </c>
-      <c r="AI29" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="AJ29" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="AK29" s="3" t="s">
-        <v>48</v>
+        <v>0</v>
+      </c>
+      <c r="AI29" s="3">
+        <v>-1</v>
+      </c>
+      <c r="AJ29" s="3">
+        <v>0</v>
+      </c>
+      <c r="AK29" s="3">
+        <v>0</v>
       </c>
       <c r="AL29" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AM29" s="3">
-        <v>1</v>
-      </c>
-      <c r="AN29" s="3" t="s">
-        <v>52</v>
+        <v>0</v>
+      </c>
+      <c r="AN29" s="3">
+        <v>0</v>
       </c>
       <c r="AO29" s="3">
-        <v>1</v>
-      </c>
-      <c r="AP29" s="3" t="s">
-        <v>54</v>
+        <v>0</v>
+      </c>
+      <c r="AP29" s="3">
+        <v>0</v>
       </c>
       <c r="AQ29" s="3">
-        <v>1</v>
-      </c>
-      <c r="AR29" s="3" t="s">
-        <v>50</v>
+        <v>0</v>
+      </c>
+      <c r="AR29" s="3">
+        <v>2</v>
       </c>
       <c r="AS29" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AT29" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AU29" s="3">
         <v>1</v>
@@ -4986,14 +4959,14 @@
       <c r="AV29" s="3">
         <v>1</v>
       </c>
-      <c r="AW29" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="AX29" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="AY29" s="3" t="s">
-        <v>49</v>
+      <c r="AW29" s="3">
+        <v>-1</v>
+      </c>
+      <c r="AX29" s="3">
+        <v>1</v>
+      </c>
+      <c r="AY29" s="3">
+        <v>1</v>
       </c>
     </row>
     <row r="30" spans="1:51" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -5004,7 +4977,7 @@
         <v>-1</v>
       </c>
       <c r="C30" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D30" s="3">
         <v>-1</v>
@@ -5024,8 +4997,8 @@
       <c r="I30" s="3">
         <v>1</v>
       </c>
-      <c r="J30" s="3" t="s">
-        <v>49</v>
+      <c r="J30" s="3">
+        <v>-1</v>
       </c>
       <c r="K30" s="3">
         <v>1</v>
@@ -5081,8 +5054,8 @@
       <c r="AB30" s="3">
         <v>-1</v>
       </c>
-      <c r="AC30" s="3" t="s">
-        <v>56</v>
+      <c r="AC30" s="3">
+        <v>-1</v>
       </c>
       <c r="AD30" s="3">
         <v>-11</v>
@@ -5179,8 +5152,8 @@
       <c r="I31" s="3">
         <v>-1</v>
       </c>
-      <c r="J31" s="3" t="s">
-        <v>50</v>
+      <c r="J31" s="3">
+        <v>2</v>
       </c>
       <c r="K31" s="3">
         <v>-1</v>
@@ -5207,7 +5180,7 @@
         <v>1</v>
       </c>
       <c r="S31" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T31" s="3">
         <v>-1</v>
@@ -5236,8 +5209,8 @@
       <c r="AB31" s="3">
         <v>0</v>
       </c>
-      <c r="AC31" s="3" t="s">
-        <v>56</v>
+      <c r="AC31" s="3">
+        <v>-1</v>
       </c>
       <c r="AD31" s="3">
         <v>0</v>
@@ -5314,7 +5287,7 @@
         <v>0</v>
       </c>
       <c r="C32" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D32" s="3">
         <v>-1</v>
@@ -5334,8 +5307,8 @@
       <c r="I32" s="3">
         <v>1</v>
       </c>
-      <c r="J32" s="3" t="s">
-        <v>48</v>
+      <c r="J32" s="3">
+        <v>1</v>
       </c>
       <c r="K32" s="3">
         <v>1</v>
@@ -5344,7 +5317,7 @@
         <v>1</v>
       </c>
       <c r="M32" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="N32" s="3">
         <v>1</v>
@@ -5391,8 +5364,8 @@
       <c r="AB32" s="3">
         <v>1</v>
       </c>
-      <c r="AC32" s="3" t="s">
-        <v>53</v>
+      <c r="AC32" s="3">
+        <v>0</v>
       </c>
       <c r="AD32" s="3">
         <v>-1</v>
@@ -5499,7 +5472,7 @@
         <v>0</v>
       </c>
       <c r="M33" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N33" s="3">
         <v>-1</v>
@@ -5517,7 +5490,7 @@
         <v>0</v>
       </c>
       <c r="S33" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T33" s="3">
         <v>1</v>
@@ -5546,8 +5519,8 @@
       <c r="AB33" s="3">
         <v>0</v>
       </c>
-      <c r="AC33" s="3" t="s">
-        <v>56</v>
+      <c r="AC33" s="3">
+        <v>-1</v>
       </c>
       <c r="AD33" s="3">
         <v>0</v>
@@ -5654,7 +5627,7 @@
         <v>1</v>
       </c>
       <c r="M34" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="N34" s="3">
         <v>0</v>
@@ -5672,7 +5645,7 @@
         <v>0</v>
       </c>
       <c r="S34" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T34" s="3">
         <v>1</v>
@@ -5702,7 +5675,7 @@
         <v>0</v>
       </c>
       <c r="AC34" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AD34" s="3">
         <v>1</v>
@@ -5779,7 +5752,7 @@
         <v>1</v>
       </c>
       <c r="C35" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="D35" s="3">
         <v>0</v>
@@ -5799,8 +5772,8 @@
       <c r="I35" s="3">
         <v>1</v>
       </c>
-      <c r="J35" s="3" t="s">
-        <v>50</v>
+      <c r="J35" s="3">
+        <v>1</v>
       </c>
       <c r="K35" s="3">
         <v>-1</v>
@@ -5809,7 +5782,7 @@
         <v>-1</v>
       </c>
       <c r="M35" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N35" s="3">
         <v>-1</v>
@@ -5827,7 +5800,7 @@
         <v>0</v>
       </c>
       <c r="S35" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T35" s="3">
         <v>0</v>
@@ -5856,8 +5829,8 @@
       <c r="AB35" s="3">
         <v>-1</v>
       </c>
-      <c r="AC35" s="3" t="s">
-        <v>56</v>
+      <c r="AC35" s="3">
+        <v>-1</v>
       </c>
       <c r="AD35" s="3">
         <v>0</v>
@@ -5934,7 +5907,7 @@
         <v>0</v>
       </c>
       <c r="C36" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="D36" s="3">
         <v>0</v>
@@ -5964,7 +5937,7 @@
         <v>-1</v>
       </c>
       <c r="M36" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="N36" s="3">
         <v>-1</v>
@@ -5982,7 +5955,7 @@
         <v>1</v>
       </c>
       <c r="S36" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="T36" s="3">
         <v>-1</v>
@@ -6011,8 +5984,8 @@
       <c r="AB36" s="3">
         <v>1</v>
       </c>
-      <c r="AC36" s="3" t="s">
-        <v>56</v>
+      <c r="AC36" s="3">
+        <v>0</v>
       </c>
       <c r="AD36" s="3">
         <v>-1</v>
@@ -6089,7 +6062,7 @@
         <v>0</v>
       </c>
       <c r="C37" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="D37" s="3">
         <v>1</v>
@@ -6110,7 +6083,7 @@
         <v>0</v>
       </c>
       <c r="J37" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="K37" s="3">
         <v>0</v>
@@ -6119,7 +6092,7 @@
         <v>1</v>
       </c>
       <c r="M37" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N37" s="3">
         <v>0</v>
@@ -6137,7 +6110,7 @@
         <v>1</v>
       </c>
       <c r="S37" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="T37" s="3">
         <v>1</v>
@@ -6166,8 +6139,8 @@
       <c r="AB37" s="3">
         <v>1</v>
       </c>
-      <c r="AC37" s="3" t="s">
-        <v>48</v>
+      <c r="AC37" s="3">
+        <v>0</v>
       </c>
       <c r="AD37" s="3">
         <v>-1</v>
@@ -6244,7 +6217,7 @@
         <v>-1</v>
       </c>
       <c r="C38" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D38" s="3">
         <v>0</v>
@@ -6264,8 +6237,8 @@
       <c r="I38" s="3">
         <v>1</v>
       </c>
-      <c r="J38" s="3" t="s">
-        <v>49</v>
+      <c r="J38" s="3">
+        <v>0</v>
       </c>
       <c r="K38" s="3">
         <v>1</v>
@@ -6274,7 +6247,7 @@
         <v>1</v>
       </c>
       <c r="M38" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="N38" s="3">
         <v>0</v>
@@ -6322,7 +6295,7 @@
         <v>1</v>
       </c>
       <c r="AC38" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AD38" s="3">
         <v>0</v>
@@ -6399,7 +6372,7 @@
         <v>0</v>
       </c>
       <c r="C39" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D39" s="3">
         <v>0</v>
@@ -6419,8 +6392,8 @@
       <c r="I39" s="3">
         <v>1</v>
       </c>
-      <c r="J39" s="3" t="s">
-        <v>49</v>
+      <c r="J39" s="3">
+        <v>0</v>
       </c>
       <c r="K39" s="3">
         <v>1</v>
@@ -6429,7 +6402,7 @@
         <v>1</v>
       </c>
       <c r="M39" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="N39" s="3">
         <v>0</v>
@@ -6477,7 +6450,7 @@
         <v>1</v>
       </c>
       <c r="AC39" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AD39" s="3">
         <v>0</v>
@@ -6554,7 +6527,7 @@
         <v>0</v>
       </c>
       <c r="C40" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D40" s="3">
         <v>-1</v>
@@ -6584,7 +6557,7 @@
         <v>1</v>
       </c>
       <c r="M40" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N40" s="3">
         <v>1</v>
@@ -6631,8 +6604,8 @@
       <c r="AB40" s="3">
         <v>-1</v>
       </c>
-      <c r="AC40" s="3" t="s">
-        <v>52</v>
+      <c r="AC40" s="3">
+        <v>0</v>
       </c>
       <c r="AD40" s="3">
         <v>1</v>
@@ -6709,7 +6682,7 @@
         <v>1</v>
       </c>
       <c r="C41" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="D41" s="3">
         <v>0</v>
@@ -6739,7 +6712,7 @@
         <v>-1</v>
       </c>
       <c r="M41" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N41" s="3">
         <v>-1</v>
@@ -6757,7 +6730,7 @@
         <v>1</v>
       </c>
       <c r="S41" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T41" s="3">
         <v>1</v>
@@ -6786,8 +6759,8 @@
       <c r="AB41" s="3">
         <v>0</v>
       </c>
-      <c r="AC41" s="3" t="s">
-        <v>48</v>
+      <c r="AC41" s="3">
+        <v>0</v>
       </c>
       <c r="AD41" s="3">
         <v>1</v>
@@ -6864,7 +6837,7 @@
         <v>-1</v>
       </c>
       <c r="C42" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="D42" s="3">
         <v>1</v>
@@ -6884,8 +6857,8 @@
       <c r="I42" s="3">
         <v>-1</v>
       </c>
-      <c r="J42" s="3" t="s">
-        <v>48</v>
+      <c r="J42" s="3">
+        <v>1</v>
       </c>
       <c r="K42" s="3">
         <v>-1</v>
@@ -6894,7 +6867,7 @@
         <v>-1</v>
       </c>
       <c r="M42" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="N42" s="3">
         <v>-1</v>
@@ -6912,7 +6885,7 @@
         <v>1</v>
       </c>
       <c r="S42" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="T42" s="3">
         <v>0</v>
@@ -6941,8 +6914,8 @@
       <c r="AB42" s="3">
         <v>0</v>
       </c>
-      <c r="AC42" s="3" t="s">
-        <v>54</v>
+      <c r="AC42" s="3">
+        <v>0</v>
       </c>
       <c r="AD42" s="3">
         <v>0</v>
@@ -7019,7 +6992,7 @@
         <v>0</v>
       </c>
       <c r="C43" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="D43" s="3">
         <v>-1</v>
@@ -7039,8 +7012,8 @@
       <c r="I43" s="3">
         <v>1</v>
       </c>
-      <c r="J43" s="3" t="s">
-        <v>49</v>
+      <c r="J43" s="3">
+        <v>-1</v>
       </c>
       <c r="K43" s="3">
         <v>1</v>
@@ -7049,7 +7022,7 @@
         <v>1</v>
       </c>
       <c r="M43" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="N43" s="3">
         <v>0</v>
@@ -7097,7 +7070,7 @@
         <v>-1</v>
       </c>
       <c r="AC43" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AD43" s="3">
         <v>1</v>
@@ -7174,7 +7147,7 @@
         <v>1</v>
       </c>
       <c r="C44" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D44" s="3">
         <v>0</v>
@@ -7194,8 +7167,8 @@
       <c r="I44" s="3">
         <v>1</v>
       </c>
-      <c r="J44" s="3" t="s">
-        <v>50</v>
+      <c r="J44" s="3">
+        <v>0</v>
       </c>
       <c r="K44" s="3">
         <v>-1</v>
@@ -7204,7 +7177,7 @@
         <v>-1</v>
       </c>
       <c r="M44" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="N44" s="3">
         <v>-1</v>
@@ -7222,7 +7195,7 @@
         <v>0</v>
       </c>
       <c r="S44" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T44" s="3">
         <v>0</v>
@@ -7251,8 +7224,8 @@
       <c r="AB44" s="3">
         <v>-1</v>
       </c>
-      <c r="AC44" s="3" t="s">
-        <v>56</v>
+      <c r="AC44" s="3">
+        <v>1</v>
       </c>
       <c r="AD44" s="3">
         <v>0</v>
@@ -7329,7 +7302,7 @@
         <v>-1</v>
       </c>
       <c r="C45" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D45" s="3">
         <v>-1</v>
@@ -7350,7 +7323,7 @@
         <v>1</v>
       </c>
       <c r="J45" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="K45" s="3">
         <v>1</v>
@@ -7359,7 +7332,7 @@
         <v>1</v>
       </c>
       <c r="M45" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="N45" s="3">
         <v>0</v>
@@ -7407,7 +7380,7 @@
         <v>-1</v>
       </c>
       <c r="AC45" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AD45" s="3">
         <v>0</v>
@@ -7505,7 +7478,7 @@
         <v>1</v>
       </c>
       <c r="J46" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K46" s="3">
         <v>0</v>
@@ -7532,7 +7505,7 @@
         <v>1</v>
       </c>
       <c r="S46" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="T46" s="3">
         <v>-1</v>
@@ -7562,7 +7535,7 @@
         <v>1</v>
       </c>
       <c r="AC46" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AD46" s="3">
         <v>-1</v>
@@ -7639,7 +7612,7 @@
         <v>1</v>
       </c>
       <c r="C47" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D47" s="3">
         <v>-1</v>
@@ -7660,7 +7633,7 @@
         <v>2</v>
       </c>
       <c r="J47" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K47" s="3">
         <v>1</v>
@@ -7669,7 +7642,7 @@
         <v>1</v>
       </c>
       <c r="M47" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="N47" s="3">
         <v>1</v>
@@ -7717,7 +7690,7 @@
         <v>1</v>
       </c>
       <c r="AC47" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AD47" s="3">
         <v>1</v>
@@ -7794,7 +7767,7 @@
         <v>0</v>
       </c>
       <c r="C48" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D48" s="3">
         <v>-1</v>
@@ -7824,7 +7797,7 @@
         <v>1</v>
       </c>
       <c r="M48" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="N48" s="3">
         <v>1</v>
@@ -7949,7 +7922,7 @@
         <v>1</v>
       </c>
       <c r="C49" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D49" s="3">
         <v>1</v>
@@ -7979,7 +7952,7 @@
         <v>3</v>
       </c>
       <c r="M49" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N49" s="3">
         <v>2</v>
@@ -8026,8 +7999,8 @@
       <c r="AB49" s="3">
         <v>1</v>
       </c>
-      <c r="AC49" s="3" t="s">
-        <v>48</v>
+      <c r="AC49" s="3">
+        <v>-1</v>
       </c>
       <c r="AD49" s="3">
         <v>-1</v>
@@ -8134,7 +8107,7 @@
         <v>1</v>
       </c>
       <c r="M50" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="N50" s="3">
         <v>0</v>
@@ -8152,7 +8125,7 @@
         <v>0</v>
       </c>
       <c r="S50" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T50" s="3">
         <v>2</v>
@@ -8181,8 +8154,8 @@
       <c r="AB50" s="3">
         <v>0</v>
       </c>
-      <c r="AC50" s="3" t="s">
-        <v>48</v>
+      <c r="AC50" s="3">
+        <v>1</v>
       </c>
       <c r="AD50" s="3">
         <v>0</v>
@@ -8259,7 +8232,7 @@
         <v>0</v>
       </c>
       <c r="C51" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D51" s="3">
         <v>1</v>
@@ -8289,7 +8262,7 @@
         <v>1</v>
       </c>
       <c r="M51" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N51" s="3">
         <v>1</v>
@@ -8336,8 +8309,8 @@
       <c r="AB51" s="3">
         <v>-1</v>
       </c>
-      <c r="AC51" s="3" t="s">
-        <v>49</v>
+      <c r="AC51" s="3">
+        <v>0</v>
       </c>
       <c r="AD51" s="3">
         <v>0</v>

</xml_diff>

<commit_message>
Correção de bugs na remoção de pontuação dos mapas
</commit_message>
<xml_diff>
--- a/dist/OWPick/_internal/heroes ally.xlsx
+++ b/dist/OWPick/_internal/heroes ally.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DAVI\Projeto\Overwatch\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FEDA322-9302-4352-A258-94E05081D888}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74646E1F-87AB-4551-99C8-B4BDC23E260F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1210,7 +1210,7 @@
         <v>0</v>
       </c>
       <c r="AM5" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AN5" s="3">
         <v>-1</v>
@@ -1243,7 +1243,7 @@
         <v>1</v>
       </c>
       <c r="AX5" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AY5" s="3">
         <v>1</v>

</xml_diff>

<commit_message>
Adaptações para a nova Season
</commit_message>
<xml_diff>
--- a/dist/OWPick/_internal/heroes ally.xlsx
+++ b/dist/OWPick/_internal/heroes ally.xlsx
@@ -125,6 +125,9 @@
   </si>
   <si>
     <t>Roadhog</t>
+  </si>
+  <si>
+    <t>Sierra</t>
   </si>
   <si>
     <t>Sigma</t>
@@ -609,6 +612,9 @@
       <c r="AY1" s="1" t="s">
         <v>50</v>
       </c>
+      <c r="AZ1" s="1" t="s">
+        <v>51</v>
+      </c>
     </row>
     <row r="2" ht="15.75" customHeight="1">
       <c r="A2" s="2" t="s">
@@ -723,16 +729,16 @@
         <v>0</v>
       </c>
       <c r="AL2" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AM2" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AN2" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AO2" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AP2" s="3">
         <v>0</v>
@@ -741,13 +747,13 @@
         <v>0</v>
       </c>
       <c r="AR2" s="3">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="AS2" s="3">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="AT2" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AU2" s="3">
         <v>0</v>
@@ -756,12 +762,15 @@
         <v>0</v>
       </c>
       <c r="AW2" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AX2" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AY2" s="3">
+        <v>0</v>
+      </c>
+      <c r="AZ2" s="3">
         <v>0</v>
       </c>
     </row>
@@ -878,16 +887,16 @@
         <v>0</v>
       </c>
       <c r="AL3" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AM3" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AN3" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AO3" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AP3" s="3">
         <v>-1</v>
@@ -896,27 +905,30 @@
         <v>-1</v>
       </c>
       <c r="AR3" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AS3" s="3">
         <v>1</v>
       </c>
       <c r="AT3" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU3" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AV3" s="3">
         <v>1</v>
       </c>
       <c r="AW3" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AX3" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AY3" s="3">
+        <v>1</v>
+      </c>
+      <c r="AZ3" s="3">
         <v>0</v>
       </c>
     </row>
@@ -1030,48 +1042,51 @@
         <v>1</v>
       </c>
       <c r="AK4" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AL4" s="3">
-        <v>-2</v>
+        <v>2</v>
       </c>
       <c r="AM4" s="3">
         <v>-2</v>
       </c>
       <c r="AN4" s="3">
-        <v>1</v>
+        <v>-2</v>
       </c>
       <c r="AO4" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AP4" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AQ4" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AR4" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AS4" s="3">
         <v>1</v>
       </c>
       <c r="AT4" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AU4" s="3">
         <v>-1</v>
       </c>
       <c r="AV4" s="3">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="AW4" s="3">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AX4" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AY4" s="3">
+        <v>1</v>
+      </c>
+      <c r="AZ4" s="3">
         <v>1</v>
       </c>
     </row>
@@ -1185,48 +1200,51 @@
         <v>1</v>
       </c>
       <c r="AK5" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AL5" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AM5" s="3">
-        <v>-2</v>
+        <v>1</v>
       </c>
       <c r="AN5" s="3">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="AO5" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AP5" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AQ5" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AR5" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="3">
         <v>0</v>
       </c>
       <c r="AT5" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AU5" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AV5" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AW5" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AX5" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AY5" s="3">
+        <v>0</v>
+      </c>
+      <c r="AZ5" s="3">
         <v>1</v>
       </c>
     </row>
@@ -1340,48 +1358,51 @@
         <v>0</v>
       </c>
       <c r="AK6" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AL6" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AM6" s="3">
-        <v>2</v>
+        <v>-1</v>
       </c>
       <c r="AN6" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AO6" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AP6" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AQ6" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AR6" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AS6" s="3">
         <v>-1</v>
       </c>
       <c r="AT6" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AU6" s="3">
         <v>0</v>
       </c>
       <c r="AV6" s="3">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="AW6" s="3">
         <v>-2</v>
       </c>
       <c r="AX6" s="3">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AY6" s="3">
+        <v>0</v>
+      </c>
+      <c r="AZ6" s="3">
         <v>0</v>
       </c>
     </row>
@@ -1495,48 +1516,51 @@
         <v>-1</v>
       </c>
       <c r="AK7" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AL7" s="3">
         <v>-1</v>
       </c>
       <c r="AM7" s="3">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="AN7" s="3">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AO7" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AP7" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AQ7" s="3">
         <v>0</v>
       </c>
       <c r="AR7" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AS7" s="3">
         <v>2</v>
       </c>
       <c r="AT7" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AU7" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AV7" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AW7" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AX7" s="3">
         <v>-1</v>
       </c>
       <c r="AY7" s="3">
+        <v>-1</v>
+      </c>
+      <c r="AZ7" s="3">
         <v>-2</v>
       </c>
     </row>
@@ -1653,19 +1677,19 @@
         <v>0</v>
       </c>
       <c r="AL8" s="3">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="AM8" s="3">
         <v>-2</v>
       </c>
       <c r="AN8" s="3">
-        <v>1</v>
+        <v>-2</v>
       </c>
       <c r="AO8" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AP8" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AQ8" s="3">
         <v>1</v>
@@ -1677,21 +1701,24 @@
         <v>1</v>
       </c>
       <c r="AT8" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU8" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AV8" s="3">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="AW8" s="3">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AX8" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AY8" s="3">
+        <v>1</v>
+      </c>
+      <c r="AZ8" s="3">
         <v>1</v>
       </c>
     </row>
@@ -1808,16 +1835,16 @@
         <v>0</v>
       </c>
       <c r="AL9" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AM9" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AN9" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AO9" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AP9" s="3">
         <v>0</v>
@@ -1826,16 +1853,16 @@
         <v>0</v>
       </c>
       <c r="AR9" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AS9" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AT9" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU9" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AV9" s="3">
         <v>1</v>
@@ -1844,9 +1871,12 @@
         <v>1</v>
       </c>
       <c r="AX9" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AY9" s="3">
+        <v>0</v>
+      </c>
+      <c r="AZ9" s="3">
         <v>-2</v>
       </c>
     </row>
@@ -1960,19 +1990,19 @@
         <v>1</v>
       </c>
       <c r="AK10" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AL10" s="3">
         <v>-1</v>
       </c>
       <c r="AM10" s="3">
-        <v>2</v>
+        <v>-1</v>
       </c>
       <c r="AN10" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AO10" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AP10" s="3">
         <v>1</v>
@@ -1981,27 +2011,30 @@
         <v>1</v>
       </c>
       <c r="AR10" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS10" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AT10" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AU10" s="3">
         <v>0</v>
       </c>
       <c r="AV10" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AW10" s="3">
         <v>1</v>
       </c>
       <c r="AX10" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AY10" s="3">
+        <v>0</v>
+      </c>
+      <c r="AZ10" s="3">
         <v>-1</v>
       </c>
     </row>
@@ -2118,22 +2151,22 @@
         <v>0</v>
       </c>
       <c r="AL11" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AM11" s="3">
-        <v>-2</v>
+        <v>1</v>
       </c>
       <c r="AN11" s="3">
-        <v>1</v>
+        <v>-2</v>
       </c>
       <c r="AO11" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AP11" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AQ11" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AR11" s="3">
         <v>1</v>
@@ -2142,21 +2175,24 @@
         <v>1</v>
       </c>
       <c r="AT11" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU11" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AV11" s="3">
         <v>1</v>
       </c>
       <c r="AW11" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AX11" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AY11" s="3">
+        <v>0</v>
+      </c>
+      <c r="AZ11" s="3">
         <v>1</v>
       </c>
     </row>
@@ -2270,48 +2306,51 @@
         <v>1</v>
       </c>
       <c r="AK12" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AL12" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AM12" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AN12" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AO12" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AP12" s="3">
         <v>-1</v>
       </c>
       <c r="AQ12" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AR12" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AS12" s="3">
         <v>1</v>
       </c>
       <c r="AT12" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU12" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AV12" s="3">
         <v>1</v>
       </c>
       <c r="AW12" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AX12" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AY12" s="3">
+        <v>1</v>
+      </c>
+      <c r="AZ12" s="3">
         <v>-1</v>
       </c>
     </row>
@@ -2425,48 +2464,51 @@
         <v>-1</v>
       </c>
       <c r="AK13" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AL13" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AM13" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AN13" s="3">
         <v>0</v>
       </c>
       <c r="AO13" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AP13" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AQ13" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AR13" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AS13" s="3">
         <v>-1</v>
       </c>
       <c r="AT13" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AU13" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AV13" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AW13" s="3">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="AX13" s="3">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="AY13" s="3">
+        <v>-1</v>
+      </c>
+      <c r="AZ13" s="3">
         <v>-1</v>
       </c>
     </row>
@@ -2580,25 +2622,25 @@
         <v>-1</v>
       </c>
       <c r="AK14" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AL14" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AM14" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AN14" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AO14" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AP14" s="3">
         <v>-1</v>
       </c>
       <c r="AQ14" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AR14" s="3">
         <v>0</v>
@@ -2610,18 +2652,21 @@
         <v>0</v>
       </c>
       <c r="AU14" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AV14" s="3">
         <v>1</v>
       </c>
       <c r="AW14" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AX14" s="3">
-        <v>-1</v>
+        <v>2</v>
       </c>
       <c r="AY14" s="3">
+        <v>-1</v>
+      </c>
+      <c r="AZ14" s="3">
         <v>1</v>
       </c>
     </row>
@@ -2738,45 +2783,48 @@
         <v>0</v>
       </c>
       <c r="AL15" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AM15" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AN15" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AO15" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AP15" s="3">
         <v>-1</v>
       </c>
       <c r="AQ15" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AR15" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AS15" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AT15" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU15" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AV15" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW15" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AX15" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AY15" s="3">
+        <v>1</v>
+      </c>
+      <c r="AZ15" s="3">
         <v>-2</v>
       </c>
     </row>
@@ -2890,19 +2938,19 @@
         <v>0</v>
       </c>
       <c r="AK16" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AL16" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AM16" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AN16" s="3">
         <v>-1</v>
       </c>
       <c r="AO16" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AP16" s="3">
         <v>0</v>
@@ -2911,27 +2959,30 @@
         <v>0</v>
       </c>
       <c r="AR16" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AS16" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AT16" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AU16" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AV16" s="3">
         <v>0</v>
       </c>
       <c r="AW16" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AX16" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AY16" s="3">
+        <v>0</v>
+      </c>
+      <c r="AZ16" s="3">
         <v>1</v>
       </c>
     </row>
@@ -3045,19 +3096,19 @@
         <v>-1</v>
       </c>
       <c r="AK17" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AL17" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AM17" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AN17" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AO17" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AP17" s="3">
         <v>-1</v>
@@ -3066,27 +3117,30 @@
         <v>-1</v>
       </c>
       <c r="AR17" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AS17" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AT17" s="3">
         <v>0</v>
       </c>
       <c r="AU17" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AV17" s="3">
         <v>1</v>
       </c>
       <c r="AW17" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AX17" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AY17" s="3">
+        <v>1</v>
+      </c>
+      <c r="AZ17" s="3">
         <v>1</v>
       </c>
     </row>
@@ -3215,33 +3269,36 @@
         <v>0</v>
       </c>
       <c r="AP18" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AQ18" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AR18" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AS18" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AT18" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU18" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AV18" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AW18" s="3">
         <v>0</v>
       </c>
       <c r="AX18" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AY18" s="3">
+        <v>1</v>
+      </c>
+      <c r="AZ18" s="3">
         <v>1</v>
       </c>
     </row>
@@ -3355,7 +3412,7 @@
         <v>-2</v>
       </c>
       <c r="AK19" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AL19" s="3">
         <v>-1</v>
@@ -3364,31 +3421,31 @@
         <v>-1</v>
       </c>
       <c r="AN19" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AO19" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AP19" s="3">
         <v>-1</v>
       </c>
       <c r="AQ19" s="3">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="AR19" s="3">
-        <v>1</v>
+        <v>-2</v>
       </c>
       <c r="AS19" s="3">
         <v>1</v>
       </c>
       <c r="AT19" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU19" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AV19" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AW19" s="3">
         <v>0</v>
@@ -3397,6 +3454,9 @@
         <v>0</v>
       </c>
       <c r="AY19" s="3">
+        <v>0</v>
+      </c>
+      <c r="AZ19" s="3">
         <v>0</v>
       </c>
     </row>
@@ -3510,34 +3570,34 @@
         <v>-1</v>
       </c>
       <c r="AK20" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AL20" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AM20" s="3">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="AN20" s="3">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AO20" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AP20" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AQ20" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AR20" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS20" s="3">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="AT20" s="3">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AU20" s="3">
         <v>0</v>
@@ -3546,12 +3606,15 @@
         <v>0</v>
       </c>
       <c r="AW20" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AX20" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AY20" s="3">
+        <v>-1</v>
+      </c>
+      <c r="AZ20" s="3">
         <v>0</v>
       </c>
     </row>
@@ -3668,10 +3731,10 @@
         <v>0</v>
       </c>
       <c r="AL21" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AM21" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AN21" s="3">
         <v>0</v>
@@ -3680,33 +3743,36 @@
         <v>0</v>
       </c>
       <c r="AP21" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AQ21" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AR21" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AS21" s="3">
         <v>-1</v>
       </c>
       <c r="AT21" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AU21" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AV21" s="3">
         <v>-1</v>
       </c>
       <c r="AW21" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AX21" s="3">
         <v>0</v>
       </c>
       <c r="AY21" s="3">
+        <v>0</v>
+      </c>
+      <c r="AZ21" s="3">
         <v>1</v>
       </c>
     </row>
@@ -3823,13 +3889,13 @@
         <v>0</v>
       </c>
       <c r="AL22" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AM22" s="3">
-        <v>2</v>
+        <v>-1</v>
       </c>
       <c r="AN22" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AO22" s="3">
         <v>0</v>
@@ -3841,19 +3907,19 @@
         <v>0</v>
       </c>
       <c r="AR22" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AS22" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AT22" s="3">
         <v>0</v>
       </c>
       <c r="AU22" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AV22" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AW22" s="3">
         <v>0</v>
@@ -3862,6 +3928,9 @@
         <v>0</v>
       </c>
       <c r="AY22" s="3">
+        <v>0</v>
+      </c>
+      <c r="AZ22" s="3">
         <v>1</v>
       </c>
     </row>
@@ -3975,48 +4044,51 @@
         <v>1</v>
       </c>
       <c r="AK23" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AL23" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AM23" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AN23" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AO23" s="3">
         <v>1</v>
       </c>
       <c r="AP23" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AQ23" s="3">
-        <v>-1</v>
+        <v>2</v>
       </c>
       <c r="AR23" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AS23" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AT23" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AU23" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AV23" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AW23" s="3">
-        <v>2</v>
+        <v>-1</v>
       </c>
       <c r="AX23" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AY23" s="3">
+        <v>0</v>
+      </c>
+      <c r="AZ23" s="3">
         <v>1</v>
       </c>
     </row>
@@ -4130,31 +4202,31 @@
         <v>-1</v>
       </c>
       <c r="AK24" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AL24" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AM24" s="3">
         <v>0</v>
       </c>
       <c r="AN24" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AO24" s="3">
         <v>-1</v>
       </c>
       <c r="AP24" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AQ24" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AR24" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AS24" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AT24" s="3">
         <v>0</v>
@@ -4163,15 +4235,18 @@
         <v>0</v>
       </c>
       <c r="AV24" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AW24" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AX24" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AY24" s="3">
+        <v>-1</v>
+      </c>
+      <c r="AZ24" s="3">
         <v>-1</v>
       </c>
     </row>
@@ -4288,45 +4363,48 @@
         <v>0</v>
       </c>
       <c r="AL25" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AM25" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AN25" s="3">
         <v>0</v>
       </c>
       <c r="AO25" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AP25" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AQ25" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AR25" s="3">
         <v>0</v>
       </c>
       <c r="AS25" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AT25" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU25" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AV25" s="3">
         <v>1</v>
       </c>
       <c r="AW25" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AX25" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AY25" s="3">
+        <v>1</v>
+      </c>
+      <c r="AZ25" s="3">
         <v>0</v>
       </c>
     </row>
@@ -4440,22 +4518,22 @@
         <v>0</v>
       </c>
       <c r="AK26" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AL26" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AM26" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AN26" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AO26" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AP26" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AQ26" s="3">
         <v>1</v>
@@ -4464,13 +4542,13 @@
         <v>1</v>
       </c>
       <c r="AS26" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AT26" s="3">
         <v>0</v>
       </c>
       <c r="AU26" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AV26" s="3">
         <v>1</v>
@@ -4482,6 +4560,9 @@
         <v>1</v>
       </c>
       <c r="AY26" s="3">
+        <v>1</v>
+      </c>
+      <c r="AZ26" s="3">
         <v>1</v>
       </c>
     </row>
@@ -4595,10 +4676,10 @@
         <v>-1</v>
       </c>
       <c r="AK27" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AL27" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AM27" s="3">
         <v>0</v>
@@ -4622,7 +4703,7 @@
         <v>0</v>
       </c>
       <c r="AT27" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AU27" s="3">
         <v>-1</v>
@@ -4631,12 +4712,15 @@
         <v>-1</v>
       </c>
       <c r="AW27" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AX27" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AY27" s="3">
+        <v>1</v>
+      </c>
+      <c r="AZ27" s="3">
         <v>-1</v>
       </c>
     </row>
@@ -4753,31 +4837,31 @@
         <v>0</v>
       </c>
       <c r="AL28" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AM28" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AN28" s="3">
         <v>-1</v>
       </c>
       <c r="AO28" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AP28" s="3">
         <v>0</v>
       </c>
       <c r="AQ28" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AR28" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS28" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AT28" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AU28" s="3">
         <v>0</v>
@@ -4786,12 +4870,15 @@
         <v>0</v>
       </c>
       <c r="AW28" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AX28" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AY28" s="3">
+        <v>0</v>
+      </c>
+      <c r="AZ28" s="3">
         <v>0</v>
       </c>
     </row>
@@ -4911,42 +4998,45 @@
         <v>0</v>
       </c>
       <c r="AM29" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AN29" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AO29" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AP29" s="3">
         <v>1</v>
       </c>
       <c r="AQ29" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AR29" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AS29" s="3">
-        <v>-2</v>
+        <v>2</v>
       </c>
       <c r="AT29" s="3">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="AU29" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AV29" s="3">
         <v>1</v>
       </c>
       <c r="AW29" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AX29" s="3">
         <v>-1</v>
       </c>
       <c r="AY29" s="3">
+        <v>-1</v>
+      </c>
+      <c r="AZ29" s="3">
         <v>0</v>
       </c>
     </row>
@@ -5060,48 +5150,51 @@
         <v>0</v>
       </c>
       <c r="AK30" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AL30" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AM30" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AN30" s="3">
         <v>1</v>
       </c>
       <c r="AO30" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AP30" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AQ30" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AR30" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AS30" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AT30" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AU30" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AV30" s="3">
-        <v>-2</v>
+        <v>1</v>
       </c>
       <c r="AW30" s="3">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="AX30" s="3">
         <v>-1</v>
       </c>
       <c r="AY30" s="3">
+        <v>-1</v>
+      </c>
+      <c r="AZ30" s="3">
         <v>-1</v>
       </c>
     </row>
@@ -5215,31 +5308,31 @@
         <v>1</v>
       </c>
       <c r="AK31" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AL31" s="3">
-        <v>-2</v>
+        <v>2</v>
       </c>
       <c r="AM31" s="3">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AN31" s="3">
         <v>0</v>
       </c>
       <c r="AO31" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AP31" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AQ31" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AR31" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AS31" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AT31" s="3">
         <v>0</v>
@@ -5254,9 +5347,12 @@
         <v>0</v>
       </c>
       <c r="AX31" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AY31" s="3">
+        <v>-1</v>
+      </c>
+      <c r="AZ31" s="3">
         <v>-1</v>
       </c>
     </row>
@@ -5373,7 +5469,7 @@
         <v>0</v>
       </c>
       <c r="AL32" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AM32" s="3">
         <v>1</v>
@@ -5382,36 +5478,39 @@
         <v>1</v>
       </c>
       <c r="AO32" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AP32" s="3">
         <v>-1</v>
       </c>
       <c r="AQ32" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AR32" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AS32" s="3">
         <v>1</v>
       </c>
       <c r="AT32" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU32" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AV32" s="3">
-        <v>-2</v>
+        <v>1</v>
       </c>
       <c r="AW32" s="3">
-        <v>2</v>
+        <v>-2</v>
       </c>
       <c r="AX32" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AY32" s="3">
+        <v>0</v>
+      </c>
+      <c r="AZ32" s="3">
         <v>1</v>
       </c>
     </row>
@@ -5525,10 +5624,10 @@
         <v>0</v>
       </c>
       <c r="AK33" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AL33" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AM33" s="3">
         <v>0</v>
@@ -5537,19 +5636,19 @@
         <v>0</v>
       </c>
       <c r="AO33" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AP33" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AQ33" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AR33" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AS33" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AT33" s="3">
         <v>0</v>
@@ -5567,6 +5666,9 @@
         <v>0</v>
       </c>
       <c r="AY33" s="3">
+        <v>0</v>
+      </c>
+      <c r="AZ33" s="3">
         <v>-1</v>
       </c>
     </row>
@@ -5680,25 +5782,25 @@
         <v>-2</v>
       </c>
       <c r="AK34" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AL34" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AM34" s="3">
-        <v>-2</v>
+        <v>1</v>
       </c>
       <c r="AN34" s="3">
-        <v>1</v>
+        <v>-2</v>
       </c>
       <c r="AO34" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AP34" s="3">
         <v>-1</v>
       </c>
       <c r="AQ34" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AR34" s="3">
         <v>1</v>
@@ -5707,7 +5809,7 @@
         <v>1</v>
       </c>
       <c r="AT34" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU34" s="3">
         <v>0</v>
@@ -5719,9 +5821,12 @@
         <v>0</v>
       </c>
       <c r="AX34" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AY34" s="3">
+        <v>-1</v>
+      </c>
+      <c r="AZ34" s="3">
         <v>0</v>
       </c>
     </row>
@@ -5835,48 +5940,51 @@
         <v>0</v>
       </c>
       <c r="AK35" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AL35" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AM35" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AN35" s="3">
         <v>0</v>
       </c>
       <c r="AO35" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AP35" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AQ35" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AR35" s="3">
         <v>-1</v>
       </c>
       <c r="AS35" s="3">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="AT35" s="3">
-        <v>1</v>
+        <v>-2</v>
       </c>
       <c r="AU35" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AV35" s="3">
         <v>-1</v>
       </c>
       <c r="AW35" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AX35" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AY35" s="3">
+        <v>0</v>
+      </c>
+      <c r="AZ35" s="3">
         <v>0</v>
       </c>
     </row>
@@ -5990,40 +6098,40 @@
         <v>-11</v>
       </c>
       <c r="AK36" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AL36" s="3">
         <v>1</v>
       </c>
       <c r="AM36" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AN36" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AO36" s="3">
         <v>0</v>
       </c>
       <c r="AP36" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AQ36" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AR36" s="3">
         <v>0</v>
       </c>
       <c r="AS36" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AT36" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AU36" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AV36" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AW36" s="3">
         <v>0</v>
@@ -6032,6 +6140,9 @@
         <v>0</v>
       </c>
       <c r="AY36" s="3">
+        <v>0</v>
+      </c>
+      <c r="AZ36" s="3">
         <v>-1</v>
       </c>
     </row>
@@ -6040,31 +6151,31 @@
         <v>36</v>
       </c>
       <c r="B37" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C37" s="3">
         <v>0</v>
       </c>
       <c r="D37" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E37" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F37" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="G37" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="H37" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I37" s="3">
         <v>0</v>
       </c>
       <c r="J37" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="K37" s="3">
         <v>0</v>
@@ -6073,52 +6184,52 @@
         <v>0</v>
       </c>
       <c r="M37" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N37" s="3">
         <v>0</v>
       </c>
       <c r="O37" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="P37" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q37" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="R37" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="S37" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T37" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U37" s="3">
         <v>0</v>
       </c>
       <c r="V37" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="W37" s="3">
         <v>0</v>
       </c>
       <c r="X37" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y37" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z37" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA37" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB37" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AC37" s="3">
         <v>0</v>
@@ -6130,66 +6241,66 @@
         <v>0</v>
       </c>
       <c r="AF37" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AG37" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AH37" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AI37" s="3">
         <v>0</v>
       </c>
       <c r="AJ37" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AK37" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AL37" s="3">
-        <v>-11</v>
+        <v>0</v>
       </c>
       <c r="AM37" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AN37" s="3">
         <v>0</v>
       </c>
       <c r="AO37" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AP37" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AQ37" s="3">
         <v>0</v>
       </c>
       <c r="AR37" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AS37" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AT37" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AU37" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AV37" s="3">
         <v>0</v>
       </c>
       <c r="AW37" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AX37" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AY37" s="3">
-        <v>1</v>
-      </c>
-      <c r="AZ37">
+        <v>0</v>
+      </c>
+      <c r="AZ37" s="3">
         <v>0</v>
       </c>
     </row>
@@ -6201,19 +6312,19 @@
         <v>1</v>
       </c>
       <c r="C38" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D38" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E38" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F38" s="3">
         <v>-1</v>
       </c>
       <c r="G38" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H38" s="3">
         <v>1</v>
@@ -6222,112 +6333,112 @@
         <v>0</v>
       </c>
       <c r="J38" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="K38" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L38" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M38" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="N38" s="3">
         <v>0</v>
       </c>
       <c r="O38" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="P38" s="3">
         <v>1</v>
       </c>
       <c r="Q38" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="R38" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="S38" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T38" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U38" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V38" s="3">
-        <v>-1</v>
+        <v>2</v>
       </c>
       <c r="W38" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="X38" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y38" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z38" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA38" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AB38" s="3">
         <v>1</v>
       </c>
       <c r="AC38" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AD38" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AE38" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AF38" s="3">
         <v>1</v>
       </c>
       <c r="AG38" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AH38" s="3">
         <v>1</v>
       </c>
       <c r="AI38" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AJ38" s="3">
         <v>1</v>
       </c>
       <c r="AK38" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AL38" s="3">
         <v>-11</v>
       </c>
       <c r="AM38" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AN38" s="3">
         <v>1</v>
       </c>
       <c r="AO38" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AP38" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AQ38" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AR38" s="3">
         <v>0</v>
       </c>
       <c r="AS38" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AT38" s="3">
         <v>-1</v>
@@ -6336,16 +6447,19 @@
         <v>-1</v>
       </c>
       <c r="AV38" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AW38" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AX38" s="3">
         <v>1</v>
       </c>
       <c r="AY38" s="3">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="AZ38" s="3">
+        <v>1</v>
       </c>
     </row>
     <row r="39" ht="15.75" customHeight="1">
@@ -6359,28 +6473,28 @@
         <v>1</v>
       </c>
       <c r="D39" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="E39" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="F39" s="3">
-        <v>2</v>
+        <v>-1</v>
       </c>
       <c r="G39" s="3">
         <v>0</v>
       </c>
       <c r="H39" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I39" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="J39" s="3">
         <v>0</v>
       </c>
       <c r="K39" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L39" s="3">
         <v>1</v>
@@ -6392,16 +6506,16 @@
         <v>0</v>
       </c>
       <c r="O39" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P39" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="Q39" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R39" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S39" s="3">
         <v>0</v>
@@ -6410,7 +6524,7 @@
         <v>0</v>
       </c>
       <c r="U39" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V39" s="3">
         <v>-1</v>
@@ -6419,7 +6533,7 @@
         <v>-1</v>
       </c>
       <c r="X39" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y39" s="3">
         <v>0</v>
@@ -6431,7 +6545,7 @@
         <v>-1</v>
       </c>
       <c r="AB39" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AC39" s="3">
         <v>-1</v>
@@ -6440,7 +6554,7 @@
         <v>1</v>
       </c>
       <c r="AE39" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AF39" s="3">
         <v>1</v>
@@ -6452,25 +6566,25 @@
         <v>1</v>
       </c>
       <c r="AI39" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AJ39" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AK39" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AL39" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AM39" s="3">
         <v>-11</v>
       </c>
       <c r="AN39" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AO39" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AP39" s="3">
         <v>-1</v>
@@ -6479,28 +6593,31 @@
         <v>-1</v>
       </c>
       <c r="AR39" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS39" s="3">
         <v>0</v>
       </c>
       <c r="AT39" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU39" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AV39" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AW39" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AX39" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AY39" s="3">
-        <v>-1</v>
+        <v>1</v>
+      </c>
+      <c r="AZ39" s="3">
+        <v>0</v>
       </c>
     </row>
     <row r="40" ht="15.75" customHeight="1">
@@ -6508,31 +6625,31 @@
         <v>39</v>
       </c>
       <c r="B40" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="C40" s="3">
         <v>1</v>
       </c>
       <c r="D40" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="E40" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="F40" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G40" s="3">
         <v>0</v>
       </c>
       <c r="H40" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I40" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="J40" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K40" s="3">
         <v>1</v>
@@ -6541,19 +6658,19 @@
         <v>1</v>
       </c>
       <c r="M40" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="N40" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O40" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P40" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="Q40" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R40" s="3">
         <v>1</v>
@@ -6568,94 +6685,97 @@
         <v>0</v>
       </c>
       <c r="V40" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="W40" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="X40" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="Y40" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="Z40" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AA40" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AB40" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AC40" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AD40" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AE40" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AF40" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG40" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AH40" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI40" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AJ40" s="3">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="AK40" s="3">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="AL40" s="3">
         <v>1</v>
       </c>
       <c r="AM40" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AN40" s="3">
         <v>-11</v>
       </c>
       <c r="AO40" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AP40" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AQ40" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AR40" s="3">
-        <v>2</v>
+        <v>-1</v>
       </c>
       <c r="AS40" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AT40" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AU40" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AV40" s="3">
         <v>1</v>
       </c>
       <c r="AW40" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AX40" s="3">
         <v>1</v>
       </c>
       <c r="AY40" s="3">
-        <v>1</v>
+        <v>-1</v>
+      </c>
+      <c r="AZ40" s="3">
+        <v>-1</v>
       </c>
     </row>
     <row r="41" ht="15.75" customHeight="1">
@@ -6663,10 +6783,10 @@
         <v>40</v>
       </c>
       <c r="B41" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="C41" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D41" s="3">
         <v>0</v>
@@ -6678,43 +6798,43 @@
         <v>0</v>
       </c>
       <c r="G41" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H41" s="3">
         <v>1</v>
       </c>
       <c r="I41" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="J41" s="3">
         <v>1</v>
       </c>
       <c r="K41" s="3">
-        <v>-2</v>
+        <v>1</v>
       </c>
       <c r="L41" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="M41" s="3">
         <v>0</v>
       </c>
       <c r="N41" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O41" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="P41" s="3">
         <v>0</v>
       </c>
       <c r="Q41" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="R41" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S41" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T41" s="3">
         <v>0</v>
@@ -6723,94 +6843,97 @@
         <v>0</v>
       </c>
       <c r="V41" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="W41" s="3">
         <v>1</v>
       </c>
       <c r="X41" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="Y41" s="3">
-        <v>2</v>
+        <v>-1</v>
       </c>
       <c r="Z41" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AA41" s="3">
         <v>0</v>
       </c>
       <c r="AB41" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AC41" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AD41" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AE41" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AF41" s="3">
         <v>0</v>
       </c>
       <c r="AG41" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AH41" s="3">
         <v>0</v>
       </c>
       <c r="AI41" s="3">
-        <v>2</v>
+        <v>-1</v>
       </c>
       <c r="AJ41" s="3">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AK41" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AL41" s="3">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AM41" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AN41" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AO41" s="3">
         <v>-11</v>
       </c>
       <c r="AP41" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AQ41" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AR41" s="3">
         <v>0</v>
       </c>
       <c r="AS41" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AT41" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU41" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AV41" s="3">
-        <v>-2</v>
+        <v>1</v>
       </c>
       <c r="AW41" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AX41" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AY41" s="3">
-        <v>-1</v>
+        <v>1</v>
+      </c>
+      <c r="AZ41" s="3">
+        <v>1</v>
       </c>
     </row>
     <row r="42" ht="15.75" customHeight="1">
@@ -6818,34 +6941,34 @@
         <v>41</v>
       </c>
       <c r="B42" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C42" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="D42" s="3">
         <v>0</v>
       </c>
       <c r="E42" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="F42" s="3">
         <v>0</v>
       </c>
       <c r="G42" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H42" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I42" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="J42" s="3">
         <v>1</v>
       </c>
       <c r="K42" s="3">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="L42" s="3">
         <v>-1</v>
@@ -6854,31 +6977,31 @@
         <v>0</v>
       </c>
       <c r="N42" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="O42" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="P42" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q42" s="3">
         <v>-1</v>
       </c>
       <c r="R42" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="S42" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="T42" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U42" s="3">
         <v>0</v>
       </c>
       <c r="V42" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W42" s="3">
         <v>1</v>
@@ -6887,34 +7010,34 @@
         <v>0</v>
       </c>
       <c r="Y42" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Z42" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA42" s="3">
         <v>0</v>
       </c>
       <c r="AB42" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AC42" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AD42" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AE42" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AF42" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AG42" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH42" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AI42" s="3">
         <v>2</v>
@@ -6926,16 +7049,16 @@
         <v>0</v>
       </c>
       <c r="AL42" s="3">
-        <v>-1</v>
+        <v>2</v>
       </c>
       <c r="AM42" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AN42" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AO42" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AP42" s="3">
         <v>-11</v>
@@ -6944,28 +7067,31 @@
         <v>0</v>
       </c>
       <c r="AR42" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AS42" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AT42" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AU42" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AV42" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AW42" s="3">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AX42" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AY42" s="3">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="AZ42" s="3">
+        <v>-1</v>
       </c>
     </row>
     <row r="43" ht="15.75" customHeight="1">
@@ -6973,13 +7099,13 @@
         <v>42</v>
       </c>
       <c r="B43" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C43" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="D43" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E43" s="3">
         <v>-1</v>
@@ -6988,61 +7114,61 @@
         <v>0</v>
       </c>
       <c r="G43" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H43" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I43" s="3">
         <v>1</v>
       </c>
       <c r="J43" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="K43" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="L43" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="M43" s="3">
         <v>0</v>
       </c>
       <c r="N43" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="O43" s="3">
-        <v>2</v>
+        <v>-1</v>
       </c>
       <c r="P43" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q43" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="R43" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="S43" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="T43" s="3">
         <v>1</v>
       </c>
       <c r="U43" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V43" s="3">
         <v>1</v>
       </c>
       <c r="W43" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X43" s="3">
         <v>0</v>
       </c>
       <c r="Y43" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z43" s="3">
         <v>1</v>
@@ -7051,31 +7177,31 @@
         <v>0</v>
       </c>
       <c r="AB43" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AC43" s="3">
         <v>0</v>
       </c>
       <c r="AD43" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AE43" s="3">
-        <v>-1</v>
+        <v>2</v>
       </c>
       <c r="AF43" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AG43" s="3">
         <v>0</v>
       </c>
       <c r="AH43" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AI43" s="3">
-        <v>-2</v>
+        <v>2</v>
       </c>
       <c r="AJ43" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AK43" s="3">
         <v>0</v>
@@ -7084,43 +7210,46 @@
         <v>0</v>
       </c>
       <c r="AM43" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AN43" s="3">
         <v>1</v>
       </c>
       <c r="AO43" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AP43" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AQ43" s="3">
         <v>-11</v>
       </c>
       <c r="AR43" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AS43" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AT43" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AU43" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AV43" s="3">
-        <v>2</v>
+        <v>-1</v>
       </c>
       <c r="AW43" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AX43" s="3">
         <v>0</v>
       </c>
       <c r="AY43" s="3">
-        <v>1</v>
+        <v>-1</v>
+      </c>
+      <c r="AZ43" s="3">
+        <v>0</v>
       </c>
     </row>
     <row r="44" ht="15.75" customHeight="1">
@@ -7128,16 +7257,16 @@
         <v>43</v>
       </c>
       <c r="B44" s="3">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="C44" s="3">
         <v>1</v>
       </c>
       <c r="D44" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="E44" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="F44" s="3">
         <v>0</v>
@@ -7146,13 +7275,13 @@
         <v>1</v>
       </c>
       <c r="H44" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="I44" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J44" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="K44" s="3">
         <v>1</v>
@@ -7161,16 +7290,16 @@
         <v>1</v>
       </c>
       <c r="M44" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="N44" s="3">
         <v>0</v>
       </c>
       <c r="O44" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P44" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q44" s="3">
         <v>1</v>
@@ -7182,10 +7311,10 @@
         <v>1</v>
       </c>
       <c r="T44" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U44" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V44" s="3">
         <v>1</v>
@@ -7197,61 +7326,61 @@
         <v>0</v>
       </c>
       <c r="Y44" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z44" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA44" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AB44" s="3">
         <v>0</v>
       </c>
       <c r="AC44" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AD44" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AE44" s="3">
         <v>-1</v>
       </c>
       <c r="AF44" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AG44" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AH44" s="3">
         <v>1</v>
       </c>
       <c r="AI44" s="3">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AJ44" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AK44" s="3">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="AL44" s="3">
         <v>0</v>
       </c>
       <c r="AM44" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AN44" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AO44" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AP44" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AQ44" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AR44" s="3">
         <v>-11</v>
@@ -7260,21 +7389,24 @@
         <v>1</v>
       </c>
       <c r="AT44" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU44" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AV44" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW44" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AX44" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AY44" s="3">
+        <v>0</v>
+      </c>
+      <c r="AZ44" s="3">
         <v>1</v>
       </c>
     </row>
@@ -7283,31 +7415,31 @@
         <v>44</v>
       </c>
       <c r="B45" s="3">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="C45" s="3">
         <v>1</v>
       </c>
       <c r="D45" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="E45" s="3">
         <v>0</v>
       </c>
       <c r="F45" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="G45" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H45" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="I45" s="3">
         <v>0</v>
       </c>
       <c r="J45" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K45" s="3">
         <v>1</v>
@@ -7325,34 +7457,34 @@
         <v>1</v>
       </c>
       <c r="P45" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q45" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R45" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S45" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T45" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U45" s="3">
         <v>0</v>
       </c>
       <c r="V45" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W45" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X45" s="3">
         <v>0</v>
       </c>
       <c r="Y45" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z45" s="3">
         <v>0</v>
@@ -7361,28 +7493,28 @@
         <v>-1</v>
       </c>
       <c r="AB45" s="3">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="AC45" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AD45" s="3">
         <v>1</v>
       </c>
       <c r="AE45" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AF45" s="3">
         <v>1</v>
       </c>
       <c r="AG45" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AH45" s="3">
         <v>1</v>
       </c>
       <c r="AI45" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AJ45" s="3">
         <v>1</v>
@@ -7391,46 +7523,49 @@
         <v>0</v>
       </c>
       <c r="AL45" s="3">
-        <v>1</v>
+        <v>-2</v>
       </c>
       <c r="AM45" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AN45" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AO45" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AP45" s="3">
         <v>-1</v>
       </c>
       <c r="AQ45" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AR45" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AS45" s="3">
         <v>-11</v>
       </c>
       <c r="AT45" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AU45" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AV45" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AW45" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AX45" s="3">
         <v>0</v>
       </c>
       <c r="AY45" s="3">
         <v>0</v>
+      </c>
+      <c r="AZ45" s="3">
+        <v>1</v>
       </c>
     </row>
     <row r="46" ht="15.75" customHeight="1">
@@ -7438,153 +7573,156 @@
         <v>45</v>
       </c>
       <c r="B46" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C46" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D46" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E46" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F46" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="G46" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H46" s="3">
         <v>0</v>
       </c>
       <c r="I46" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="J46" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K46" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L46" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M46" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="N46" s="3">
         <v>0</v>
       </c>
       <c r="O46" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P46" s="3">
         <v>0</v>
       </c>
       <c r="Q46" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="R46" s="3">
         <v>1</v>
       </c>
       <c r="S46" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="T46" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U46" s="3">
         <v>0</v>
       </c>
       <c r="V46" s="3">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="W46" s="3">
-        <v>-2</v>
+        <v>1</v>
       </c>
       <c r="X46" s="3">
         <v>0</v>
       </c>
       <c r="Y46" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="Z46" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AA46" s="3">
         <v>-1</v>
       </c>
       <c r="AB46" s="3">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AC46" s="3">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="AD46" s="3">
-        <v>-2</v>
+        <v>1</v>
       </c>
       <c r="AE46" s="3">
         <v>0</v>
       </c>
       <c r="AF46" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG46" s="3">
         <v>0</v>
       </c>
       <c r="AH46" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI46" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AJ46" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AK46" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AL46" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AM46" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AN46" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AO46" s="3">
         <v>1</v>
       </c>
       <c r="AP46" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AQ46" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AR46" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS46" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AT46" s="3">
         <v>-11</v>
       </c>
       <c r="AU46" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AV46" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AW46" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AX46" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AY46" s="3">
+        <v>0</v>
+      </c>
+      <c r="AZ46" s="3">
         <v>0</v>
       </c>
     </row>
@@ -7593,34 +7731,34 @@
         <v>46</v>
       </c>
       <c r="B47" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="C47" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D47" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="E47" s="3">
         <v>1</v>
       </c>
       <c r="F47" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="G47" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="H47" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="I47" s="3">
-        <v>2</v>
+        <v>-1</v>
       </c>
       <c r="J47" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K47" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L47" s="3">
         <v>0</v>
@@ -7632,16 +7770,16 @@
         <v>0</v>
       </c>
       <c r="O47" s="3">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="P47" s="3">
         <v>0</v>
       </c>
       <c r="Q47" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="R47" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="S47" s="3">
         <v>-1</v>
@@ -7653,94 +7791,97 @@
         <v>0</v>
       </c>
       <c r="V47" s="3">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="W47" s="3">
         <v>-2</v>
       </c>
       <c r="X47" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="Y47" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="Z47" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AA47" s="3">
         <v>-1</v>
       </c>
       <c r="AB47" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AC47" s="3">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AD47" s="3">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AE47" s="3">
         <v>0</v>
       </c>
       <c r="AF47" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AG47" s="3">
         <v>0</v>
       </c>
       <c r="AH47" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AI47" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AJ47" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AK47" s="3">
         <v>0</v>
       </c>
       <c r="AL47" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AM47" s="3">
         <v>-1</v>
       </c>
       <c r="AN47" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AO47" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AP47" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AQ47" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AR47" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AS47" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AT47" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AU47" s="3">
         <v>-11</v>
       </c>
       <c r="AV47" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AW47" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AX47" s="3">
         <v>1</v>
       </c>
       <c r="AY47" s="3">
-        <v>-1</v>
+        <v>0</v>
+      </c>
+      <c r="AZ47" s="3">
+        <v>0</v>
       </c>
     </row>
     <row r="48" ht="15.75" customHeight="1">
@@ -7748,28 +7889,28 @@
         <v>47</v>
       </c>
       <c r="B48" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C48" s="3">
         <v>1</v>
       </c>
       <c r="D48" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E48" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="F48" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G48" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H48" s="3">
         <v>0</v>
       </c>
       <c r="I48" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J48" s="3">
         <v>0</v>
@@ -7778,16 +7919,16 @@
         <v>1</v>
       </c>
       <c r="L48" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M48" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="N48" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O48" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="P48" s="3">
         <v>1</v>
@@ -7796,70 +7937,70 @@
         <v>1</v>
       </c>
       <c r="R48" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S48" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="T48" s="3">
         <v>0</v>
       </c>
       <c r="U48" s="3">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="V48" s="3">
         <v>1</v>
       </c>
       <c r="W48" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X48" s="3">
         <v>0</v>
       </c>
       <c r="Y48" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Z48" s="3">
         <v>1</v>
       </c>
       <c r="AA48" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AB48" s="3">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="AC48" s="3">
         <v>0</v>
       </c>
       <c r="AD48" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE48" s="3">
         <v>0</v>
       </c>
       <c r="AF48" s="3">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="AG48" s="3">
         <v>0</v>
       </c>
       <c r="AH48" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AI48" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AJ48" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AK48" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AL48" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AM48" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AN48" s="3">
         <v>1</v>
@@ -7868,34 +8009,37 @@
         <v>1</v>
       </c>
       <c r="AP48" s="3">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="AQ48" s="3">
-        <v>1</v>
+        <v>-2</v>
       </c>
       <c r="AR48" s="3">
         <v>2</v>
       </c>
       <c r="AS48" s="3">
-        <v>-1</v>
+        <v>2</v>
       </c>
       <c r="AT48" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU48" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AV48" s="3">
         <v>-11</v>
       </c>
       <c r="AW48" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AX48" s="3">
         <v>0</v>
       </c>
       <c r="AY48" s="3">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="AZ48" s="3">
+        <v>1</v>
       </c>
     </row>
     <row r="49" ht="15.75" customHeight="1">
@@ -7903,13 +8047,13 @@
         <v>48</v>
       </c>
       <c r="B49" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="C49" s="3">
-        <v>-2</v>
+        <v>1</v>
       </c>
       <c r="D49" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="E49" s="3">
         <v>-1</v>
@@ -7918,10 +8062,10 @@
         <v>0</v>
       </c>
       <c r="G49" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H49" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="I49" s="3">
         <v>1</v>
@@ -7930,82 +8074,82 @@
         <v>0</v>
       </c>
       <c r="K49" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L49" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="M49" s="3">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="N49" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O49" s="3">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="P49" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q49" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R49" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="S49" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="T49" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U49" s="3">
         <v>0</v>
       </c>
       <c r="V49" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W49" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="X49" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y49" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z49" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AA49" s="3">
         <v>-1</v>
       </c>
       <c r="AB49" s="3">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AC49" s="3">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="AD49" s="3">
         <v>0</v>
       </c>
       <c r="AE49" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AF49" s="3">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AG49" s="3">
         <v>0</v>
       </c>
       <c r="AH49" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AI49" s="3">
         <v>0</v>
       </c>
       <c r="AJ49" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AK49" s="3">
         <v>0</v>
@@ -8014,42 +8158,45 @@
         <v>1</v>
       </c>
       <c r="AM49" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AN49" s="3">
-        <v>2</v>
+        <v>-1</v>
       </c>
       <c r="AO49" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AP49" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AQ49" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AR49" s="3">
         <v>1</v>
       </c>
       <c r="AS49" s="3">
-        <v>-1</v>
+        <v>2</v>
       </c>
       <c r="AT49" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AU49" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AV49" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AW49" s="3">
         <v>-11</v>
       </c>
       <c r="AX49" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AY49" s="3">
+        <v>0</v>
+      </c>
+      <c r="AZ49" s="3">
         <v>0</v>
       </c>
     </row>
@@ -8058,46 +8205,46 @@
         <v>49</v>
       </c>
       <c r="B50" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="C50" s="3">
-        <v>1</v>
+        <v>-2</v>
       </c>
       <c r="D50" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="E50" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="F50" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G50" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="H50" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="I50" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J50" s="3">
         <v>0</v>
       </c>
       <c r="K50" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L50" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="M50" s="3">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="N50" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O50" s="3">
-        <v>1</v>
+        <v>-2</v>
       </c>
       <c r="P50" s="3">
         <v>0</v>
@@ -8106,79 +8253,79 @@
         <v>2</v>
       </c>
       <c r="R50" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="S50" s="3">
         <v>0</v>
       </c>
       <c r="T50" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U50" s="3">
         <v>0</v>
       </c>
       <c r="V50" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W50" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="X50" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y50" s="3">
         <v>1</v>
       </c>
       <c r="Z50" s="3">
-        <v>2</v>
+        <v>-1</v>
       </c>
       <c r="AA50" s="3">
-        <v>2</v>
+        <v>-1</v>
       </c>
       <c r="AB50" s="3">
         <v>0</v>
       </c>
       <c r="AC50" s="3">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AD50" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AE50" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AF50" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AG50" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AH50" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AI50" s="3">
         <v>0</v>
       </c>
       <c r="AJ50" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AK50" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AL50" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AM50" s="3">
         <v>1</v>
       </c>
       <c r="AN50" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AO50" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AP50" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AQ50" s="3">
         <v>0</v>
@@ -8187,25 +8334,28 @@
         <v>0</v>
       </c>
       <c r="AS50" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AT50" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AU50" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AV50" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AW50" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AX50" s="3">
         <v>-11</v>
       </c>
       <c r="AY50" s="3">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="AZ50" s="3">
+        <v>0</v>
       </c>
     </row>
     <row r="51" ht="15.75" customHeight="1">
@@ -8219,10 +8369,10 @@
         <v>1</v>
       </c>
       <c r="D51" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E51" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F51" s="3">
         <v>1</v>
@@ -8243,22 +8393,22 @@
         <v>1</v>
       </c>
       <c r="L51" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M51" s="3">
-        <v>2</v>
+        <v>-1</v>
       </c>
       <c r="N51" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O51" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P51" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q51" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="R51" s="3">
         <v>1</v>
@@ -8267,58 +8417,58 @@
         <v>0</v>
       </c>
       <c r="T51" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="U51" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="V51" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W51" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="X51" s="3">
         <v>0</v>
       </c>
       <c r="Y51" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z51" s="3">
         <v>2</v>
       </c>
       <c r="AA51" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AB51" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AC51" s="3">
         <v>0</v>
       </c>
       <c r="AD51" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE51" s="3">
         <v>1</v>
       </c>
       <c r="AF51" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AG51" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH51" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AI51" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AJ51" s="3">
         <v>1</v>
       </c>
       <c r="AK51" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AL51" s="3">
         <v>1</v>
@@ -8327,10 +8477,10 @@
         <v>2</v>
       </c>
       <c r="AN51" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AO51" s="3">
-        <v>-2</v>
+        <v>1</v>
       </c>
       <c r="AP51" s="3">
         <v>0</v>
@@ -8339,7 +8489,7 @@
         <v>1</v>
       </c>
       <c r="AR51" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AS51" s="3">
         <v>0</v>
@@ -8348,13 +8498,13 @@
         <v>0</v>
       </c>
       <c r="AU51" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AV51" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW51" s="3">
-        <v>-2</v>
+        <v>1</v>
       </c>
       <c r="AX51" s="3">
         <v>1</v>
@@ -8362,11 +8512,171 @@
       <c r="AY51" s="3">
         <v>-11</v>
       </c>
+      <c r="AZ51" s="3">
+        <v>2</v>
+      </c>
     </row>
     <row r="52" ht="15.75" customHeight="1">
-      <c r="J52" s="3"/>
+      <c r="A52" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B52" s="3">
+        <v>1</v>
+      </c>
+      <c r="C52" s="3">
+        <v>1</v>
+      </c>
+      <c r="D52" s="3">
+        <v>2</v>
+      </c>
+      <c r="E52" s="3">
+        <v>2</v>
+      </c>
+      <c r="F52" s="3">
+        <v>1</v>
+      </c>
+      <c r="G52" s="3">
+        <v>-1</v>
+      </c>
+      <c r="H52" s="3">
+        <v>1</v>
+      </c>
+      <c r="I52" s="3">
+        <v>0</v>
+      </c>
+      <c r="J52" s="3">
+        <v>0</v>
+      </c>
+      <c r="K52" s="3">
+        <v>1</v>
+      </c>
+      <c r="L52" s="3">
+        <v>0</v>
+      </c>
+      <c r="M52" s="3">
+        <v>2</v>
+      </c>
+      <c r="N52" s="3">
+        <v>1</v>
+      </c>
+      <c r="O52" s="3">
+        <v>0</v>
+      </c>
+      <c r="P52" s="3">
+        <v>1</v>
+      </c>
+      <c r="Q52" s="3">
+        <v>0</v>
+      </c>
+      <c r="R52" s="3">
+        <v>1</v>
+      </c>
+      <c r="S52" s="3">
+        <v>0</v>
+      </c>
+      <c r="T52" s="3">
+        <v>0</v>
+      </c>
+      <c r="U52" s="3">
+        <v>2</v>
+      </c>
+      <c r="V52" s="3">
+        <v>2</v>
+      </c>
+      <c r="W52" s="3">
+        <v>2</v>
+      </c>
+      <c r="X52" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y52" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z52" s="3">
+        <v>2</v>
+      </c>
+      <c r="AA52" s="3">
+        <v>0</v>
+      </c>
+      <c r="AB52" s="3">
+        <v>1</v>
+      </c>
+      <c r="AC52" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD52" s="3">
+        <v>0</v>
+      </c>
+      <c r="AE52" s="3">
+        <v>1</v>
+      </c>
+      <c r="AF52" s="3">
+        <v>1</v>
+      </c>
+      <c r="AG52" s="3">
+        <v>0</v>
+      </c>
+      <c r="AH52" s="3">
+        <v>2</v>
+      </c>
+      <c r="AI52" s="3">
+        <v>2</v>
+      </c>
+      <c r="AJ52" s="3">
+        <v>1</v>
+      </c>
+      <c r="AK52" s="3">
+        <v>0</v>
+      </c>
+      <c r="AL52" s="3">
+        <v>2</v>
+      </c>
+      <c r="AM52" s="3">
+        <v>1</v>
+      </c>
+      <c r="AN52" s="3">
+        <v>2</v>
+      </c>
+      <c r="AO52" s="3">
+        <v>-1</v>
+      </c>
+      <c r="AP52" s="3">
+        <v>-2</v>
+      </c>
+      <c r="AQ52" s="3">
+        <v>0</v>
+      </c>
+      <c r="AR52" s="3">
+        <v>1</v>
+      </c>
+      <c r="AS52" s="3">
+        <v>2</v>
+      </c>
+      <c r="AT52" s="3">
+        <v>0</v>
+      </c>
+      <c r="AU52" s="3">
+        <v>0</v>
+      </c>
+      <c r="AV52" s="3">
+        <v>1</v>
+      </c>
+      <c r="AW52" s="3">
+        <v>1</v>
+      </c>
+      <c r="AX52" s="3">
+        <v>-2</v>
+      </c>
+      <c r="AY52" s="3">
+        <v>1</v>
+      </c>
+      <c r="AZ52" s="3">
+        <v>-11</v>
+      </c>
     </row>
-    <row r="53" ht="15.75" customHeight="1"/>
+    <row r="53" ht="15.75" customHeight="1">
+      <c r="J53" s="3"/>
+    </row>
     <row r="54" ht="15.75" customHeight="1"/>
     <row r="55" ht="15.75" customHeight="1"/>
     <row r="56" ht="15.75" customHeight="1"/>
@@ -9314,6 +9624,7 @@
     <row r="998" ht="15.75" customHeight="1"/>
     <row r="999" ht="15.75" customHeight="1"/>
     <row r="1000" ht="15.75" customHeight="1"/>
+    <row r="1001" ht="15.75" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.5118055" right="0.5118055" top="0.7875" bottom="0.7875" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>

<commit_message>
Mudanças na planilha parra Tracer, Soldier e Genji
</commit_message>
<xml_diff>
--- a/dist/OWPick/_internal/heroes ally.xlsx
+++ b/dist/OWPick/_internal/heroes ally.xlsx
@@ -2675,28 +2675,28 @@
         <v>14</v>
       </c>
       <c r="B15" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C15" s="3">
         <v>1</v>
       </c>
       <c r="D15" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E15" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="F15" s="3">
         <v>0</v>
       </c>
       <c r="G15" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H15" s="3">
         <v>0</v>
       </c>
       <c r="I15" s="3">
-        <v>-2</v>
+        <v>1</v>
       </c>
       <c r="J15" s="3">
         <v>-1</v>
@@ -2705,46 +2705,46 @@
         <v>2</v>
       </c>
       <c r="L15" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M15" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="N15" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O15" s="3">
         <v>-11</v>
       </c>
       <c r="P15" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="Q15" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R15" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S15" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="T15" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U15" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="V15" s="3">
         <v>0</v>
       </c>
       <c r="W15" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X15" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y15" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z15" s="3">
         <v>0</v>
@@ -2753,31 +2753,31 @@
         <v>-1</v>
       </c>
       <c r="AB15" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AC15" s="3">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="AD15" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AE15" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AF15" s="3">
         <v>0</v>
       </c>
       <c r="AG15" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AH15" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AI15" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AJ15" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AK15" s="3">
         <v>0</v>
@@ -2789,25 +2789,25 @@
         <v>1</v>
       </c>
       <c r="AN15" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AO15" s="3">
         <v>1</v>
       </c>
       <c r="AP15" s="3">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="AQ15" s="3">
         <v>-1</v>
       </c>
       <c r="AR15" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AS15" s="3">
         <v>2</v>
       </c>
       <c r="AT15" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AU15" s="3">
         <v>0</v>
@@ -2816,16 +2816,16 @@
         <v>2</v>
       </c>
       <c r="AW15" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AX15" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AY15" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AZ15" s="3">
-        <v>-2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16" ht="15.75" customHeight="1">
@@ -6476,7 +6476,7 @@
         <v>0</v>
       </c>
       <c r="E39" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F39" s="3">
         <v>-1</v>
@@ -6628,10 +6628,10 @@
         <v>1</v>
       </c>
       <c r="C40" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D40" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="E40" s="3">
         <v>-1</v>
@@ -6643,16 +6643,16 @@
         <v>0</v>
       </c>
       <c r="H40" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I40" s="3">
         <v>-1</v>
       </c>
       <c r="J40" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K40" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="L40" s="3">
         <v>1</v>
@@ -6664,10 +6664,10 @@
         <v>0</v>
       </c>
       <c r="O40" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P40" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="Q40" s="3">
         <v>0</v>
@@ -6676,40 +6676,40 @@
         <v>1</v>
       </c>
       <c r="S40" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T40" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U40" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V40" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="W40" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="X40" s="3">
         <v>1</v>
       </c>
       <c r="Y40" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z40" s="3">
         <v>0</v>
       </c>
       <c r="AA40" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AB40" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AC40" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AD40" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AE40" s="3">
         <v>1</v>
@@ -6718,13 +6718,13 @@
         <v>1</v>
       </c>
       <c r="AG40" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH40" s="3">
         <v>1</v>
       </c>
       <c r="AI40" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AJ40" s="3">
         <v>-1</v>
@@ -6733,7 +6733,7 @@
         <v>0</v>
       </c>
       <c r="AL40" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AM40" s="3">
         <v>0</v>
@@ -6742,16 +6742,16 @@
         <v>-11</v>
       </c>
       <c r="AO40" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AP40" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AQ40" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AR40" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AS40" s="3">
         <v>0</v>
@@ -6763,19 +6763,19 @@
         <v>0</v>
       </c>
       <c r="AV40" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AW40" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AX40" s="3">
         <v>1</v>
       </c>
       <c r="AY40" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AZ40" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41" ht="15.75" customHeight="1">
@@ -7272,7 +7272,7 @@
         <v>0</v>
       </c>
       <c r="G44" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H44" s="3">
         <v>0</v>
@@ -7281,10 +7281,10 @@
         <v>1</v>
       </c>
       <c r="J44" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="K44" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L44" s="3">
         <v>1</v>
@@ -7305,22 +7305,22 @@
         <v>1</v>
       </c>
       <c r="R44" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="S44" s="3">
         <v>1</v>
       </c>
       <c r="T44" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U44" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V44" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W44" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X44" s="3">
         <v>0</v>
@@ -7329,13 +7329,13 @@
         <v>1</v>
       </c>
       <c r="Z44" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA44" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB44" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AC44" s="3">
         <v>0</v>
@@ -7344,10 +7344,10 @@
         <v>0</v>
       </c>
       <c r="AE44" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AF44" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG44" s="3">
         <v>0</v>
@@ -7356,7 +7356,7 @@
         <v>1</v>
       </c>
       <c r="AI44" s="3">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="AJ44" s="3">
         <v>-1</v>
@@ -7377,16 +7377,16 @@
         <v>1</v>
       </c>
       <c r="AP44" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AQ44" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AR44" s="3">
         <v>-11</v>
       </c>
       <c r="AS44" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AT44" s="3">
         <v>1</v>
@@ -7407,7 +7407,7 @@
         <v>0</v>
       </c>
       <c r="AZ44" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="45" ht="15.75" customHeight="1">

</xml_diff>

<commit_message>
Modificações na Sojourn e Orisa
</commit_message>
<xml_diff>
--- a/dist/OWPick/_internal/heroes ally.xlsx
+++ b/dist/OWPick/_internal/heroes ally.xlsx
@@ -5203,25 +5203,25 @@
         <v>30</v>
       </c>
       <c r="B31" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="C31" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="D31" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E31" s="3">
-        <v>-1</v>
+        <v>2</v>
       </c>
       <c r="F31" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="G31" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="H31" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I31" s="3">
         <v>-1</v>
@@ -5236,7 +5236,7 @@
         <v>0</v>
       </c>
       <c r="M31" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="N31" s="3">
         <v>0</v>
@@ -5245,16 +5245,16 @@
         <v>0</v>
       </c>
       <c r="P31" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="Q31" s="3">
         <v>0</v>
       </c>
       <c r="R31" s="3">
-        <v>-2</v>
+        <v>2</v>
       </c>
       <c r="S31" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T31" s="3">
         <v>-1</v>
@@ -5263,43 +5263,43 @@
         <v>1</v>
       </c>
       <c r="V31" s="3">
-        <v>-2</v>
+        <v>1</v>
       </c>
       <c r="W31" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X31" s="3">
         <v>0</v>
       </c>
       <c r="Y31" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z31" s="3">
         <v>0</v>
       </c>
       <c r="AA31" s="3">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="AB31" s="3">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="AC31" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AD31" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AE31" s="3">
         <v>-11</v>
       </c>
       <c r="AF31" s="3">
-        <v>-2</v>
+        <v>2</v>
       </c>
       <c r="AG31" s="3">
         <v>1</v>
       </c>
       <c r="AH31" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AI31" s="3">
         <v>0</v>
@@ -5308,37 +5308,37 @@
         <v>1</v>
       </c>
       <c r="AK31" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AL31" s="3">
         <v>2</v>
       </c>
       <c r="AM31" s="3">
-        <v>-2</v>
+        <v>1</v>
       </c>
       <c r="AN31" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AO31" s="3">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AP31" s="3">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="AQ31" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AR31" s="3">
         <v>-1</v>
       </c>
       <c r="AS31" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AT31" s="3">
         <v>0</v>
       </c>
       <c r="AU31" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AV31" s="3">
         <v>0</v>
@@ -5353,7 +5353,7 @@
         <v>-1</v>
       </c>
       <c r="AZ31" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32" ht="15.75" customHeight="1">
@@ -6470,10 +6470,10 @@
         <v>1</v>
       </c>
       <c r="C39" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D39" s="3">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="E39" s="3">
         <v>2</v>
@@ -6485,76 +6485,76 @@
         <v>0</v>
       </c>
       <c r="H39" s="3">
-        <v>1</v>
+        <v>-2</v>
       </c>
       <c r="I39" s="3">
         <v>0</v>
       </c>
       <c r="J39" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K39" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L39" s="3">
         <v>1</v>
       </c>
       <c r="M39" s="3">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="N39" s="3">
         <v>0</v>
       </c>
       <c r="O39" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P39" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q39" s="3">
         <v>1</v>
       </c>
       <c r="R39" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S39" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="T39" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U39" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V39" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="W39" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="X39" s="3">
         <v>0</v>
       </c>
       <c r="Y39" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z39" s="3">
         <v>0</v>
       </c>
       <c r="AA39" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AB39" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AC39" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AD39" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AE39" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AF39" s="3">
         <v>1</v>
@@ -6566,13 +6566,13 @@
         <v>1</v>
       </c>
       <c r="AI39" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AJ39" s="3">
         <v>1</v>
       </c>
       <c r="AK39" s="3">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AL39" s="3">
         <v>1</v>
@@ -6581,13 +6581,13 @@
         <v>-11</v>
       </c>
       <c r="AN39" s="3">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AO39" s="3">
         <v>1</v>
       </c>
       <c r="AP39" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AQ39" s="3">
         <v>-1</v>
@@ -6596,7 +6596,7 @@
         <v>1</v>
       </c>
       <c r="AS39" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AT39" s="3">
         <v>1</v>
@@ -6605,10 +6605,10 @@
         <v>-1</v>
       </c>
       <c r="AV39" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AW39" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AX39" s="3">
         <v>1</v>

</xml_diff>

<commit_message>
Testes na Priorização de Counters
</commit_message>
<xml_diff>
--- a/dist/OWPick/_internal/heroes ally.xlsx
+++ b/dist/OWPick/_internal/heroes ally.xlsx
@@ -1569,13 +1569,13 @@
         <v>7</v>
       </c>
       <c r="B8" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C8" s="3">
         <v>0</v>
       </c>
       <c r="D8" s="3">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="E8" s="3">
         <v>1</v>
@@ -1599,10 +1599,10 @@
         <v>-1</v>
       </c>
       <c r="L8" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="M8" s="3">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="N8" s="3">
         <v>0</v>
@@ -1611,10 +1611,10 @@
         <v>0</v>
       </c>
       <c r="P8" s="3">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="Q8" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="R8" s="3">
         <v>1</v>
@@ -1629,7 +1629,7 @@
         <v>0</v>
       </c>
       <c r="V8" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W8" s="3">
         <v>0</v>
@@ -1641,7 +1641,7 @@
         <v>1</v>
       </c>
       <c r="Z8" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA8" s="3">
         <v>1</v>
@@ -1650,7 +1650,7 @@
         <v>1</v>
       </c>
       <c r="AC8" s="3">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="AD8" s="3">
         <v>0</v>
@@ -1659,13 +1659,13 @@
         <v>1</v>
       </c>
       <c r="AF8" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AG8" s="3">
         <v>1</v>
       </c>
       <c r="AH8" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AI8" s="3">
         <v>1</v>
@@ -1674,25 +1674,25 @@
         <v>0</v>
       </c>
       <c r="AK8" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AL8" s="3">
         <v>0</v>
       </c>
       <c r="AM8" s="3">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="AN8" s="3">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="AO8" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AP8" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AQ8" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AR8" s="3">
         <v>1</v>

</xml_diff>

<commit_message>
Ajustes no calculo do multiplicador, ajustes no Roadhog na planilha
</commit_message>
<xml_diff>
--- a/dist/OWPick/_internal/heroes ally.xlsx
+++ b/dist/OWPick/_internal/heroes ally.xlsx
@@ -1,23 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Eden\Repositorio Teste Eden\Overwatch-Best-Picks\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DAVI\Projeto\Overwatch-Best-Picks\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{035280BD-097B-4B33-9AA2-3335DC94B400}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Página1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="52">
   <si>
     <t>Hero</t>
   </si>
@@ -89,9 +92,6 @@
   </si>
   <si>
     <t>Lifeweaver</t>
-  </si>
-  <si>
-    <t>Lucio</t>
   </si>
   <si>
     <t>Mauga</t>
@@ -174,12 +174,15 @@
   <si>
     <t>Zenyatta</t>
   </si>
+  <si>
+    <t>Lúcio</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="4">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -226,20 +229,26 @@
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="4">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -248,6 +257,14 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -445,20 +462,23 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
-    <outlinePr summaryRight="0" summaryBelow="0"/>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr defaultColWidth="12.57031" defaultRowHeight="15" customHeight="1"/>
+  <dimension ref="A1:AZ1001"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="7" width="12.57031" customWidth="1"/>
+    <col min="1" max="7" width="12.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.75" customHeight="1">
+    <row r="1" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -532,91 +552,91 @@
         <v>23</v>
       </c>
       <c r="Y1" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="Z1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AB1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="AB1" s="1" t="s">
+      <c r="AC1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="AC1" s="1" t="s">
+      <c r="AD1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="AD1" s="1" t="s">
+      <c r="AE1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="AE1" s="1" t="s">
+      <c r="AF1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="AF1" s="1" t="s">
+      <c r="AG1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="AG1" s="1" t="s">
+      <c r="AH1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="AH1" s="1" t="s">
+      <c r="AI1" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="AI1" s="1" t="s">
+      <c r="AJ1" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="AJ1" s="1" t="s">
+      <c r="AK1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="AK1" s="1" t="s">
+      <c r="AL1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="AL1" s="1" t="s">
+      <c r="AM1" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="AM1" s="1" t="s">
+      <c r="AN1" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="AN1" s="1" t="s">
+      <c r="AO1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="AO1" s="1" t="s">
+      <c r="AP1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="AP1" s="1" t="s">
+      <c r="AQ1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="AQ1" s="1" t="s">
+      <c r="AR1" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="AR1" s="1" t="s">
+      <c r="AS1" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="AS1" s="1" t="s">
+      <c r="AT1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="AT1" s="1" t="s">
+      <c r="AU1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="AU1" s="1" t="s">
+      <c r="AV1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="AV1" s="1" t="s">
+      <c r="AW1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="AW1" s="1" t="s">
+      <c r="AX1" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="AX1" s="1" t="s">
+      <c r="AY1" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="AY1" s="1" t="s">
+      <c r="AZ1" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="AZ1" s="1" t="s">
-        <v>51</v>
-      </c>
     </row>
-    <row r="2" ht="15.75" customHeight="1">
+    <row r="2" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -774,7 +794,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" ht="15.75" customHeight="1">
+    <row r="3" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
@@ -932,7 +952,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" ht="15.75" customHeight="1">
+    <row r="4" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
@@ -1090,7 +1110,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" ht="15.75" customHeight="1">
+    <row r="5" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>4</v>
       </c>
@@ -1248,7 +1268,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" ht="15.75" customHeight="1">
+    <row r="6" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>5</v>
       </c>
@@ -1406,7 +1426,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" ht="15.75" customHeight="1">
+    <row r="7" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>6</v>
       </c>
@@ -1564,7 +1584,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="8" ht="15.75" customHeight="1">
+    <row r="8" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>7</v>
       </c>
@@ -1722,7 +1742,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" ht="15.75" customHeight="1">
+    <row r="9" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>8</v>
       </c>
@@ -1880,7 +1900,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="10" ht="15.75" customHeight="1">
+    <row r="10" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>9</v>
       </c>
@@ -2038,7 +2058,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="11" ht="15.75" customHeight="1">
+    <row r="11" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>10</v>
       </c>
@@ -2196,7 +2216,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" ht="15.75" customHeight="1">
+    <row r="12" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>11</v>
       </c>
@@ -2354,7 +2374,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="13" ht="15.75" customHeight="1">
+    <row r="13" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>12</v>
       </c>
@@ -2512,7 +2532,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="14" ht="15.75" customHeight="1">
+    <row r="14" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>13</v>
       </c>
@@ -2670,7 +2690,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" ht="15.75" customHeight="1">
+    <row r="15" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>14</v>
       </c>
@@ -2828,7 +2848,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" ht="15.75" customHeight="1">
+    <row r="16" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>15</v>
       </c>
@@ -2986,7 +3006,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" ht="15.75" customHeight="1">
+    <row r="17" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>16</v>
       </c>
@@ -3144,7 +3164,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" ht="15.75" customHeight="1">
+    <row r="18" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>17</v>
       </c>
@@ -3302,7 +3322,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" ht="15.75" customHeight="1">
+    <row r="19" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>18</v>
       </c>
@@ -3460,7 +3480,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" ht="15.75" customHeight="1">
+    <row r="20" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>19</v>
       </c>
@@ -3618,7 +3638,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" ht="15.75" customHeight="1">
+    <row r="21" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>20</v>
       </c>
@@ -3776,7 +3796,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" ht="15.75" customHeight="1">
+    <row r="22" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>21</v>
       </c>
@@ -3934,7 +3954,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" ht="15.75" customHeight="1">
+    <row r="23" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>22</v>
       </c>
@@ -4092,7 +4112,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" ht="15.75" customHeight="1">
+    <row r="24" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>23</v>
       </c>
@@ -4250,9 +4270,9 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="25" ht="15.75" customHeight="1">
+    <row r="25" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>24</v>
+        <v>51</v>
       </c>
       <c r="B25" s="3">
         <v>-1</v>
@@ -4408,9 +4428,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" ht="15.75" customHeight="1">
+    <row r="26" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B26" s="3">
         <v>-1</v>
@@ -4566,9 +4586,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" ht="15.75" customHeight="1">
+    <row r="27" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B27" s="3">
         <v>1</v>
@@ -4724,9 +4744,9 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="28" ht="15.75" customHeight="1">
+    <row r="28" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B28" s="3">
         <v>0</v>
@@ -4882,9 +4902,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" ht="15.75" customHeight="1">
+    <row r="29" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B29" s="3">
         <v>2</v>
@@ -5040,9 +5060,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" ht="15.75" customHeight="1">
+    <row r="30" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B30" s="3">
         <v>-1</v>
@@ -5198,9 +5218,9 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="31" ht="15.75" customHeight="1">
+    <row r="31" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B31" s="3">
         <v>1</v>
@@ -5356,9 +5376,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" ht="15.75" customHeight="1">
+    <row r="32" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B32" s="3">
         <v>-2</v>
@@ -5514,9 +5534,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" ht="15.75" customHeight="1">
+    <row r="33" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B33" s="3">
         <v>-1</v>
@@ -5672,9 +5692,9 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="34" ht="15.75" customHeight="1">
+    <row r="34" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B34" s="3">
         <v>-1</v>
@@ -5830,9 +5850,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" ht="15.75" customHeight="1">
+    <row r="35" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B35" s="3">
         <v>1</v>
@@ -5988,9 +6008,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" ht="15.75" customHeight="1">
+    <row r="36" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B36" s="3">
         <v>2</v>
@@ -6146,167 +6166,167 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="37" ht="15.75" customHeight="1">
+    <row r="37" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B37" s="3">
+        <v>0</v>
+      </c>
+      <c r="C37" s="3">
+        <v>0</v>
+      </c>
+      <c r="D37" s="3">
+        <v>0</v>
+      </c>
+      <c r="E37" s="3">
+        <v>0</v>
+      </c>
+      <c r="F37" s="3">
+        <v>0</v>
+      </c>
+      <c r="G37" s="3">
+        <v>0</v>
+      </c>
+      <c r="H37" s="3">
+        <v>0</v>
+      </c>
+      <c r="I37" s="3">
+        <v>0</v>
+      </c>
+      <c r="J37" s="3">
+        <v>0</v>
+      </c>
+      <c r="K37" s="3">
+        <v>0</v>
+      </c>
+      <c r="L37" s="3">
+        <v>0</v>
+      </c>
+      <c r="M37" s="3">
+        <v>0</v>
+      </c>
+      <c r="N37" s="3">
+        <v>0</v>
+      </c>
+      <c r="O37" s="3">
+        <v>0</v>
+      </c>
+      <c r="P37" s="3">
+        <v>0</v>
+      </c>
+      <c r="Q37" s="3">
+        <v>0</v>
+      </c>
+      <c r="R37" s="3">
+        <v>0</v>
+      </c>
+      <c r="S37" s="3">
+        <v>0</v>
+      </c>
+      <c r="T37" s="3">
+        <v>0</v>
+      </c>
+      <c r="U37" s="3">
+        <v>0</v>
+      </c>
+      <c r="V37" s="3">
+        <v>0</v>
+      </c>
+      <c r="W37" s="3">
+        <v>0</v>
+      </c>
+      <c r="X37" s="3">
+        <v>0</v>
+      </c>
+      <c r="Y37" s="3">
+        <v>0</v>
+      </c>
+      <c r="Z37" s="3">
+        <v>0</v>
+      </c>
+      <c r="AA37" s="3">
+        <v>0</v>
+      </c>
+      <c r="AB37" s="3">
+        <v>0</v>
+      </c>
+      <c r="AC37" s="3">
+        <v>0</v>
+      </c>
+      <c r="AD37" s="3">
+        <v>0</v>
+      </c>
+      <c r="AE37" s="3">
+        <v>0</v>
+      </c>
+      <c r="AF37" s="3">
+        <v>0</v>
+      </c>
+      <c r="AG37" s="3">
+        <v>0</v>
+      </c>
+      <c r="AH37" s="3">
+        <v>0</v>
+      </c>
+      <c r="AI37" s="3">
+        <v>0</v>
+      </c>
+      <c r="AJ37" s="3">
+        <v>0</v>
+      </c>
+      <c r="AK37" s="3">
+        <v>0</v>
+      </c>
+      <c r="AL37" s="3">
+        <v>0</v>
+      </c>
+      <c r="AM37" s="3">
+        <v>0</v>
+      </c>
+      <c r="AN37" s="3">
+        <v>0</v>
+      </c>
+      <c r="AO37" s="3">
+        <v>0</v>
+      </c>
+      <c r="AP37" s="3">
+        <v>0</v>
+      </c>
+      <c r="AQ37" s="3">
+        <v>0</v>
+      </c>
+      <c r="AR37" s="3">
+        <v>0</v>
+      </c>
+      <c r="AS37" s="3">
+        <v>0</v>
+      </c>
+      <c r="AT37" s="3">
+        <v>0</v>
+      </c>
+      <c r="AU37" s="3">
+        <v>0</v>
+      </c>
+      <c r="AV37" s="3">
+        <v>0</v>
+      </c>
+      <c r="AW37" s="3">
+        <v>0</v>
+      </c>
+      <c r="AX37" s="3">
+        <v>0</v>
+      </c>
+      <c r="AY37" s="3">
+        <v>0</v>
+      </c>
+      <c r="AZ37" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="2" t="s">
         <v>36</v>
-      </c>
-      <c r="B37" s="3">
-        <v>0</v>
-      </c>
-      <c r="C37" s="3">
-        <v>0</v>
-      </c>
-      <c r="D37" s="3">
-        <v>0</v>
-      </c>
-      <c r="E37" s="3">
-        <v>0</v>
-      </c>
-      <c r="F37" s="3">
-        <v>0</v>
-      </c>
-      <c r="G37" s="3">
-        <v>0</v>
-      </c>
-      <c r="H37" s="3">
-        <v>0</v>
-      </c>
-      <c r="I37" s="3">
-        <v>0</v>
-      </c>
-      <c r="J37" s="3">
-        <v>0</v>
-      </c>
-      <c r="K37" s="3">
-        <v>0</v>
-      </c>
-      <c r="L37" s="3">
-        <v>0</v>
-      </c>
-      <c r="M37" s="3">
-        <v>0</v>
-      </c>
-      <c r="N37" s="3">
-        <v>0</v>
-      </c>
-      <c r="O37" s="3">
-        <v>0</v>
-      </c>
-      <c r="P37" s="3">
-        <v>0</v>
-      </c>
-      <c r="Q37" s="3">
-        <v>0</v>
-      </c>
-      <c r="R37" s="3">
-        <v>0</v>
-      </c>
-      <c r="S37" s="3">
-        <v>0</v>
-      </c>
-      <c r="T37" s="3">
-        <v>0</v>
-      </c>
-      <c r="U37" s="3">
-        <v>0</v>
-      </c>
-      <c r="V37" s="3">
-        <v>0</v>
-      </c>
-      <c r="W37" s="3">
-        <v>0</v>
-      </c>
-      <c r="X37" s="3">
-        <v>0</v>
-      </c>
-      <c r="Y37" s="3">
-        <v>0</v>
-      </c>
-      <c r="Z37" s="3">
-        <v>0</v>
-      </c>
-      <c r="AA37" s="3">
-        <v>0</v>
-      </c>
-      <c r="AB37" s="3">
-        <v>0</v>
-      </c>
-      <c r="AC37" s="3">
-        <v>0</v>
-      </c>
-      <c r="AD37" s="3">
-        <v>0</v>
-      </c>
-      <c r="AE37" s="3">
-        <v>0</v>
-      </c>
-      <c r="AF37" s="3">
-        <v>0</v>
-      </c>
-      <c r="AG37" s="3">
-        <v>0</v>
-      </c>
-      <c r="AH37" s="3">
-        <v>0</v>
-      </c>
-      <c r="AI37" s="3">
-        <v>0</v>
-      </c>
-      <c r="AJ37" s="3">
-        <v>0</v>
-      </c>
-      <c r="AK37" s="3">
-        <v>0</v>
-      </c>
-      <c r="AL37" s="3">
-        <v>0</v>
-      </c>
-      <c r="AM37" s="3">
-        <v>0</v>
-      </c>
-      <c r="AN37" s="3">
-        <v>0</v>
-      </c>
-      <c r="AO37" s="3">
-        <v>0</v>
-      </c>
-      <c r="AP37" s="3">
-        <v>0</v>
-      </c>
-      <c r="AQ37" s="3">
-        <v>0</v>
-      </c>
-      <c r="AR37" s="3">
-        <v>0</v>
-      </c>
-      <c r="AS37" s="3">
-        <v>0</v>
-      </c>
-      <c r="AT37" s="3">
-        <v>0</v>
-      </c>
-      <c r="AU37" s="3">
-        <v>0</v>
-      </c>
-      <c r="AV37" s="3">
-        <v>0</v>
-      </c>
-      <c r="AW37" s="3">
-        <v>0</v>
-      </c>
-      <c r="AX37" s="3">
-        <v>0</v>
-      </c>
-      <c r="AY37" s="3">
-        <v>0</v>
-      </c>
-      <c r="AZ37" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38" ht="15.75" customHeight="1">
-      <c r="A38" s="2" t="s">
-        <v>37</v>
       </c>
       <c r="B38" s="3">
         <v>1</v>
@@ -6462,9 +6482,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" ht="15.75" customHeight="1">
+    <row r="39" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B39" s="3">
         <v>1</v>
@@ -6620,9 +6640,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" ht="15.75" customHeight="1">
+    <row r="40" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B40" s="3">
         <v>1</v>
@@ -6778,9 +6798,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" ht="15.75" customHeight="1">
+    <row r="41" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B41" s="3">
         <v>-1</v>
@@ -6936,9 +6956,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" ht="15.75" customHeight="1">
+    <row r="42" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B42" s="3">
         <v>0</v>
@@ -7094,9 +7114,9 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="43" ht="15.75" customHeight="1">
+    <row r="43" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B43" s="3">
         <v>1</v>
@@ -7252,9 +7272,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" ht="15.75" customHeight="1">
+    <row r="44" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B44" s="3">
         <v>0</v>
@@ -7410,9 +7430,9 @@
         <v>2</v>
       </c>
     </row>
-    <row r="45" ht="15.75" customHeight="1">
+    <row r="45" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B45" s="3">
         <v>-2</v>
@@ -7568,9 +7588,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46" ht="15.75" customHeight="1">
+    <row r="46" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B46" s="3">
         <v>0</v>
@@ -7726,9 +7746,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" ht="15.75" customHeight="1">
+    <row r="47" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B47" s="3">
         <v>1</v>
@@ -7884,9 +7904,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" ht="15.75" customHeight="1">
+    <row r="48" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B48" s="3">
         <v>2</v>
@@ -8042,9 +8062,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="49" ht="15.75" customHeight="1">
+    <row r="49" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B49" s="3">
         <v>0</v>
@@ -8200,9 +8220,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" ht="15.75" customHeight="1">
+    <row r="50" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B50" s="3">
         <v>-1</v>
@@ -8358,9 +8378,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" ht="15.75" customHeight="1">
+    <row r="51" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B51" s="3">
         <v>1</v>
@@ -8516,9 +8536,9 @@
         <v>2</v>
       </c>
     </row>
-    <row r="52" ht="15.75" customHeight="1">
+    <row r="52" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B52" s="3">
         <v>1</v>
@@ -8674,959 +8694,959 @@
         <v>-11</v>
       </c>
     </row>
-    <row r="53" ht="15.75" customHeight="1">
+    <row r="53" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="J53" s="3"/>
     </row>
-    <row r="54" ht="15.75" customHeight="1"/>
-    <row r="55" ht="15.75" customHeight="1"/>
-    <row r="56" ht="15.75" customHeight="1"/>
-    <row r="57" ht="15.75" customHeight="1"/>
-    <row r="58" ht="15.75" customHeight="1"/>
-    <row r="59" ht="15.75" customHeight="1"/>
-    <row r="60" ht="15.75" customHeight="1"/>
-    <row r="61" ht="15.75" customHeight="1"/>
-    <row r="62" ht="15.75" customHeight="1"/>
-    <row r="63" ht="15.75" customHeight="1"/>
-    <row r="64" ht="15.75" customHeight="1"/>
-    <row r="65" ht="15.75" customHeight="1"/>
-    <row r="66" ht="15.75" customHeight="1"/>
-    <row r="67" ht="15.75" customHeight="1"/>
-    <row r="68" ht="15.75" customHeight="1"/>
-    <row r="69" ht="15.75" customHeight="1"/>
-    <row r="70" ht="15.75" customHeight="1"/>
-    <row r="71" ht="15.75" customHeight="1"/>
-    <row r="72" ht="15.75" customHeight="1"/>
-    <row r="73" ht="15.75" customHeight="1"/>
-    <row r="74" ht="15.75" customHeight="1"/>
-    <row r="75" ht="15.75" customHeight="1"/>
-    <row r="76" ht="15.75" customHeight="1"/>
-    <row r="77" ht="15.75" customHeight="1"/>
-    <row r="78" ht="15.75" customHeight="1"/>
-    <row r="79" ht="15.75" customHeight="1"/>
-    <row r="80" ht="15.75" customHeight="1"/>
-    <row r="81" ht="15.75" customHeight="1"/>
-    <row r="82" ht="15.75" customHeight="1"/>
-    <row r="83" ht="15.75" customHeight="1"/>
-    <row r="84" ht="15.75" customHeight="1"/>
-    <row r="85" ht="15.75" customHeight="1"/>
-    <row r="86" ht="15.75" customHeight="1"/>
-    <row r="87" ht="15.75" customHeight="1"/>
-    <row r="88" ht="15.75" customHeight="1"/>
-    <row r="89" ht="15.75" customHeight="1"/>
-    <row r="90" ht="15.75" customHeight="1"/>
-    <row r="91" ht="15.75" customHeight="1"/>
-    <row r="92" ht="15.75" customHeight="1"/>
-    <row r="93" ht="15.75" customHeight="1"/>
-    <row r="94" ht="15.75" customHeight="1"/>
-    <row r="95" ht="15.75" customHeight="1"/>
-    <row r="96" ht="15.75" customHeight="1"/>
-    <row r="97" ht="15.75" customHeight="1"/>
-    <row r="98" ht="15.75" customHeight="1"/>
-    <row r="99" ht="15.75" customHeight="1"/>
-    <row r="100" ht="15.75" customHeight="1"/>
-    <row r="101" ht="15.75" customHeight="1"/>
-    <row r="102" ht="15.75" customHeight="1"/>
-    <row r="103" ht="15.75" customHeight="1"/>
-    <row r="104" ht="15.75" customHeight="1"/>
-    <row r="105" ht="15.75" customHeight="1"/>
-    <row r="106" ht="15.75" customHeight="1"/>
-    <row r="107" ht="15.75" customHeight="1"/>
-    <row r="108" ht="15.75" customHeight="1"/>
-    <row r="109" ht="15.75" customHeight="1"/>
-    <row r="110" ht="15.75" customHeight="1"/>
-    <row r="111" ht="15.75" customHeight="1"/>
-    <row r="112" ht="15.75" customHeight="1"/>
-    <row r="113" ht="15.75" customHeight="1"/>
-    <row r="114" ht="15.75" customHeight="1"/>
-    <row r="115" ht="15.75" customHeight="1"/>
-    <row r="116" ht="15.75" customHeight="1"/>
-    <row r="117" ht="15.75" customHeight="1"/>
-    <row r="118" ht="15.75" customHeight="1"/>
-    <row r="119" ht="15.75" customHeight="1"/>
-    <row r="120" ht="15.75" customHeight="1"/>
-    <row r="121" ht="15.75" customHeight="1"/>
-    <row r="122" ht="15.75" customHeight="1"/>
-    <row r="123" ht="15.75" customHeight="1"/>
-    <row r="124" ht="15.75" customHeight="1"/>
-    <row r="125" ht="15.75" customHeight="1"/>
-    <row r="126" ht="15.75" customHeight="1"/>
-    <row r="127" ht="15.75" customHeight="1"/>
-    <row r="128" ht="15.75" customHeight="1"/>
-    <row r="129" ht="15.75" customHeight="1"/>
-    <row r="130" ht="15.75" customHeight="1"/>
-    <row r="131" ht="15.75" customHeight="1"/>
-    <row r="132" ht="15.75" customHeight="1"/>
-    <row r="133" ht="15.75" customHeight="1"/>
-    <row r="134" ht="15.75" customHeight="1"/>
-    <row r="135" ht="15.75" customHeight="1"/>
-    <row r="136" ht="15.75" customHeight="1"/>
-    <row r="137" ht="15.75" customHeight="1"/>
-    <row r="138" ht="15.75" customHeight="1"/>
-    <row r="139" ht="15.75" customHeight="1"/>
-    <row r="140" ht="15.75" customHeight="1"/>
-    <row r="141" ht="15.75" customHeight="1"/>
-    <row r="142" ht="15.75" customHeight="1"/>
-    <row r="143" ht="15.75" customHeight="1"/>
-    <row r="144" ht="15.75" customHeight="1"/>
-    <row r="145" ht="15.75" customHeight="1"/>
-    <row r="146" ht="15.75" customHeight="1"/>
-    <row r="147" ht="15.75" customHeight="1"/>
-    <row r="148" ht="15.75" customHeight="1"/>
-    <row r="149" ht="15.75" customHeight="1"/>
-    <row r="150" ht="15.75" customHeight="1"/>
-    <row r="151" ht="15.75" customHeight="1"/>
-    <row r="152" ht="15.75" customHeight="1"/>
-    <row r="153" ht="15.75" customHeight="1"/>
-    <row r="154" ht="15.75" customHeight="1"/>
-    <row r="155" ht="15.75" customHeight="1"/>
-    <row r="156" ht="15.75" customHeight="1"/>
-    <row r="157" ht="15.75" customHeight="1"/>
-    <row r="158" ht="15.75" customHeight="1"/>
-    <row r="159" ht="15.75" customHeight="1"/>
-    <row r="160" ht="15.75" customHeight="1"/>
-    <row r="161" ht="15.75" customHeight="1"/>
-    <row r="162" ht="15.75" customHeight="1"/>
-    <row r="163" ht="15.75" customHeight="1"/>
-    <row r="164" ht="15.75" customHeight="1"/>
-    <row r="165" ht="15.75" customHeight="1"/>
-    <row r="166" ht="15.75" customHeight="1"/>
-    <row r="167" ht="15.75" customHeight="1"/>
-    <row r="168" ht="15.75" customHeight="1"/>
-    <row r="169" ht="15.75" customHeight="1"/>
-    <row r="170" ht="15.75" customHeight="1"/>
-    <row r="171" ht="15.75" customHeight="1"/>
-    <row r="172" ht="15.75" customHeight="1"/>
-    <row r="173" ht="15.75" customHeight="1"/>
-    <row r="174" ht="15.75" customHeight="1"/>
-    <row r="175" ht="15.75" customHeight="1"/>
-    <row r="176" ht="15.75" customHeight="1"/>
-    <row r="177" ht="15.75" customHeight="1"/>
-    <row r="178" ht="15.75" customHeight="1"/>
-    <row r="179" ht="15.75" customHeight="1"/>
-    <row r="180" ht="15.75" customHeight="1"/>
-    <row r="181" ht="15.75" customHeight="1"/>
-    <row r="182" ht="15.75" customHeight="1"/>
-    <row r="183" ht="15.75" customHeight="1"/>
-    <row r="184" ht="15.75" customHeight="1"/>
-    <row r="185" ht="15.75" customHeight="1"/>
-    <row r="186" ht="15.75" customHeight="1"/>
-    <row r="187" ht="15.75" customHeight="1"/>
-    <row r="188" ht="15.75" customHeight="1"/>
-    <row r="189" ht="15.75" customHeight="1"/>
-    <row r="190" ht="15.75" customHeight="1"/>
-    <row r="191" ht="15.75" customHeight="1"/>
-    <row r="192" ht="15.75" customHeight="1"/>
-    <row r="193" ht="15.75" customHeight="1"/>
-    <row r="194" ht="15.75" customHeight="1"/>
-    <row r="195" ht="15.75" customHeight="1"/>
-    <row r="196" ht="15.75" customHeight="1"/>
-    <row r="197" ht="15.75" customHeight="1"/>
-    <row r="198" ht="15.75" customHeight="1"/>
-    <row r="199" ht="15.75" customHeight="1"/>
-    <row r="200" ht="15.75" customHeight="1"/>
-    <row r="201" ht="15.75" customHeight="1"/>
-    <row r="202" ht="15.75" customHeight="1"/>
-    <row r="203" ht="15.75" customHeight="1"/>
-    <row r="204" ht="15.75" customHeight="1"/>
-    <row r="205" ht="15.75" customHeight="1"/>
-    <row r="206" ht="15.75" customHeight="1"/>
-    <row r="207" ht="15.75" customHeight="1"/>
-    <row r="208" ht="15.75" customHeight="1"/>
-    <row r="209" ht="15.75" customHeight="1"/>
-    <row r="210" ht="15.75" customHeight="1"/>
-    <row r="211" ht="15.75" customHeight="1"/>
-    <row r="212" ht="15.75" customHeight="1"/>
-    <row r="213" ht="15.75" customHeight="1"/>
-    <row r="214" ht="15.75" customHeight="1"/>
-    <row r="215" ht="15.75" customHeight="1"/>
-    <row r="216" ht="15.75" customHeight="1"/>
-    <row r="217" ht="15.75" customHeight="1"/>
-    <row r="218" ht="15.75" customHeight="1"/>
-    <row r="219" ht="15.75" customHeight="1"/>
-    <row r="220" ht="15.75" customHeight="1"/>
-    <row r="221" ht="15.75" customHeight="1"/>
-    <row r="222" ht="15.75" customHeight="1"/>
-    <row r="223" ht="15.75" customHeight="1"/>
-    <row r="224" ht="15.75" customHeight="1"/>
-    <row r="225" ht="15.75" customHeight="1"/>
-    <row r="226" ht="15.75" customHeight="1"/>
-    <row r="227" ht="15.75" customHeight="1"/>
-    <row r="228" ht="15.75" customHeight="1"/>
-    <row r="229" ht="15.75" customHeight="1"/>
-    <row r="230" ht="15.75" customHeight="1"/>
-    <row r="231" ht="15.75" customHeight="1"/>
-    <row r="232" ht="15.75" customHeight="1"/>
-    <row r="233" ht="15.75" customHeight="1"/>
-    <row r="234" ht="15.75" customHeight="1"/>
-    <row r="235" ht="15.75" customHeight="1"/>
-    <row r="236" ht="15.75" customHeight="1"/>
-    <row r="237" ht="15.75" customHeight="1"/>
-    <row r="238" ht="15.75" customHeight="1"/>
-    <row r="239" ht="15.75" customHeight="1"/>
-    <row r="240" ht="15.75" customHeight="1"/>
-    <row r="241" ht="15.75" customHeight="1"/>
-    <row r="242" ht="15.75" customHeight="1"/>
-    <row r="243" ht="15.75" customHeight="1"/>
-    <row r="244" ht="15.75" customHeight="1"/>
-    <row r="245" ht="15.75" customHeight="1"/>
-    <row r="246" ht="15.75" customHeight="1"/>
-    <row r="247" ht="15.75" customHeight="1"/>
-    <row r="248" ht="15.75" customHeight="1"/>
-    <row r="249" ht="15.75" customHeight="1"/>
-    <row r="250" ht="15.75" customHeight="1"/>
-    <row r="251" ht="15.75" customHeight="1"/>
-    <row r="252" ht="15.75" customHeight="1"/>
-    <row r="253" ht="15.75" customHeight="1"/>
-    <row r="254" ht="15.75" customHeight="1"/>
-    <row r="255" ht="15.75" customHeight="1"/>
-    <row r="256" ht="15.75" customHeight="1"/>
-    <row r="257" ht="15.75" customHeight="1"/>
-    <row r="258" ht="15.75" customHeight="1"/>
-    <row r="259" ht="15.75" customHeight="1"/>
-    <row r="260" ht="15.75" customHeight="1"/>
-    <row r="261" ht="15.75" customHeight="1"/>
-    <row r="262" ht="15.75" customHeight="1"/>
-    <row r="263" ht="15.75" customHeight="1"/>
-    <row r="264" ht="15.75" customHeight="1"/>
-    <row r="265" ht="15.75" customHeight="1"/>
-    <row r="266" ht="15.75" customHeight="1"/>
-    <row r="267" ht="15.75" customHeight="1"/>
-    <row r="268" ht="15.75" customHeight="1"/>
-    <row r="269" ht="15.75" customHeight="1"/>
-    <row r="270" ht="15.75" customHeight="1"/>
-    <row r="271" ht="15.75" customHeight="1"/>
-    <row r="272" ht="15.75" customHeight="1"/>
-    <row r="273" ht="15.75" customHeight="1"/>
-    <row r="274" ht="15.75" customHeight="1"/>
-    <row r="275" ht="15.75" customHeight="1"/>
-    <row r="276" ht="15.75" customHeight="1"/>
-    <row r="277" ht="15.75" customHeight="1"/>
-    <row r="278" ht="15.75" customHeight="1"/>
-    <row r="279" ht="15.75" customHeight="1"/>
-    <row r="280" ht="15.75" customHeight="1"/>
-    <row r="281" ht="15.75" customHeight="1"/>
-    <row r="282" ht="15.75" customHeight="1"/>
-    <row r="283" ht="15.75" customHeight="1"/>
-    <row r="284" ht="15.75" customHeight="1"/>
-    <row r="285" ht="15.75" customHeight="1"/>
-    <row r="286" ht="15.75" customHeight="1"/>
-    <row r="287" ht="15.75" customHeight="1"/>
-    <row r="288" ht="15.75" customHeight="1"/>
-    <row r="289" ht="15.75" customHeight="1"/>
-    <row r="290" ht="15.75" customHeight="1"/>
-    <row r="291" ht="15.75" customHeight="1"/>
-    <row r="292" ht="15.75" customHeight="1"/>
-    <row r="293" ht="15.75" customHeight="1"/>
-    <row r="294" ht="15.75" customHeight="1"/>
-    <row r="295" ht="15.75" customHeight="1"/>
-    <row r="296" ht="15.75" customHeight="1"/>
-    <row r="297" ht="15.75" customHeight="1"/>
-    <row r="298" ht="15.75" customHeight="1"/>
-    <row r="299" ht="15.75" customHeight="1"/>
-    <row r="300" ht="15.75" customHeight="1"/>
-    <row r="301" ht="15.75" customHeight="1"/>
-    <row r="302" ht="15.75" customHeight="1"/>
-    <row r="303" ht="15.75" customHeight="1"/>
-    <row r="304" ht="15.75" customHeight="1"/>
-    <row r="305" ht="15.75" customHeight="1"/>
-    <row r="306" ht="15.75" customHeight="1"/>
-    <row r="307" ht="15.75" customHeight="1"/>
-    <row r="308" ht="15.75" customHeight="1"/>
-    <row r="309" ht="15.75" customHeight="1"/>
-    <row r="310" ht="15.75" customHeight="1"/>
-    <row r="311" ht="15.75" customHeight="1"/>
-    <row r="312" ht="15.75" customHeight="1"/>
-    <row r="313" ht="15.75" customHeight="1"/>
-    <row r="314" ht="15.75" customHeight="1"/>
-    <row r="315" ht="15.75" customHeight="1"/>
-    <row r="316" ht="15.75" customHeight="1"/>
-    <row r="317" ht="15.75" customHeight="1"/>
-    <row r="318" ht="15.75" customHeight="1"/>
-    <row r="319" ht="15.75" customHeight="1"/>
-    <row r="320" ht="15.75" customHeight="1"/>
-    <row r="321" ht="15.75" customHeight="1"/>
-    <row r="322" ht="15.75" customHeight="1"/>
-    <row r="323" ht="15.75" customHeight="1"/>
-    <row r="324" ht="15.75" customHeight="1"/>
-    <row r="325" ht="15.75" customHeight="1"/>
-    <row r="326" ht="15.75" customHeight="1"/>
-    <row r="327" ht="15.75" customHeight="1"/>
-    <row r="328" ht="15.75" customHeight="1"/>
-    <row r="329" ht="15.75" customHeight="1"/>
-    <row r="330" ht="15.75" customHeight="1"/>
-    <row r="331" ht="15.75" customHeight="1"/>
-    <row r="332" ht="15.75" customHeight="1"/>
-    <row r="333" ht="15.75" customHeight="1"/>
-    <row r="334" ht="15.75" customHeight="1"/>
-    <row r="335" ht="15.75" customHeight="1"/>
-    <row r="336" ht="15.75" customHeight="1"/>
-    <row r="337" ht="15.75" customHeight="1"/>
-    <row r="338" ht="15.75" customHeight="1"/>
-    <row r="339" ht="15.75" customHeight="1"/>
-    <row r="340" ht="15.75" customHeight="1"/>
-    <row r="341" ht="15.75" customHeight="1"/>
-    <row r="342" ht="15.75" customHeight="1"/>
-    <row r="343" ht="15.75" customHeight="1"/>
-    <row r="344" ht="15.75" customHeight="1"/>
-    <row r="345" ht="15.75" customHeight="1"/>
-    <row r="346" ht="15.75" customHeight="1"/>
-    <row r="347" ht="15.75" customHeight="1"/>
-    <row r="348" ht="15.75" customHeight="1"/>
-    <row r="349" ht="15.75" customHeight="1"/>
-    <row r="350" ht="15.75" customHeight="1"/>
-    <row r="351" ht="15.75" customHeight="1"/>
-    <row r="352" ht="15.75" customHeight="1"/>
-    <row r="353" ht="15.75" customHeight="1"/>
-    <row r="354" ht="15.75" customHeight="1"/>
-    <row r="355" ht="15.75" customHeight="1"/>
-    <row r="356" ht="15.75" customHeight="1"/>
-    <row r="357" ht="15.75" customHeight="1"/>
-    <row r="358" ht="15.75" customHeight="1"/>
-    <row r="359" ht="15.75" customHeight="1"/>
-    <row r="360" ht="15.75" customHeight="1"/>
-    <row r="361" ht="15.75" customHeight="1"/>
-    <row r="362" ht="15.75" customHeight="1"/>
-    <row r="363" ht="15.75" customHeight="1"/>
-    <row r="364" ht="15.75" customHeight="1"/>
-    <row r="365" ht="15.75" customHeight="1"/>
-    <row r="366" ht="15.75" customHeight="1"/>
-    <row r="367" ht="15.75" customHeight="1"/>
-    <row r="368" ht="15.75" customHeight="1"/>
-    <row r="369" ht="15.75" customHeight="1"/>
-    <row r="370" ht="15.75" customHeight="1"/>
-    <row r="371" ht="15.75" customHeight="1"/>
-    <row r="372" ht="15.75" customHeight="1"/>
-    <row r="373" ht="15.75" customHeight="1"/>
-    <row r="374" ht="15.75" customHeight="1"/>
-    <row r="375" ht="15.75" customHeight="1"/>
-    <row r="376" ht="15.75" customHeight="1"/>
-    <row r="377" ht="15.75" customHeight="1"/>
-    <row r="378" ht="15.75" customHeight="1"/>
-    <row r="379" ht="15.75" customHeight="1"/>
-    <row r="380" ht="15.75" customHeight="1"/>
-    <row r="381" ht="15.75" customHeight="1"/>
-    <row r="382" ht="15.75" customHeight="1"/>
-    <row r="383" ht="15.75" customHeight="1"/>
-    <row r="384" ht="15.75" customHeight="1"/>
-    <row r="385" ht="15.75" customHeight="1"/>
-    <row r="386" ht="15.75" customHeight="1"/>
-    <row r="387" ht="15.75" customHeight="1"/>
-    <row r="388" ht="15.75" customHeight="1"/>
-    <row r="389" ht="15.75" customHeight="1"/>
-    <row r="390" ht="15.75" customHeight="1"/>
-    <row r="391" ht="15.75" customHeight="1"/>
-    <row r="392" ht="15.75" customHeight="1"/>
-    <row r="393" ht="15.75" customHeight="1"/>
-    <row r="394" ht="15.75" customHeight="1"/>
-    <row r="395" ht="15.75" customHeight="1"/>
-    <row r="396" ht="15.75" customHeight="1"/>
-    <row r="397" ht="15.75" customHeight="1"/>
-    <row r="398" ht="15.75" customHeight="1"/>
-    <row r="399" ht="15.75" customHeight="1"/>
-    <row r="400" ht="15.75" customHeight="1"/>
-    <row r="401" ht="15.75" customHeight="1"/>
-    <row r="402" ht="15.75" customHeight="1"/>
-    <row r="403" ht="15.75" customHeight="1"/>
-    <row r="404" ht="15.75" customHeight="1"/>
-    <row r="405" ht="15.75" customHeight="1"/>
-    <row r="406" ht="15.75" customHeight="1"/>
-    <row r="407" ht="15.75" customHeight="1"/>
-    <row r="408" ht="15.75" customHeight="1"/>
-    <row r="409" ht="15.75" customHeight="1"/>
-    <row r="410" ht="15.75" customHeight="1"/>
-    <row r="411" ht="15.75" customHeight="1"/>
-    <row r="412" ht="15.75" customHeight="1"/>
-    <row r="413" ht="15.75" customHeight="1"/>
-    <row r="414" ht="15.75" customHeight="1"/>
-    <row r="415" ht="15.75" customHeight="1"/>
-    <row r="416" ht="15.75" customHeight="1"/>
-    <row r="417" ht="15.75" customHeight="1"/>
-    <row r="418" ht="15.75" customHeight="1"/>
-    <row r="419" ht="15.75" customHeight="1"/>
-    <row r="420" ht="15.75" customHeight="1"/>
-    <row r="421" ht="15.75" customHeight="1"/>
-    <row r="422" ht="15.75" customHeight="1"/>
-    <row r="423" ht="15.75" customHeight="1"/>
-    <row r="424" ht="15.75" customHeight="1"/>
-    <row r="425" ht="15.75" customHeight="1"/>
-    <row r="426" ht="15.75" customHeight="1"/>
-    <row r="427" ht="15.75" customHeight="1"/>
-    <row r="428" ht="15.75" customHeight="1"/>
-    <row r="429" ht="15.75" customHeight="1"/>
-    <row r="430" ht="15.75" customHeight="1"/>
-    <row r="431" ht="15.75" customHeight="1"/>
-    <row r="432" ht="15.75" customHeight="1"/>
-    <row r="433" ht="15.75" customHeight="1"/>
-    <row r="434" ht="15.75" customHeight="1"/>
-    <row r="435" ht="15.75" customHeight="1"/>
-    <row r="436" ht="15.75" customHeight="1"/>
-    <row r="437" ht="15.75" customHeight="1"/>
-    <row r="438" ht="15.75" customHeight="1"/>
-    <row r="439" ht="15.75" customHeight="1"/>
-    <row r="440" ht="15.75" customHeight="1"/>
-    <row r="441" ht="15.75" customHeight="1"/>
-    <row r="442" ht="15.75" customHeight="1"/>
-    <row r="443" ht="15.75" customHeight="1"/>
-    <row r="444" ht="15.75" customHeight="1"/>
-    <row r="445" ht="15.75" customHeight="1"/>
-    <row r="446" ht="15.75" customHeight="1"/>
-    <row r="447" ht="15.75" customHeight="1"/>
-    <row r="448" ht="15.75" customHeight="1"/>
-    <row r="449" ht="15.75" customHeight="1"/>
-    <row r="450" ht="15.75" customHeight="1"/>
-    <row r="451" ht="15.75" customHeight="1"/>
-    <row r="452" ht="15.75" customHeight="1"/>
-    <row r="453" ht="15.75" customHeight="1"/>
-    <row r="454" ht="15.75" customHeight="1"/>
-    <row r="455" ht="15.75" customHeight="1"/>
-    <row r="456" ht="15.75" customHeight="1"/>
-    <row r="457" ht="15.75" customHeight="1"/>
-    <row r="458" ht="15.75" customHeight="1"/>
-    <row r="459" ht="15.75" customHeight="1"/>
-    <row r="460" ht="15.75" customHeight="1"/>
-    <row r="461" ht="15.75" customHeight="1"/>
-    <row r="462" ht="15.75" customHeight="1"/>
-    <row r="463" ht="15.75" customHeight="1"/>
-    <row r="464" ht="15.75" customHeight="1"/>
-    <row r="465" ht="15.75" customHeight="1"/>
-    <row r="466" ht="15.75" customHeight="1"/>
-    <row r="467" ht="15.75" customHeight="1"/>
-    <row r="468" ht="15.75" customHeight="1"/>
-    <row r="469" ht="15.75" customHeight="1"/>
-    <row r="470" ht="15.75" customHeight="1"/>
-    <row r="471" ht="15.75" customHeight="1"/>
-    <row r="472" ht="15.75" customHeight="1"/>
-    <row r="473" ht="15.75" customHeight="1"/>
-    <row r="474" ht="15.75" customHeight="1"/>
-    <row r="475" ht="15.75" customHeight="1"/>
-    <row r="476" ht="15.75" customHeight="1"/>
-    <row r="477" ht="15.75" customHeight="1"/>
-    <row r="478" ht="15.75" customHeight="1"/>
-    <row r="479" ht="15.75" customHeight="1"/>
-    <row r="480" ht="15.75" customHeight="1"/>
-    <row r="481" ht="15.75" customHeight="1"/>
-    <row r="482" ht="15.75" customHeight="1"/>
-    <row r="483" ht="15.75" customHeight="1"/>
-    <row r="484" ht="15.75" customHeight="1"/>
-    <row r="485" ht="15.75" customHeight="1"/>
-    <row r="486" ht="15.75" customHeight="1"/>
-    <row r="487" ht="15.75" customHeight="1"/>
-    <row r="488" ht="15.75" customHeight="1"/>
-    <row r="489" ht="15.75" customHeight="1"/>
-    <row r="490" ht="15.75" customHeight="1"/>
-    <row r="491" ht="15.75" customHeight="1"/>
-    <row r="492" ht="15.75" customHeight="1"/>
-    <row r="493" ht="15.75" customHeight="1"/>
-    <row r="494" ht="15.75" customHeight="1"/>
-    <row r="495" ht="15.75" customHeight="1"/>
-    <row r="496" ht="15.75" customHeight="1"/>
-    <row r="497" ht="15.75" customHeight="1"/>
-    <row r="498" ht="15.75" customHeight="1"/>
-    <row r="499" ht="15.75" customHeight="1"/>
-    <row r="500" ht="15.75" customHeight="1"/>
-    <row r="501" ht="15.75" customHeight="1"/>
-    <row r="502" ht="15.75" customHeight="1"/>
-    <row r="503" ht="15.75" customHeight="1"/>
-    <row r="504" ht="15.75" customHeight="1"/>
-    <row r="505" ht="15.75" customHeight="1"/>
-    <row r="506" ht="15.75" customHeight="1"/>
-    <row r="507" ht="15.75" customHeight="1"/>
-    <row r="508" ht="15.75" customHeight="1"/>
-    <row r="509" ht="15.75" customHeight="1"/>
-    <row r="510" ht="15.75" customHeight="1"/>
-    <row r="511" ht="15.75" customHeight="1"/>
-    <row r="512" ht="15.75" customHeight="1"/>
-    <row r="513" ht="15.75" customHeight="1"/>
-    <row r="514" ht="15.75" customHeight="1"/>
-    <row r="515" ht="15.75" customHeight="1"/>
-    <row r="516" ht="15.75" customHeight="1"/>
-    <row r="517" ht="15.75" customHeight="1"/>
-    <row r="518" ht="15.75" customHeight="1"/>
-    <row r="519" ht="15.75" customHeight="1"/>
-    <row r="520" ht="15.75" customHeight="1"/>
-    <row r="521" ht="15.75" customHeight="1"/>
-    <row r="522" ht="15.75" customHeight="1"/>
-    <row r="523" ht="15.75" customHeight="1"/>
-    <row r="524" ht="15.75" customHeight="1"/>
-    <row r="525" ht="15.75" customHeight="1"/>
-    <row r="526" ht="15.75" customHeight="1"/>
-    <row r="527" ht="15.75" customHeight="1"/>
-    <row r="528" ht="15.75" customHeight="1"/>
-    <row r="529" ht="15.75" customHeight="1"/>
-    <row r="530" ht="15.75" customHeight="1"/>
-    <row r="531" ht="15.75" customHeight="1"/>
-    <row r="532" ht="15.75" customHeight="1"/>
-    <row r="533" ht="15.75" customHeight="1"/>
-    <row r="534" ht="15.75" customHeight="1"/>
-    <row r="535" ht="15.75" customHeight="1"/>
-    <row r="536" ht="15.75" customHeight="1"/>
-    <row r="537" ht="15.75" customHeight="1"/>
-    <row r="538" ht="15.75" customHeight="1"/>
-    <row r="539" ht="15.75" customHeight="1"/>
-    <row r="540" ht="15.75" customHeight="1"/>
-    <row r="541" ht="15.75" customHeight="1"/>
-    <row r="542" ht="15.75" customHeight="1"/>
-    <row r="543" ht="15.75" customHeight="1"/>
-    <row r="544" ht="15.75" customHeight="1"/>
-    <row r="545" ht="15.75" customHeight="1"/>
-    <row r="546" ht="15.75" customHeight="1"/>
-    <row r="547" ht="15.75" customHeight="1"/>
-    <row r="548" ht="15.75" customHeight="1"/>
-    <row r="549" ht="15.75" customHeight="1"/>
-    <row r="550" ht="15.75" customHeight="1"/>
-    <row r="551" ht="15.75" customHeight="1"/>
-    <row r="552" ht="15.75" customHeight="1"/>
-    <row r="553" ht="15.75" customHeight="1"/>
-    <row r="554" ht="15.75" customHeight="1"/>
-    <row r="555" ht="15.75" customHeight="1"/>
-    <row r="556" ht="15.75" customHeight="1"/>
-    <row r="557" ht="15.75" customHeight="1"/>
-    <row r="558" ht="15.75" customHeight="1"/>
-    <row r="559" ht="15.75" customHeight="1"/>
-    <row r="560" ht="15.75" customHeight="1"/>
-    <row r="561" ht="15.75" customHeight="1"/>
-    <row r="562" ht="15.75" customHeight="1"/>
-    <row r="563" ht="15.75" customHeight="1"/>
-    <row r="564" ht="15.75" customHeight="1"/>
-    <row r="565" ht="15.75" customHeight="1"/>
-    <row r="566" ht="15.75" customHeight="1"/>
-    <row r="567" ht="15.75" customHeight="1"/>
-    <row r="568" ht="15.75" customHeight="1"/>
-    <row r="569" ht="15.75" customHeight="1"/>
-    <row r="570" ht="15.75" customHeight="1"/>
-    <row r="571" ht="15.75" customHeight="1"/>
-    <row r="572" ht="15.75" customHeight="1"/>
-    <row r="573" ht="15.75" customHeight="1"/>
-    <row r="574" ht="15.75" customHeight="1"/>
-    <row r="575" ht="15.75" customHeight="1"/>
-    <row r="576" ht="15.75" customHeight="1"/>
-    <row r="577" ht="15.75" customHeight="1"/>
-    <row r="578" ht="15.75" customHeight="1"/>
-    <row r="579" ht="15.75" customHeight="1"/>
-    <row r="580" ht="15.75" customHeight="1"/>
-    <row r="581" ht="15.75" customHeight="1"/>
-    <row r="582" ht="15.75" customHeight="1"/>
-    <row r="583" ht="15.75" customHeight="1"/>
-    <row r="584" ht="15.75" customHeight="1"/>
-    <row r="585" ht="15.75" customHeight="1"/>
-    <row r="586" ht="15.75" customHeight="1"/>
-    <row r="587" ht="15.75" customHeight="1"/>
-    <row r="588" ht="15.75" customHeight="1"/>
-    <row r="589" ht="15.75" customHeight="1"/>
-    <row r="590" ht="15.75" customHeight="1"/>
-    <row r="591" ht="15.75" customHeight="1"/>
-    <row r="592" ht="15.75" customHeight="1"/>
-    <row r="593" ht="15.75" customHeight="1"/>
-    <row r="594" ht="15.75" customHeight="1"/>
-    <row r="595" ht="15.75" customHeight="1"/>
-    <row r="596" ht="15.75" customHeight="1"/>
-    <row r="597" ht="15.75" customHeight="1"/>
-    <row r="598" ht="15.75" customHeight="1"/>
-    <row r="599" ht="15.75" customHeight="1"/>
-    <row r="600" ht="15.75" customHeight="1"/>
-    <row r="601" ht="15.75" customHeight="1"/>
-    <row r="602" ht="15.75" customHeight="1"/>
-    <row r="603" ht="15.75" customHeight="1"/>
-    <row r="604" ht="15.75" customHeight="1"/>
-    <row r="605" ht="15.75" customHeight="1"/>
-    <row r="606" ht="15.75" customHeight="1"/>
-    <row r="607" ht="15.75" customHeight="1"/>
-    <row r="608" ht="15.75" customHeight="1"/>
-    <row r="609" ht="15.75" customHeight="1"/>
-    <row r="610" ht="15.75" customHeight="1"/>
-    <row r="611" ht="15.75" customHeight="1"/>
-    <row r="612" ht="15.75" customHeight="1"/>
-    <row r="613" ht="15.75" customHeight="1"/>
-    <row r="614" ht="15.75" customHeight="1"/>
-    <row r="615" ht="15.75" customHeight="1"/>
-    <row r="616" ht="15.75" customHeight="1"/>
-    <row r="617" ht="15.75" customHeight="1"/>
-    <row r="618" ht="15.75" customHeight="1"/>
-    <row r="619" ht="15.75" customHeight="1"/>
-    <row r="620" ht="15.75" customHeight="1"/>
-    <row r="621" ht="15.75" customHeight="1"/>
-    <row r="622" ht="15.75" customHeight="1"/>
-    <row r="623" ht="15.75" customHeight="1"/>
-    <row r="624" ht="15.75" customHeight="1"/>
-    <row r="625" ht="15.75" customHeight="1"/>
-    <row r="626" ht="15.75" customHeight="1"/>
-    <row r="627" ht="15.75" customHeight="1"/>
-    <row r="628" ht="15.75" customHeight="1"/>
-    <row r="629" ht="15.75" customHeight="1"/>
-    <row r="630" ht="15.75" customHeight="1"/>
-    <row r="631" ht="15.75" customHeight="1"/>
-    <row r="632" ht="15.75" customHeight="1"/>
-    <row r="633" ht="15.75" customHeight="1"/>
-    <row r="634" ht="15.75" customHeight="1"/>
-    <row r="635" ht="15.75" customHeight="1"/>
-    <row r="636" ht="15.75" customHeight="1"/>
-    <row r="637" ht="15.75" customHeight="1"/>
-    <row r="638" ht="15.75" customHeight="1"/>
-    <row r="639" ht="15.75" customHeight="1"/>
-    <row r="640" ht="15.75" customHeight="1"/>
-    <row r="641" ht="15.75" customHeight="1"/>
-    <row r="642" ht="15.75" customHeight="1"/>
-    <row r="643" ht="15.75" customHeight="1"/>
-    <row r="644" ht="15.75" customHeight="1"/>
-    <row r="645" ht="15.75" customHeight="1"/>
-    <row r="646" ht="15.75" customHeight="1"/>
-    <row r="647" ht="15.75" customHeight="1"/>
-    <row r="648" ht="15.75" customHeight="1"/>
-    <row r="649" ht="15.75" customHeight="1"/>
-    <row r="650" ht="15.75" customHeight="1"/>
-    <row r="651" ht="15.75" customHeight="1"/>
-    <row r="652" ht="15.75" customHeight="1"/>
-    <row r="653" ht="15.75" customHeight="1"/>
-    <row r="654" ht="15.75" customHeight="1"/>
-    <row r="655" ht="15.75" customHeight="1"/>
-    <row r="656" ht="15.75" customHeight="1"/>
-    <row r="657" ht="15.75" customHeight="1"/>
-    <row r="658" ht="15.75" customHeight="1"/>
-    <row r="659" ht="15.75" customHeight="1"/>
-    <row r="660" ht="15.75" customHeight="1"/>
-    <row r="661" ht="15.75" customHeight="1"/>
-    <row r="662" ht="15.75" customHeight="1"/>
-    <row r="663" ht="15.75" customHeight="1"/>
-    <row r="664" ht="15.75" customHeight="1"/>
-    <row r="665" ht="15.75" customHeight="1"/>
-    <row r="666" ht="15.75" customHeight="1"/>
-    <row r="667" ht="15.75" customHeight="1"/>
-    <row r="668" ht="15.75" customHeight="1"/>
-    <row r="669" ht="15.75" customHeight="1"/>
-    <row r="670" ht="15.75" customHeight="1"/>
-    <row r="671" ht="15.75" customHeight="1"/>
-    <row r="672" ht="15.75" customHeight="1"/>
-    <row r="673" ht="15.75" customHeight="1"/>
-    <row r="674" ht="15.75" customHeight="1"/>
-    <row r="675" ht="15.75" customHeight="1"/>
-    <row r="676" ht="15.75" customHeight="1"/>
-    <row r="677" ht="15.75" customHeight="1"/>
-    <row r="678" ht="15.75" customHeight="1"/>
-    <row r="679" ht="15.75" customHeight="1"/>
-    <row r="680" ht="15.75" customHeight="1"/>
-    <row r="681" ht="15.75" customHeight="1"/>
-    <row r="682" ht="15.75" customHeight="1"/>
-    <row r="683" ht="15.75" customHeight="1"/>
-    <row r="684" ht="15.75" customHeight="1"/>
-    <row r="685" ht="15.75" customHeight="1"/>
-    <row r="686" ht="15.75" customHeight="1"/>
-    <row r="687" ht="15.75" customHeight="1"/>
-    <row r="688" ht="15.75" customHeight="1"/>
-    <row r="689" ht="15.75" customHeight="1"/>
-    <row r="690" ht="15.75" customHeight="1"/>
-    <row r="691" ht="15.75" customHeight="1"/>
-    <row r="692" ht="15.75" customHeight="1"/>
-    <row r="693" ht="15.75" customHeight="1"/>
-    <row r="694" ht="15.75" customHeight="1"/>
-    <row r="695" ht="15.75" customHeight="1"/>
-    <row r="696" ht="15.75" customHeight="1"/>
-    <row r="697" ht="15.75" customHeight="1"/>
-    <row r="698" ht="15.75" customHeight="1"/>
-    <row r="699" ht="15.75" customHeight="1"/>
-    <row r="700" ht="15.75" customHeight="1"/>
-    <row r="701" ht="15.75" customHeight="1"/>
-    <row r="702" ht="15.75" customHeight="1"/>
-    <row r="703" ht="15.75" customHeight="1"/>
-    <row r="704" ht="15.75" customHeight="1"/>
-    <row r="705" ht="15.75" customHeight="1"/>
-    <row r="706" ht="15.75" customHeight="1"/>
-    <row r="707" ht="15.75" customHeight="1"/>
-    <row r="708" ht="15.75" customHeight="1"/>
-    <row r="709" ht="15.75" customHeight="1"/>
-    <row r="710" ht="15.75" customHeight="1"/>
-    <row r="711" ht="15.75" customHeight="1"/>
-    <row r="712" ht="15.75" customHeight="1"/>
-    <row r="713" ht="15.75" customHeight="1"/>
-    <row r="714" ht="15.75" customHeight="1"/>
-    <row r="715" ht="15.75" customHeight="1"/>
-    <row r="716" ht="15.75" customHeight="1"/>
-    <row r="717" ht="15.75" customHeight="1"/>
-    <row r="718" ht="15.75" customHeight="1"/>
-    <row r="719" ht="15.75" customHeight="1"/>
-    <row r="720" ht="15.75" customHeight="1"/>
-    <row r="721" ht="15.75" customHeight="1"/>
-    <row r="722" ht="15.75" customHeight="1"/>
-    <row r="723" ht="15.75" customHeight="1"/>
-    <row r="724" ht="15.75" customHeight="1"/>
-    <row r="725" ht="15.75" customHeight="1"/>
-    <row r="726" ht="15.75" customHeight="1"/>
-    <row r="727" ht="15.75" customHeight="1"/>
-    <row r="728" ht="15.75" customHeight="1"/>
-    <row r="729" ht="15.75" customHeight="1"/>
-    <row r="730" ht="15.75" customHeight="1"/>
-    <row r="731" ht="15.75" customHeight="1"/>
-    <row r="732" ht="15.75" customHeight="1"/>
-    <row r="733" ht="15.75" customHeight="1"/>
-    <row r="734" ht="15.75" customHeight="1"/>
-    <row r="735" ht="15.75" customHeight="1"/>
-    <row r="736" ht="15.75" customHeight="1"/>
-    <row r="737" ht="15.75" customHeight="1"/>
-    <row r="738" ht="15.75" customHeight="1"/>
-    <row r="739" ht="15.75" customHeight="1"/>
-    <row r="740" ht="15.75" customHeight="1"/>
-    <row r="741" ht="15.75" customHeight="1"/>
-    <row r="742" ht="15.75" customHeight="1"/>
-    <row r="743" ht="15.75" customHeight="1"/>
-    <row r="744" ht="15.75" customHeight="1"/>
-    <row r="745" ht="15.75" customHeight="1"/>
-    <row r="746" ht="15.75" customHeight="1"/>
-    <row r="747" ht="15.75" customHeight="1"/>
-    <row r="748" ht="15.75" customHeight="1"/>
-    <row r="749" ht="15.75" customHeight="1"/>
-    <row r="750" ht="15.75" customHeight="1"/>
-    <row r="751" ht="15.75" customHeight="1"/>
-    <row r="752" ht="15.75" customHeight="1"/>
-    <row r="753" ht="15.75" customHeight="1"/>
-    <row r="754" ht="15.75" customHeight="1"/>
-    <row r="755" ht="15.75" customHeight="1"/>
-    <row r="756" ht="15.75" customHeight="1"/>
-    <row r="757" ht="15.75" customHeight="1"/>
-    <row r="758" ht="15.75" customHeight="1"/>
-    <row r="759" ht="15.75" customHeight="1"/>
-    <row r="760" ht="15.75" customHeight="1"/>
-    <row r="761" ht="15.75" customHeight="1"/>
-    <row r="762" ht="15.75" customHeight="1"/>
-    <row r="763" ht="15.75" customHeight="1"/>
-    <row r="764" ht="15.75" customHeight="1"/>
-    <row r="765" ht="15.75" customHeight="1"/>
-    <row r="766" ht="15.75" customHeight="1"/>
-    <row r="767" ht="15.75" customHeight="1"/>
-    <row r="768" ht="15.75" customHeight="1"/>
-    <row r="769" ht="15.75" customHeight="1"/>
-    <row r="770" ht="15.75" customHeight="1"/>
-    <row r="771" ht="15.75" customHeight="1"/>
-    <row r="772" ht="15.75" customHeight="1"/>
-    <row r="773" ht="15.75" customHeight="1"/>
-    <row r="774" ht="15.75" customHeight="1"/>
-    <row r="775" ht="15.75" customHeight="1"/>
-    <row r="776" ht="15.75" customHeight="1"/>
-    <row r="777" ht="15.75" customHeight="1"/>
-    <row r="778" ht="15.75" customHeight="1"/>
-    <row r="779" ht="15.75" customHeight="1"/>
-    <row r="780" ht="15.75" customHeight="1"/>
-    <row r="781" ht="15.75" customHeight="1"/>
-    <row r="782" ht="15.75" customHeight="1"/>
-    <row r="783" ht="15.75" customHeight="1"/>
-    <row r="784" ht="15.75" customHeight="1"/>
-    <row r="785" ht="15.75" customHeight="1"/>
-    <row r="786" ht="15.75" customHeight="1"/>
-    <row r="787" ht="15.75" customHeight="1"/>
-    <row r="788" ht="15.75" customHeight="1"/>
-    <row r="789" ht="15.75" customHeight="1"/>
-    <row r="790" ht="15.75" customHeight="1"/>
-    <row r="791" ht="15.75" customHeight="1"/>
-    <row r="792" ht="15.75" customHeight="1"/>
-    <row r="793" ht="15.75" customHeight="1"/>
-    <row r="794" ht="15.75" customHeight="1"/>
-    <row r="795" ht="15.75" customHeight="1"/>
-    <row r="796" ht="15.75" customHeight="1"/>
-    <row r="797" ht="15.75" customHeight="1"/>
-    <row r="798" ht="15.75" customHeight="1"/>
-    <row r="799" ht="15.75" customHeight="1"/>
-    <row r="800" ht="15.75" customHeight="1"/>
-    <row r="801" ht="15.75" customHeight="1"/>
-    <row r="802" ht="15.75" customHeight="1"/>
-    <row r="803" ht="15.75" customHeight="1"/>
-    <row r="804" ht="15.75" customHeight="1"/>
-    <row r="805" ht="15.75" customHeight="1"/>
-    <row r="806" ht="15.75" customHeight="1"/>
-    <row r="807" ht="15.75" customHeight="1"/>
-    <row r="808" ht="15.75" customHeight="1"/>
-    <row r="809" ht="15.75" customHeight="1"/>
-    <row r="810" ht="15.75" customHeight="1"/>
-    <row r="811" ht="15.75" customHeight="1"/>
-    <row r="812" ht="15.75" customHeight="1"/>
-    <row r="813" ht="15.75" customHeight="1"/>
-    <row r="814" ht="15.75" customHeight="1"/>
-    <row r="815" ht="15.75" customHeight="1"/>
-    <row r="816" ht="15.75" customHeight="1"/>
-    <row r="817" ht="15.75" customHeight="1"/>
-    <row r="818" ht="15.75" customHeight="1"/>
-    <row r="819" ht="15.75" customHeight="1"/>
-    <row r="820" ht="15.75" customHeight="1"/>
-    <row r="821" ht="15.75" customHeight="1"/>
-    <row r="822" ht="15.75" customHeight="1"/>
-    <row r="823" ht="15.75" customHeight="1"/>
-    <row r="824" ht="15.75" customHeight="1"/>
-    <row r="825" ht="15.75" customHeight="1"/>
-    <row r="826" ht="15.75" customHeight="1"/>
-    <row r="827" ht="15.75" customHeight="1"/>
-    <row r="828" ht="15.75" customHeight="1"/>
-    <row r="829" ht="15.75" customHeight="1"/>
-    <row r="830" ht="15.75" customHeight="1"/>
-    <row r="831" ht="15.75" customHeight="1"/>
-    <row r="832" ht="15.75" customHeight="1"/>
-    <row r="833" ht="15.75" customHeight="1"/>
-    <row r="834" ht="15.75" customHeight="1"/>
-    <row r="835" ht="15.75" customHeight="1"/>
-    <row r="836" ht="15.75" customHeight="1"/>
-    <row r="837" ht="15.75" customHeight="1"/>
-    <row r="838" ht="15.75" customHeight="1"/>
-    <row r="839" ht="15.75" customHeight="1"/>
-    <row r="840" ht="15.75" customHeight="1"/>
-    <row r="841" ht="15.75" customHeight="1"/>
-    <row r="842" ht="15.75" customHeight="1"/>
-    <row r="843" ht="15.75" customHeight="1"/>
-    <row r="844" ht="15.75" customHeight="1"/>
-    <row r="845" ht="15.75" customHeight="1"/>
-    <row r="846" ht="15.75" customHeight="1"/>
-    <row r="847" ht="15.75" customHeight="1"/>
-    <row r="848" ht="15.75" customHeight="1"/>
-    <row r="849" ht="15.75" customHeight="1"/>
-    <row r="850" ht="15.75" customHeight="1"/>
-    <row r="851" ht="15.75" customHeight="1"/>
-    <row r="852" ht="15.75" customHeight="1"/>
-    <row r="853" ht="15.75" customHeight="1"/>
-    <row r="854" ht="15.75" customHeight="1"/>
-    <row r="855" ht="15.75" customHeight="1"/>
-    <row r="856" ht="15.75" customHeight="1"/>
-    <row r="857" ht="15.75" customHeight="1"/>
-    <row r="858" ht="15.75" customHeight="1"/>
-    <row r="859" ht="15.75" customHeight="1"/>
-    <row r="860" ht="15.75" customHeight="1"/>
-    <row r="861" ht="15.75" customHeight="1"/>
-    <row r="862" ht="15.75" customHeight="1"/>
-    <row r="863" ht="15.75" customHeight="1"/>
-    <row r="864" ht="15.75" customHeight="1"/>
-    <row r="865" ht="15.75" customHeight="1"/>
-    <row r="866" ht="15.75" customHeight="1"/>
-    <row r="867" ht="15.75" customHeight="1"/>
-    <row r="868" ht="15.75" customHeight="1"/>
-    <row r="869" ht="15.75" customHeight="1"/>
-    <row r="870" ht="15.75" customHeight="1"/>
-    <row r="871" ht="15.75" customHeight="1"/>
-    <row r="872" ht="15.75" customHeight="1"/>
-    <row r="873" ht="15.75" customHeight="1"/>
-    <row r="874" ht="15.75" customHeight="1"/>
-    <row r="875" ht="15.75" customHeight="1"/>
-    <row r="876" ht="15.75" customHeight="1"/>
-    <row r="877" ht="15.75" customHeight="1"/>
-    <row r="878" ht="15.75" customHeight="1"/>
-    <row r="879" ht="15.75" customHeight="1"/>
-    <row r="880" ht="15.75" customHeight="1"/>
-    <row r="881" ht="15.75" customHeight="1"/>
-    <row r="882" ht="15.75" customHeight="1"/>
-    <row r="883" ht="15.75" customHeight="1"/>
-    <row r="884" ht="15.75" customHeight="1"/>
-    <row r="885" ht="15.75" customHeight="1"/>
-    <row r="886" ht="15.75" customHeight="1"/>
-    <row r="887" ht="15.75" customHeight="1"/>
-    <row r="888" ht="15.75" customHeight="1"/>
-    <row r="889" ht="15.75" customHeight="1"/>
-    <row r="890" ht="15.75" customHeight="1"/>
-    <row r="891" ht="15.75" customHeight="1"/>
-    <row r="892" ht="15.75" customHeight="1"/>
-    <row r="893" ht="15.75" customHeight="1"/>
-    <row r="894" ht="15.75" customHeight="1"/>
-    <row r="895" ht="15.75" customHeight="1"/>
-    <row r="896" ht="15.75" customHeight="1"/>
-    <row r="897" ht="15.75" customHeight="1"/>
-    <row r="898" ht="15.75" customHeight="1"/>
-    <row r="899" ht="15.75" customHeight="1"/>
-    <row r="900" ht="15.75" customHeight="1"/>
-    <row r="901" ht="15.75" customHeight="1"/>
-    <row r="902" ht="15.75" customHeight="1"/>
-    <row r="903" ht="15.75" customHeight="1"/>
-    <row r="904" ht="15.75" customHeight="1"/>
-    <row r="905" ht="15.75" customHeight="1"/>
-    <row r="906" ht="15.75" customHeight="1"/>
-    <row r="907" ht="15.75" customHeight="1"/>
-    <row r="908" ht="15.75" customHeight="1"/>
-    <row r="909" ht="15.75" customHeight="1"/>
-    <row r="910" ht="15.75" customHeight="1"/>
-    <row r="911" ht="15.75" customHeight="1"/>
-    <row r="912" ht="15.75" customHeight="1"/>
-    <row r="913" ht="15.75" customHeight="1"/>
-    <row r="914" ht="15.75" customHeight="1"/>
-    <row r="915" ht="15.75" customHeight="1"/>
-    <row r="916" ht="15.75" customHeight="1"/>
-    <row r="917" ht="15.75" customHeight="1"/>
-    <row r="918" ht="15.75" customHeight="1"/>
-    <row r="919" ht="15.75" customHeight="1"/>
-    <row r="920" ht="15.75" customHeight="1"/>
-    <row r="921" ht="15.75" customHeight="1"/>
-    <row r="922" ht="15.75" customHeight="1"/>
-    <row r="923" ht="15.75" customHeight="1"/>
-    <row r="924" ht="15.75" customHeight="1"/>
-    <row r="925" ht="15.75" customHeight="1"/>
-    <row r="926" ht="15.75" customHeight="1"/>
-    <row r="927" ht="15.75" customHeight="1"/>
-    <row r="928" ht="15.75" customHeight="1"/>
-    <row r="929" ht="15.75" customHeight="1"/>
-    <row r="930" ht="15.75" customHeight="1"/>
-    <row r="931" ht="15.75" customHeight="1"/>
-    <row r="932" ht="15.75" customHeight="1"/>
-    <row r="933" ht="15.75" customHeight="1"/>
-    <row r="934" ht="15.75" customHeight="1"/>
-    <row r="935" ht="15.75" customHeight="1"/>
-    <row r="936" ht="15.75" customHeight="1"/>
-    <row r="937" ht="15.75" customHeight="1"/>
-    <row r="938" ht="15.75" customHeight="1"/>
-    <row r="939" ht="15.75" customHeight="1"/>
-    <row r="940" ht="15.75" customHeight="1"/>
-    <row r="941" ht="15.75" customHeight="1"/>
-    <row r="942" ht="15.75" customHeight="1"/>
-    <row r="943" ht="15.75" customHeight="1"/>
-    <row r="944" ht="15.75" customHeight="1"/>
-    <row r="945" ht="15.75" customHeight="1"/>
-    <row r="946" ht="15.75" customHeight="1"/>
-    <row r="947" ht="15.75" customHeight="1"/>
-    <row r="948" ht="15.75" customHeight="1"/>
-    <row r="949" ht="15.75" customHeight="1"/>
-    <row r="950" ht="15.75" customHeight="1"/>
-    <row r="951" ht="15.75" customHeight="1"/>
-    <row r="952" ht="15.75" customHeight="1"/>
-    <row r="953" ht="15.75" customHeight="1"/>
-    <row r="954" ht="15.75" customHeight="1"/>
-    <row r="955" ht="15.75" customHeight="1"/>
-    <row r="956" ht="15.75" customHeight="1"/>
-    <row r="957" ht="15.75" customHeight="1"/>
-    <row r="958" ht="15.75" customHeight="1"/>
-    <row r="959" ht="15.75" customHeight="1"/>
-    <row r="960" ht="15.75" customHeight="1"/>
-    <row r="961" ht="15.75" customHeight="1"/>
-    <row r="962" ht="15.75" customHeight="1"/>
-    <row r="963" ht="15.75" customHeight="1"/>
-    <row r="964" ht="15.75" customHeight="1"/>
-    <row r="965" ht="15.75" customHeight="1"/>
-    <row r="966" ht="15.75" customHeight="1"/>
-    <row r="967" ht="15.75" customHeight="1"/>
-    <row r="968" ht="15.75" customHeight="1"/>
-    <row r="969" ht="15.75" customHeight="1"/>
-    <row r="970" ht="15.75" customHeight="1"/>
-    <row r="971" ht="15.75" customHeight="1"/>
-    <row r="972" ht="15.75" customHeight="1"/>
-    <row r="973" ht="15.75" customHeight="1"/>
-    <row r="974" ht="15.75" customHeight="1"/>
-    <row r="975" ht="15.75" customHeight="1"/>
-    <row r="976" ht="15.75" customHeight="1"/>
-    <row r="977" ht="15.75" customHeight="1"/>
-    <row r="978" ht="15.75" customHeight="1"/>
-    <row r="979" ht="15.75" customHeight="1"/>
-    <row r="980" ht="15.75" customHeight="1"/>
-    <row r="981" ht="15.75" customHeight="1"/>
-    <row r="982" ht="15.75" customHeight="1"/>
-    <row r="983" ht="15.75" customHeight="1"/>
-    <row r="984" ht="15.75" customHeight="1"/>
-    <row r="985" ht="15.75" customHeight="1"/>
-    <row r="986" ht="15.75" customHeight="1"/>
-    <row r="987" ht="15.75" customHeight="1"/>
-    <row r="988" ht="15.75" customHeight="1"/>
-    <row r="989" ht="15.75" customHeight="1"/>
-    <row r="990" ht="15.75" customHeight="1"/>
-    <row r="991" ht="15.75" customHeight="1"/>
-    <row r="992" ht="15.75" customHeight="1"/>
-    <row r="993" ht="15.75" customHeight="1"/>
-    <row r="994" ht="15.75" customHeight="1"/>
-    <row r="995" ht="15.75" customHeight="1"/>
-    <row r="996" ht="15.75" customHeight="1"/>
-    <row r="997" ht="15.75" customHeight="1"/>
-    <row r="998" ht="15.75" customHeight="1"/>
-    <row r="999" ht="15.75" customHeight="1"/>
-    <row r="1000" ht="15.75" customHeight="1"/>
-    <row r="1001" ht="15.75" customHeight="1"/>
+    <row r="54" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="55" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="56" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="57" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="58" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="59" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="60" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="61" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="62" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="63" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="64" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="65" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="66" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="67" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="68" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="69" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="70" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="71" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="72" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="73" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="74" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="75" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="76" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="77" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="78" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="79" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="80" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="81" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="82" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="83" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="84" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="85" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="86" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="87" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="88" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="89" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="90" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="91" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="92" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="93" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="94" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="95" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="96" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="97" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="98" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="99" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="100" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="101" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="102" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="103" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="104" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="105" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="106" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="107" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="108" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="109" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="110" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="111" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="112" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="113" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="114" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="115" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="116" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="117" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="118" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="119" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="120" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="121" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="122" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="123" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="124" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="125" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="126" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="127" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="128" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="129" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="130" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="131" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="132" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="133" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="134" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="135" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="136" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="137" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="138" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="139" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="140" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="141" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="142" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="143" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="144" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="145" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="146" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="147" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="148" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="149" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="150" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="151" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="152" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="153" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="154" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="155" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="156" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="157" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="158" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="159" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="160" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="161" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="162" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="163" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="164" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="165" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="166" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="167" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="168" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="169" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="170" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="171" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="172" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="173" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="174" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="175" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="176" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="177" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="178" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="179" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="180" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="181" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="182" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="183" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="184" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="185" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="186" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="187" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="188" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="189" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="190" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="191" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="192" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="193" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="194" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="195" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="196" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="197" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="198" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="199" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="200" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="201" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="202" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="203" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="204" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="205" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="206" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="207" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="208" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="209" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="210" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="211" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="212" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="213" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="214" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="215" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="216" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="217" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="218" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="219" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="220" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="221" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="222" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="223" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="224" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="225" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="226" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="227" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="228" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="229" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="230" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="231" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="232" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="233" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="234" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="235" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="236" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="237" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="238" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="239" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="240" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="241" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="242" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="243" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="244" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="245" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="246" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="247" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="248" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="249" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="250" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="251" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="252" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="253" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="254" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="255" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="256" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="257" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="258" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="259" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="260" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="261" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="262" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="263" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="264" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="265" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="266" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="267" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="268" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="269" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="270" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="271" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="272" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="273" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="274" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="275" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="276" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="277" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="278" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="279" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="280" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="281" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="282" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="283" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="284" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="285" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="286" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="287" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="288" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="289" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="290" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="291" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="292" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="293" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="294" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="295" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="296" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="297" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="298" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="299" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="300" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="301" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="302" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="303" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="304" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="305" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="306" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="307" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="308" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="309" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="310" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="311" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="312" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="313" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="314" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="315" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="316" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="317" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="318" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="319" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="320" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="321" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="322" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="323" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="324" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="325" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="326" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="327" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="328" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="329" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="330" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="331" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="332" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="333" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="334" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="335" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="336" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="337" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="338" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="339" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="340" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="341" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="342" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="343" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="344" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="345" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="346" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="347" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="348" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="349" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="350" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="351" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="352" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="353" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="354" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="355" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="356" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="357" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="358" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="359" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="360" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="361" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="362" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="363" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="364" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="365" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="366" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="367" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="368" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="369" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="370" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="371" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="372" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="373" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="374" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="375" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="376" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="377" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="378" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="379" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="380" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="381" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="382" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="383" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="384" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="385" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="386" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="387" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="388" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="389" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="390" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="391" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="392" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="393" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="394" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="395" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="396" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="397" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="398" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="399" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="400" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="401" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="402" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="403" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="404" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="405" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="406" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="407" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="408" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="409" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="410" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="411" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="412" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="413" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="414" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="415" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="416" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="417" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="418" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="419" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="420" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="421" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="422" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="423" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="424" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="425" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="426" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="427" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="428" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="429" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="430" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="431" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="432" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="433" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="434" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="435" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="436" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="437" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="438" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="439" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="440" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="441" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="442" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="443" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="444" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="445" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="446" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="447" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="448" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="449" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="450" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="451" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="452" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="453" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="454" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="455" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="456" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="457" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="458" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="459" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="460" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="461" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="462" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="463" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="464" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="465" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="466" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="467" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="468" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="469" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="470" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="471" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="472" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="473" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="474" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="475" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="476" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="477" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="478" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="479" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="480" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="481" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="482" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="483" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="484" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="485" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="486" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="487" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="488" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="489" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="490" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="491" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="492" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="493" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="494" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="495" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="496" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="497" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="498" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="499" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="500" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="501" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="502" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="503" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="504" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="505" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="506" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="507" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="508" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="509" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="510" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="511" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="512" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="513" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="514" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="515" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="516" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="517" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="518" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="519" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="520" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="521" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="522" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="523" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="524" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="525" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="526" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="527" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="528" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="529" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="530" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="531" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="532" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="533" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="534" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="535" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="536" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="537" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="538" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="539" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="540" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="541" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="542" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="543" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="544" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="545" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="546" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="547" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="548" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="549" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="550" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="551" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="552" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="553" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="554" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="555" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="556" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="557" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="558" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="559" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="560" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="561" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="562" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="563" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="564" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="565" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="566" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="567" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="568" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="569" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="570" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="571" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="572" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="573" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="574" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="575" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="576" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="577" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="578" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="579" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="580" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="581" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="582" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="583" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="584" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="585" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="586" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="587" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="588" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="589" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="590" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="591" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="592" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="593" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="594" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="595" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="596" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="597" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="598" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="599" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="600" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="601" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="602" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="603" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="604" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="605" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="606" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="607" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="608" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="609" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="610" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="611" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="612" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="613" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="614" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="615" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="616" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="617" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="618" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="619" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="620" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="621" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="622" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="623" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="624" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="625" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="626" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="627" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="628" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="629" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="630" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="631" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="632" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="633" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="634" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="635" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="636" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="637" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="638" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="639" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="640" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="641" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="642" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="643" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="644" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="645" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="646" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="647" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="648" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="649" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="650" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="651" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="652" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="653" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="654" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="655" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="656" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="657" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="658" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="659" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="660" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="661" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="662" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="663" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="664" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="665" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="666" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="667" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="668" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="669" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="670" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="671" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="672" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="673" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="674" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="675" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="676" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="677" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="678" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="679" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="680" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="681" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="682" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="683" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="684" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="685" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="686" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="687" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="688" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="689" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="690" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="691" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="692" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="693" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="694" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="695" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="696" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="697" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="698" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="699" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="700" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="701" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="702" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="703" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="704" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="705" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="706" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="707" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="708" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="709" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="710" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="711" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="712" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="713" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="714" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="715" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="716" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="717" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="718" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="719" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="720" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="721" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="722" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="723" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="724" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="725" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="726" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="727" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="728" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="729" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="730" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="731" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="732" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="733" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="734" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="735" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="736" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="737" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="738" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="739" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="740" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="741" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="742" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="743" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="744" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="745" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="746" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="747" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="748" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="749" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="750" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="751" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="752" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="753" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="754" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="755" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="756" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="757" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="758" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="759" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="760" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="761" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="762" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="763" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="764" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="765" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="766" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="767" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="768" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="769" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="770" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="771" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="772" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="773" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="774" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="775" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="776" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="777" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="778" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="779" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="780" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="781" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="782" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="783" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="784" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="785" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="786" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="787" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="788" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="789" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="790" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="791" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="792" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="793" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="794" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="795" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="796" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="797" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="798" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="799" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="800" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="801" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="802" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="803" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="804" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="805" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="806" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="807" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="808" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="809" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="810" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="811" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="812" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="813" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="814" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="815" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="816" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="817" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="818" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="819" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="820" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="821" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="822" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="823" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="824" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="825" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="826" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="827" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="828" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="829" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="830" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="831" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="832" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="833" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="834" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="835" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="836" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="837" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="838" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="839" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="840" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="841" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="842" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="843" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="844" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="845" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="846" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="847" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="848" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="849" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="850" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="851" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="852" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="853" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="854" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="855" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="856" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="857" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="858" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="859" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="860" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="861" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="862" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="863" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="864" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="865" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="866" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="867" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="868" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="869" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="870" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="871" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="872" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="873" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="874" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="875" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="876" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="877" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="878" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="879" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="880" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="881" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="882" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="883" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="884" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="885" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="886" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="887" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="888" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="889" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="890" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="891" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="892" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="893" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="894" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="895" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="896" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="897" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="898" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="899" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="900" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="901" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="902" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="903" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="904" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="905" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="906" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="907" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="908" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="909" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="910" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="911" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="912" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="913" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="914" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="915" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="916" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="917" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="918" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="919" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="920" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="921" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="922" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="923" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="924" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="925" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="926" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="927" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="928" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="929" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="930" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="931" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="932" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="933" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="934" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="935" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="936" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="937" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="938" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="939" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="940" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="941" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="942" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="943" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="944" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="945" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="946" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="947" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="948" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="949" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="950" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="951" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="952" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="953" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="954" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="955" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="956" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="957" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="958" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="959" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="960" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="961" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="962" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="963" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="964" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="965" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="966" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="967" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="968" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="969" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="970" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="971" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="972" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="973" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="974" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="975" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="976" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="977" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="978" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="979" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="980" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="981" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="982" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="983" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="984" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="985" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="986" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="987" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="988" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="989" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="990" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="991" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="992" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="993" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="994" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="995" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="996" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="997" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="998" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="999" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="1001" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
-  <pageMargins left="0.5118055" right="0.5118055" top="0.7875" bottom="0.7875" header="0" footer="0"/>
+  <pageMargins left="0.51180550000000002" right="0.51180550000000002" top="0.78749999999999998" bottom="0.78749999999999998" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Correção do erro de atualização infinita e realização de ajustes no sistema de pontuação dos heróis.
</commit_message>
<xml_diff>
--- a/dist/OWPick/_internal/heroes ally.xlsx
+++ b/dist/OWPick/_internal/heroes ally.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DAVI\Projeto\Overwatch-Best-Picks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{841A1235-B230-4D4D-A883-06E895A471B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF91B967-6564-4AEF-86CA-349691FEBF1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -94,6 +94,9 @@
     <t>Lifeweaver</t>
   </si>
   <si>
+    <t>Lúcio</t>
+  </si>
+  <si>
     <t>Mauga</t>
   </si>
   <si>
@@ -174,9 +177,6 @@
   <si>
     <t>Zenyatta</t>
   </si>
-  <si>
-    <t>Lúcio</t>
-  </si>
 </sst>
 </file>
 
@@ -255,8 +255,17 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
-  <tableStyles count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF0000"/>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -552,88 +561,88 @@
         <v>23</v>
       </c>
       <c r="Y1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Z1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="AA1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="AB1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="AC1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="AD1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="AE1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="AF1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="AG1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="AH1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="AI1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="AJ1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="AK1" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AL1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AM1" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="AN1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="AO1" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="AP1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="AQ1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="AR1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="AS1" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="AT1" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="AU1" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="AV1" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="AW1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="AX1" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="AY1" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="AZ1" s="1" t="s">
         <v>51</v>
-      </c>
-      <c r="Z1" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="AA1" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="AB1" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="AC1" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="AD1" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="AE1" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="AF1" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="AG1" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="AH1" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="AI1" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="AJ1" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="AK1" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="AL1" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="AM1" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="AN1" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="AO1" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="AP1" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="AQ1" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="AR1" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="AS1" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="AT1" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="AU1" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="AV1" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="AW1" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="AX1" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="AY1" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="AZ1" s="1" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="2" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -2224,154 +2233,154 @@
         <v>1</v>
       </c>
       <c r="C12" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D12" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E12" s="3">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="F12" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="G12" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H12" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="I12" s="3">
         <v>2</v>
       </c>
       <c r="J12" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K12" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L12" s="3">
         <v>-11</v>
       </c>
       <c r="M12" s="3">
-        <v>-1</v>
+        <v>2</v>
       </c>
       <c r="N12" s="3">
         <v>1</v>
       </c>
       <c r="O12" s="3">
-        <v>1</v>
+        <v>-2</v>
       </c>
       <c r="P12" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="Q12" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R12" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S12" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T12" s="3">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="U12" s="3">
-        <v>1</v>
+        <v>-2</v>
       </c>
       <c r="V12" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="W12" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="X12" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="Y12" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="Z12" s="3">
         <v>1</v>
       </c>
       <c r="AA12" s="3">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="AB12" s="3">
         <v>2</v>
       </c>
       <c r="AC12" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AD12" s="3">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="AE12" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AF12" s="3">
-        <v>1</v>
+        <v>-2</v>
       </c>
       <c r="AG12" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH12" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AI12" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AJ12" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AK12" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AL12" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AM12" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AN12" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AO12" s="3">
-        <v>1</v>
+        <v>-2</v>
       </c>
       <c r="AP12" s="3">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="AQ12" s="3">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="AR12" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS12" s="3">
-        <v>1</v>
+        <v>-2</v>
       </c>
       <c r="AT12" s="3">
-        <v>1</v>
+        <v>-2</v>
       </c>
       <c r="AU12" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AV12" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW12" s="3">
         <v>1</v>
       </c>
       <c r="AX12" s="3">
-        <v>2</v>
+        <v>-1</v>
       </c>
       <c r="AY12" s="3">
         <v>1</v>
       </c>
       <c r="AZ12" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4272,7 +4281,7 @@
     </row>
     <row r="25" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>51</v>
+        <v>24</v>
       </c>
       <c r="B25" s="3">
         <v>-1</v>
@@ -4430,7 +4439,7 @@
     </row>
     <row r="26" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B26" s="3">
         <v>-1</v>
@@ -4588,7 +4597,7 @@
     </row>
     <row r="27" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B27" s="3">
         <v>1</v>
@@ -4746,7 +4755,7 @@
     </row>
     <row r="28" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B28" s="3">
         <v>0</v>
@@ -4904,7 +4913,7 @@
     </row>
     <row r="29" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B29" s="3">
         <v>2</v>
@@ -5062,7 +5071,7 @@
     </row>
     <row r="30" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B30" s="3">
         <v>-1</v>
@@ -5220,7 +5229,7 @@
     </row>
     <row r="31" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B31" s="3">
         <v>1</v>
@@ -5378,7 +5387,7 @@
     </row>
     <row r="32" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B32" s="3">
         <v>-2</v>
@@ -5536,7 +5545,7 @@
     </row>
     <row r="33" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B33" s="3">
         <v>-1</v>
@@ -5694,7 +5703,7 @@
     </row>
     <row r="34" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B34" s="3">
         <v>-1</v>
@@ -5852,7 +5861,7 @@
     </row>
     <row r="35" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B35" s="3">
         <v>1</v>
@@ -6010,7 +6019,7 @@
     </row>
     <row r="36" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B36" s="3">
         <v>1</v>
@@ -6168,7 +6177,7 @@
     </row>
     <row r="37" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B37" s="3">
         <v>0</v>
@@ -6326,7 +6335,7 @@
     </row>
     <row r="38" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B38" s="3">
         <v>1</v>
@@ -6484,7 +6493,7 @@
     </row>
     <row r="39" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B39" s="3">
         <v>1</v>
@@ -6642,7 +6651,7 @@
     </row>
     <row r="40" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B40" s="3">
         <v>1</v>
@@ -6800,16 +6809,16 @@
     </row>
     <row r="41" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B41" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="C41" s="3">
-        <v>1</v>
+        <v>-2</v>
       </c>
       <c r="D41" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E41" s="3">
         <v>1</v>
@@ -6818,70 +6827,70 @@
         <v>0</v>
       </c>
       <c r="G41" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H41" s="3">
         <v>1</v>
       </c>
       <c r="I41" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J41" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K41" s="3">
         <v>1</v>
       </c>
       <c r="L41" s="3">
-        <v>1</v>
+        <v>-2</v>
       </c>
       <c r="M41" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N41" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="O41" s="3">
-        <v>2</v>
+        <v>-2</v>
       </c>
       <c r="P41" s="3">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="Q41" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R41" s="3">
-        <v>1</v>
+        <v>-2</v>
       </c>
       <c r="S41" s="3">
         <v>0</v>
       </c>
       <c r="T41" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U41" s="3">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="V41" s="3">
         <v>0</v>
       </c>
       <c r="W41" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X41" s="3">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="Y41" s="3">
-        <v>-1</v>
+        <v>2</v>
       </c>
       <c r="Z41" s="3">
         <v>2</v>
       </c>
       <c r="AA41" s="3">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AB41" s="3">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="AC41" s="3">
         <v>0</v>
@@ -6893,28 +6902,28 @@
         <v>-1</v>
       </c>
       <c r="AF41" s="3">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AG41" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AH41" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI41" s="3">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="AJ41" s="3">
-        <v>-2</v>
+        <v>1</v>
       </c>
       <c r="AK41" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AL41" s="3">
-        <v>-2</v>
+        <v>1</v>
       </c>
       <c r="AM41" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AN41" s="3">
         <v>-1</v>
@@ -6923,34 +6932,34 @@
         <v>-11</v>
       </c>
       <c r="AP41" s="3">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="AQ41" s="3">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="AR41" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS41" s="3">
-        <v>2</v>
+        <v>-2</v>
       </c>
       <c r="AT41" s="3">
-        <v>1</v>
+        <v>-2</v>
       </c>
       <c r="AU41" s="3">
-        <v>1</v>
+        <v>-2</v>
       </c>
       <c r="AV41" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW41" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AX41" s="3">
-        <v>2</v>
+        <v>-1</v>
       </c>
       <c r="AY41" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AZ41" s="3">
         <v>1</v>
@@ -6958,7 +6967,7 @@
     </row>
     <row r="42" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B42" s="3">
         <v>0</v>
@@ -7116,7 +7125,7 @@
     </row>
     <row r="43" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B43" s="3">
         <v>1</v>
@@ -7274,7 +7283,7 @@
     </row>
     <row r="44" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B44" s="3">
         <v>0</v>
@@ -7432,142 +7441,142 @@
     </row>
     <row r="45" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B45" s="3">
-        <v>-2</v>
+        <v>1</v>
       </c>
       <c r="C45" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="D45" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="E45" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="F45" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G45" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H45" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="I45" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J45" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K45" s="3">
-        <v>1</v>
+        <v>-2</v>
       </c>
       <c r="L45" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="M45" s="3">
-        <v>-1</v>
+        <v>2</v>
       </c>
       <c r="N45" s="3">
         <v>0</v>
       </c>
       <c r="O45" s="3">
-        <v>1</v>
+        <v>-2</v>
       </c>
       <c r="P45" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="Q45" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R45" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="S45" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="T45" s="3">
         <v>0</v>
       </c>
       <c r="U45" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="V45" s="3">
         <v>1</v>
       </c>
       <c r="W45" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="X45" s="3">
         <v>0</v>
       </c>
       <c r="Y45" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Z45" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AA45" s="3">
         <v>-1</v>
       </c>
       <c r="AB45" s="3">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AC45" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AD45" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AE45" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AF45" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AG45" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AH45" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AI45" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AJ45" s="3">
-        <v>1</v>
+        <v>-2</v>
       </c>
       <c r="AK45" s="3">
         <v>0</v>
       </c>
       <c r="AL45" s="3">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="AM45" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AN45" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AO45" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AP45" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AQ45" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AR45" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AS45" s="3">
         <v>-11</v>
       </c>
       <c r="AT45" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AU45" s="3">
         <v>0</v>
@@ -7576,21 +7585,21 @@
         <v>1</v>
       </c>
       <c r="AW45" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AX45" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AY45" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AZ45" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="46" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B46" s="3">
         <v>0</v>
@@ -7748,7 +7757,7 @@
     </row>
     <row r="47" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B47" s="3">
         <v>1</v>
@@ -7906,7 +7915,7 @@
     </row>
     <row r="48" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B48" s="3">
         <v>2</v>
@@ -8064,10 +8073,10 @@
     </row>
     <row r="49" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B49" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C49" s="3">
         <v>1</v>
@@ -8079,10 +8088,10 @@
         <v>-1</v>
       </c>
       <c r="F49" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G49" s="3">
-        <v>1</v>
+        <v>-2</v>
       </c>
       <c r="H49" s="3">
         <v>0</v>
@@ -8097,28 +8106,28 @@
         <v>1</v>
       </c>
       <c r="L49" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M49" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="N49" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O49" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="P49" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q49" s="3">
-        <v>1</v>
+        <v>-2</v>
       </c>
       <c r="R49" s="3">
-        <v>1</v>
+        <v>-2</v>
       </c>
       <c r="S49" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="T49" s="3">
         <v>0</v>
@@ -8127,28 +8136,28 @@
         <v>0</v>
       </c>
       <c r="V49" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W49" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X49" s="3">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="Y49" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Z49" s="3">
         <v>1</v>
       </c>
       <c r="AA49" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AB49" s="3">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="AC49" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AD49" s="3">
         <v>0</v>
@@ -8157,7 +8166,7 @@
         <v>0</v>
       </c>
       <c r="AF49" s="3">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="AG49" s="3">
         <v>0</v>
@@ -8181,25 +8190,25 @@
         <v>1</v>
       </c>
       <c r="AN49" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AO49" s="3">
         <v>1</v>
       </c>
       <c r="AP49" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AQ49" s="3">
         <v>-1</v>
       </c>
       <c r="AR49" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AS49" s="3">
         <v>2</v>
       </c>
       <c r="AT49" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AU49" s="3">
         <v>0</v>
@@ -8211,18 +8220,18 @@
         <v>-11</v>
       </c>
       <c r="AX49" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AY49" s="3">
         <v>0</v>
       </c>
       <c r="AZ49" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="50" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B50" s="3">
         <v>-1</v>
@@ -8380,7 +8389,7 @@
     </row>
     <row r="51" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B51" s="3">
         <v>1</v>
@@ -8538,7 +8547,7 @@
     </row>
     <row r="52" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B52" s="3">
         <v>1</v>
@@ -9646,6 +9655,11 @@
     <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="1001" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
+  <conditionalFormatting sqref="B2:AZ53">
+    <cfRule type="expression" dxfId="0" priority="8">
+      <formula>B2&lt;&gt;INDIRECT(ADDRESS(MATCH(B$1,$A:$A,0),MATCH($A2,$1:$1,0)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.51180550000000002" right="0.51180550000000002" top="0.78749999999999998" bottom="0.78749999999999998" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>

</xml_diff>

<commit_message>
Ajustes no sistema de pontuação dos heróis inimigos.
</commit_message>
<xml_diff>
--- a/dist/OWPick/_internal/heroes ally.xlsx
+++ b/dist/OWPick/_internal/heroes ally.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DAVI\Projeto\Overwatch-Best-Picks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF91B967-6564-4AEF-86CA-349691FEBF1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98A9007E-3CED-4B27-9AA8-DF816AA2112F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -746,7 +746,7 @@
         <v>-1</v>
       </c>
       <c r="AH2" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AI2" s="3">
         <v>1</v>

</xml_diff>

<commit_message>
Ajustes no sistema de pontuação dos heróis inimigos e aliados.
</commit_message>
<xml_diff>
--- a/dist/OWPick/_internal/heroes ally.xlsx
+++ b/dist/OWPick/_internal/heroes ally.xlsx
@@ -1,26 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
-  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DAVI\Projeto\Overwatch-Best-Picks\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DAVI\Projetos\Overwatch-Best-Picks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98A9007E-3CED-4B27-9AA8-DF816AA2112F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
   </bookViews>
   <sheets>
     <sheet name="Página1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <si>
     <t>Hero</t>
   </si>
@@ -181,8 +179,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="4">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -229,13 +227,7 @@
     </fill>
   </fills>
   <borders count="1">
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
+    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -266,14 +258,6 @@
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
@@ -471,23 +455,20 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <outlinePr summaryRight="0" summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:AZ1001"/>
-  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="12.57031" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="7" width="12.5703125" customWidth="1"/>
+    <col min="1" max="7" width="12.57031" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" ht="15.75" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -645,7 +626,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="2" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" ht="15.75" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -656,7 +637,7 @@
         <v>0</v>
       </c>
       <c r="D2" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="E2" s="3">
         <v>0</v>
@@ -668,7 +649,7 @@
         <v>-1</v>
       </c>
       <c r="H2" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I2" s="3">
         <v>-1</v>
@@ -689,7 +670,7 @@
         <v>-2</v>
       </c>
       <c r="O2" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P2" s="3">
         <v>-1</v>
@@ -803,7 +784,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" ht="15.75" customHeight="1">
       <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
@@ -814,7 +795,7 @@
         <v>-11</v>
       </c>
       <c r="D3" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E3" s="3">
         <v>0</v>
@@ -826,7 +807,7 @@
         <v>0</v>
       </c>
       <c r="H3" s="3">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="I3" s="3">
         <v>-1</v>
@@ -847,7 +828,7 @@
         <v>0</v>
       </c>
       <c r="O3" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P3" s="3">
         <v>-1</v>
@@ -961,12 +942,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" ht="15.75" customHeight="1">
       <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
       <c r="B4" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C4" s="3">
         <v>0</v>
@@ -984,7 +965,7 @@
         <v>1</v>
       </c>
       <c r="H4" s="3">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="I4" s="3">
         <v>-1</v>
@@ -999,16 +980,16 @@
         <v>1</v>
       </c>
       <c r="M4" s="3">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="N4" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="O4" s="3">
         <v>0</v>
       </c>
       <c r="P4" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q4" s="3">
         <v>-1</v>
@@ -1017,28 +998,28 @@
         <v>1</v>
       </c>
       <c r="S4" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T4" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="U4" s="3">
         <v>0</v>
       </c>
       <c r="V4" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W4" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X4" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y4" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z4" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AA4" s="3">
         <v>0</v>
@@ -1050,37 +1031,37 @@
         <v>1</v>
       </c>
       <c r="AD4" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AE4" s="3">
         <v>1</v>
       </c>
       <c r="AF4" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AG4" s="3">
         <v>1</v>
       </c>
       <c r="AH4" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AI4" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AJ4" s="3">
         <v>1</v>
       </c>
       <c r="AK4" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AL4" s="3">
         <v>2</v>
       </c>
       <c r="AM4" s="3">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="AN4" s="3">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="AO4" s="3">
         <v>1</v>
@@ -1092,7 +1073,7 @@
         <v>1</v>
       </c>
       <c r="AR4" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AS4" s="3">
         <v>1</v>
@@ -1107,19 +1088,19 @@
         <v>-1</v>
       </c>
       <c r="AW4" s="3">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="AX4" s="3">
         <v>0</v>
       </c>
       <c r="AY4" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AZ4" s="3">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" ht="15.75" customHeight="1">
       <c r="A5" s="2" t="s">
         <v>4</v>
       </c>
@@ -1130,7 +1111,7 @@
         <v>0</v>
       </c>
       <c r="D5" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E5" s="3">
         <v>-11</v>
@@ -1163,7 +1144,7 @@
         <v>0</v>
       </c>
       <c r="O5" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="P5" s="3">
         <v>-1</v>
@@ -1277,7 +1258,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" ht="15.75" customHeight="1">
       <c r="A6" s="2" t="s">
         <v>5</v>
       </c>
@@ -1288,7 +1269,7 @@
         <v>-1</v>
       </c>
       <c r="D6" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E6" s="3">
         <v>1</v>
@@ -1321,7 +1302,7 @@
         <v>-1</v>
       </c>
       <c r="O6" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="P6" s="3">
         <v>-1</v>
@@ -1435,7 +1416,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" ht="15.75" customHeight="1">
       <c r="A7" s="2" t="s">
         <v>6</v>
       </c>
@@ -1446,7 +1427,7 @@
         <v>1</v>
       </c>
       <c r="D7" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="E7" s="3">
         <v>1</v>
@@ -1458,7 +1439,7 @@
         <v>-11</v>
       </c>
       <c r="H7" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I7" s="3">
         <v>-2</v>
@@ -1479,7 +1460,7 @@
         <v>1</v>
       </c>
       <c r="O7" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="P7" s="3">
         <v>0</v>
@@ -1509,7 +1490,7 @@
         <v>-1</v>
       </c>
       <c r="Y7" s="3">
-        <v>-1</v>
+        <v>-4</v>
       </c>
       <c r="Z7" s="3">
         <v>0</v>
@@ -1593,7 +1574,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="8" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" ht="15.75" customHeight="1">
       <c r="A8" s="2" t="s">
         <v>7</v>
       </c>
@@ -1613,7 +1594,7 @@
         <v>0</v>
       </c>
       <c r="G8" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H8" s="3">
         <v>-11</v>
@@ -1640,7 +1621,7 @@
         <v>0</v>
       </c>
       <c r="P8" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="Q8" s="3">
         <v>0</v>
@@ -1670,7 +1651,7 @@
         <v>1</v>
       </c>
       <c r="Z8" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA8" s="3">
         <v>1</v>
@@ -1679,7 +1660,7 @@
         <v>1</v>
       </c>
       <c r="AC8" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AD8" s="3">
         <v>0</v>
@@ -1706,7 +1687,7 @@
         <v>-1</v>
       </c>
       <c r="AL8" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AM8" s="3">
         <v>-1</v>
@@ -1718,28 +1699,28 @@
         <v>0</v>
       </c>
       <c r="AP8" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AQ8" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AR8" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AS8" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AT8" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AU8" s="3">
         <v>0</v>
       </c>
       <c r="AV8" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AW8" s="3">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="AX8" s="3">
         <v>0</v>
@@ -1751,7 +1732,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" ht="15.75" customHeight="1">
       <c r="A9" s="2" t="s">
         <v>8</v>
       </c>
@@ -1795,7 +1776,7 @@
         <v>1</v>
       </c>
       <c r="O9" s="3">
-        <v>-2</v>
+        <v>1</v>
       </c>
       <c r="P9" s="3">
         <v>1</v>
@@ -1909,7 +1890,7 @@
         <v>-2</v>
       </c>
     </row>
-    <row r="10" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" ht="15.75" customHeight="1">
       <c r="A10" s="2" t="s">
         <v>9</v>
       </c>
@@ -1920,7 +1901,7 @@
         <v>-1</v>
       </c>
       <c r="D10" s="3">
-        <v>-2</v>
+        <v>1</v>
       </c>
       <c r="E10" s="3">
         <v>-1</v>
@@ -1932,7 +1913,7 @@
         <v>0</v>
       </c>
       <c r="H10" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I10" s="3">
         <v>0</v>
@@ -1953,7 +1934,7 @@
         <v>0</v>
       </c>
       <c r="O10" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="P10" s="3">
         <v>0</v>
@@ -2067,7 +2048,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="11" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" ht="15.75" customHeight="1">
       <c r="A11" s="2" t="s">
         <v>10</v>
       </c>
@@ -2078,7 +2059,7 @@
         <v>0</v>
       </c>
       <c r="D11" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="E11" s="3">
         <v>1</v>
@@ -2090,7 +2071,7 @@
         <v>1</v>
       </c>
       <c r="H11" s="3">
-        <v>2</v>
+        <v>-1</v>
       </c>
       <c r="I11" s="3">
         <v>1</v>
@@ -2111,7 +2092,7 @@
         <v>0</v>
       </c>
       <c r="O11" s="3">
-        <v>-2</v>
+        <v>2</v>
       </c>
       <c r="P11" s="3">
         <v>2</v>
@@ -2225,7 +2206,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" ht="15.75" customHeight="1">
       <c r="A12" s="2" t="s">
         <v>11</v>
       </c>
@@ -2248,7 +2229,7 @@
         <v>2</v>
       </c>
       <c r="H12" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I12" s="3">
         <v>2</v>
@@ -2269,7 +2250,7 @@
         <v>1</v>
       </c>
       <c r="O12" s="3">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="P12" s="3">
         <v>0</v>
@@ -2383,7 +2364,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" ht="15.75" customHeight="1">
       <c r="A13" s="2" t="s">
         <v>12</v>
       </c>
@@ -2391,22 +2372,22 @@
         <v>0</v>
       </c>
       <c r="C13" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="D13" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="E13" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="F13" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="G13" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H13" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="I13" s="3">
         <v>0</v>
@@ -2427,7 +2408,7 @@
         <v>-1</v>
       </c>
       <c r="O13" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="P13" s="3">
         <v>1</v>
@@ -2541,7 +2522,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="14" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" ht="15.75" customHeight="1">
       <c r="A14" s="2" t="s">
         <v>13</v>
       </c>
@@ -2699,7 +2680,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" ht="15.75" customHeight="1">
       <c r="A15" s="2" t="s">
         <v>14</v>
       </c>
@@ -2707,7 +2688,7 @@
         <v>2</v>
       </c>
       <c r="C15" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D15" s="3">
         <v>0</v>
@@ -2734,13 +2715,13 @@
         <v>2</v>
       </c>
       <c r="L15" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="M15" s="3">
         <v>0</v>
       </c>
       <c r="N15" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O15" s="3">
         <v>-11</v>
@@ -2749,7 +2730,7 @@
         <v>-1</v>
       </c>
       <c r="Q15" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R15" s="3">
         <v>0</v>
@@ -2764,7 +2745,7 @@
         <v>0</v>
       </c>
       <c r="V15" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W15" s="3">
         <v>1</v>
@@ -2821,7 +2802,7 @@
         <v>0</v>
       </c>
       <c r="AO15" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AP15" s="3">
         <v>-2</v>
@@ -2830,13 +2811,13 @@
         <v>-1</v>
       </c>
       <c r="AR15" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AS15" s="3">
-        <v>2</v>
+        <v>-1</v>
       </c>
       <c r="AT15" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AU15" s="3">
         <v>0</v>
@@ -2854,10 +2835,10 @@
         <v>2</v>
       </c>
       <c r="AZ15" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" ht="15.75" customHeight="1">
       <c r="A16" s="2" t="s">
         <v>15</v>
       </c>
@@ -2880,7 +2861,7 @@
         <v>1</v>
       </c>
       <c r="H16" s="3">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="I16" s="3">
         <v>0</v>
@@ -2901,7 +2882,7 @@
         <v>1</v>
       </c>
       <c r="O16" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="P16" s="3">
         <v>-11</v>
@@ -3015,7 +2996,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" ht="15.75" customHeight="1">
       <c r="A17" s="2" t="s">
         <v>16</v>
       </c>
@@ -3026,7 +3007,7 @@
         <v>1</v>
       </c>
       <c r="D17" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="E17" s="3">
         <v>1</v>
@@ -3038,7 +3019,7 @@
         <v>1</v>
       </c>
       <c r="H17" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I17" s="3">
         <v>1</v>
@@ -3173,7 +3154,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" ht="15.75" customHeight="1">
       <c r="A18" s="2" t="s">
         <v>17</v>
       </c>
@@ -3184,7 +3165,7 @@
         <v>-1</v>
       </c>
       <c r="D18" s="3">
-        <v>-2</v>
+        <v>1</v>
       </c>
       <c r="E18" s="3">
         <v>1</v>
@@ -3217,7 +3198,7 @@
         <v>-1</v>
       </c>
       <c r="O18" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P18" s="3">
         <v>1</v>
@@ -3331,7 +3312,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" ht="15.75" customHeight="1">
       <c r="A19" s="2" t="s">
         <v>18</v>
       </c>
@@ -3342,7 +3323,7 @@
         <v>-1</v>
       </c>
       <c r="D19" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E19" s="3">
         <v>-1</v>
@@ -3354,7 +3335,7 @@
         <v>0</v>
       </c>
       <c r="H19" s="3">
-        <v>-2</v>
+        <v>2</v>
       </c>
       <c r="I19" s="3">
         <v>-2</v>
@@ -3375,7 +3356,7 @@
         <v>0</v>
       </c>
       <c r="O19" s="3">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="P19" s="3">
         <v>-2</v>
@@ -3489,7 +3470,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" ht="15.75" customHeight="1">
       <c r="A20" s="2" t="s">
         <v>19</v>
       </c>
@@ -3512,7 +3493,7 @@
         <v>0</v>
       </c>
       <c r="H20" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I20" s="3">
         <v>-1</v>
@@ -3533,7 +3514,7 @@
         <v>0</v>
       </c>
       <c r="O20" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P20" s="3">
         <v>-2</v>
@@ -3647,7 +3628,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="2" t="s">
         <v>20</v>
       </c>
@@ -3658,7 +3639,7 @@
         <v>-1</v>
       </c>
       <c r="D21" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E21" s="3">
         <v>-2</v>
@@ -3670,7 +3651,7 @@
         <v>0</v>
       </c>
       <c r="H21" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="I21" s="3">
         <v>-1</v>
@@ -3691,7 +3672,7 @@
         <v>-1</v>
       </c>
       <c r="O21" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="P21" s="3">
         <v>0</v>
@@ -3805,7 +3786,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="2" t="s">
         <v>21</v>
       </c>
@@ -3816,7 +3797,7 @@
         <v>1</v>
       </c>
       <c r="D22" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="E22" s="3">
         <v>-1</v>
@@ -3963,7 +3944,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="2" t="s">
         <v>22</v>
       </c>
@@ -3974,7 +3955,7 @@
         <v>1</v>
       </c>
       <c r="D23" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E23" s="3">
         <v>-1</v>
@@ -4007,7 +3988,7 @@
         <v>1</v>
       </c>
       <c r="O23" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P23" s="3">
         <v>1</v>
@@ -4121,7 +4102,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="2" t="s">
         <v>23</v>
       </c>
@@ -4144,7 +4125,7 @@
         <v>0</v>
       </c>
       <c r="H24" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="I24" s="3">
         <v>0</v>
@@ -4165,7 +4146,7 @@
         <v>0</v>
       </c>
       <c r="O24" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P24" s="3">
         <v>0</v>
@@ -4279,7 +4260,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="25" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="2" t="s">
         <v>24</v>
       </c>
@@ -4290,7 +4271,7 @@
         <v>0</v>
       </c>
       <c r="D25" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E25" s="3">
         <v>0</v>
@@ -4323,7 +4304,7 @@
         <v>0</v>
       </c>
       <c r="O25" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P25" s="3">
         <v>0</v>
@@ -4344,7 +4325,7 @@
         <v>0</v>
       </c>
       <c r="V25" s="3">
-        <v>1</v>
+        <v>-2</v>
       </c>
       <c r="W25" s="3">
         <v>1</v>
@@ -4437,7 +4418,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="2" t="s">
         <v>25</v>
       </c>
@@ -4460,7 +4441,7 @@
         <v>0</v>
       </c>
       <c r="H26" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="I26" s="3">
         <v>0</v>
@@ -4481,7 +4462,7 @@
         <v>0</v>
       </c>
       <c r="O26" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="P26" s="3">
         <v>0</v>
@@ -4595,7 +4576,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" ht="15.75" customHeight="1">
       <c r="A27" s="2" t="s">
         <v>26</v>
       </c>
@@ -4603,10 +4584,10 @@
         <v>1</v>
       </c>
       <c r="C27" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="D27" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E27" s="3">
         <v>1</v>
@@ -4753,7 +4734,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="28" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" ht="15.75" customHeight="1">
       <c r="A28" s="2" t="s">
         <v>27</v>
       </c>
@@ -4764,7 +4745,7 @@
         <v>0</v>
       </c>
       <c r="D28" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E28" s="3">
         <v>0</v>
@@ -4776,7 +4757,7 @@
         <v>0</v>
       </c>
       <c r="H28" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I28" s="3">
         <v>1</v>
@@ -4911,7 +4892,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" ht="15.75" customHeight="1">
       <c r="A29" s="2" t="s">
         <v>28</v>
       </c>
@@ -4922,7 +4903,7 @@
         <v>2</v>
       </c>
       <c r="D29" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E29" s="3">
         <v>-1</v>
@@ -5069,7 +5050,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" ht="15.75" customHeight="1">
       <c r="A30" s="2" t="s">
         <v>29</v>
       </c>
@@ -5092,7 +5073,7 @@
         <v>0</v>
       </c>
       <c r="H30" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="I30" s="3">
         <v>1</v>
@@ -5227,7 +5208,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="31" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" ht="15.75" customHeight="1">
       <c r="A31" s="2" t="s">
         <v>30</v>
       </c>
@@ -5385,7 +5366,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" ht="15.75" customHeight="1">
       <c r="A32" s="2" t="s">
         <v>31</v>
       </c>
@@ -5408,7 +5389,7 @@
         <v>0</v>
       </c>
       <c r="H32" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="I32" s="3">
         <v>0</v>
@@ -5429,7 +5410,7 @@
         <v>1</v>
       </c>
       <c r="O32" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P32" s="3">
         <v>0</v>
@@ -5543,7 +5524,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" ht="15.75" customHeight="1">
       <c r="A33" s="2" t="s">
         <v>32</v>
       </c>
@@ -5566,7 +5547,7 @@
         <v>0</v>
       </c>
       <c r="H33" s="3">
-        <v>-2</v>
+        <v>1</v>
       </c>
       <c r="I33" s="3">
         <v>0</v>
@@ -5701,7 +5682,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="34" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" ht="15.75" customHeight="1">
       <c r="A34" s="2" t="s">
         <v>33</v>
       </c>
@@ -5712,7 +5693,7 @@
         <v>0</v>
       </c>
       <c r="D34" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E34" s="3">
         <v>-2</v>
@@ -5745,7 +5726,7 @@
         <v>0</v>
       </c>
       <c r="O34" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P34" s="3">
         <v>0</v>
@@ -5859,7 +5840,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" ht="15.75" customHeight="1">
       <c r="A35" s="2" t="s">
         <v>34</v>
       </c>
@@ -5882,7 +5863,7 @@
         <v>-1</v>
       </c>
       <c r="H35" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I35" s="3">
         <v>1</v>
@@ -5903,7 +5884,7 @@
         <v>1</v>
       </c>
       <c r="O35" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="P35" s="3">
         <v>0</v>
@@ -6017,7 +5998,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" ht="15.75" customHeight="1">
       <c r="A36" s="2" t="s">
         <v>35</v>
       </c>
@@ -6028,7 +6009,7 @@
         <v>-1</v>
       </c>
       <c r="D36" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E36" s="3">
         <v>1</v>
@@ -6061,7 +6042,7 @@
         <v>0</v>
       </c>
       <c r="O36" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="P36" s="3">
         <v>1</v>
@@ -6175,7 +6156,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" ht="15.75" customHeight="1">
       <c r="A37" s="2" t="s">
         <v>36</v>
       </c>
@@ -6186,7 +6167,7 @@
         <v>0</v>
       </c>
       <c r="D37" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="E37" s="3">
         <v>0</v>
@@ -6198,7 +6179,7 @@
         <v>0</v>
       </c>
       <c r="H37" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="I37" s="3">
         <v>0</v>
@@ -6333,7 +6314,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" ht="15.75" customHeight="1">
       <c r="A38" s="2" t="s">
         <v>37</v>
       </c>
@@ -6344,7 +6325,7 @@
         <v>0</v>
       </c>
       <c r="D38" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E38" s="3">
         <v>2</v>
@@ -6377,7 +6358,7 @@
         <v>0</v>
       </c>
       <c r="O38" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="P38" s="3">
         <v>1</v>
@@ -6491,7 +6472,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" ht="15.75" customHeight="1">
       <c r="A39" s="2" t="s">
         <v>38</v>
       </c>
@@ -6502,7 +6483,7 @@
         <v>0</v>
       </c>
       <c r="D39" s="3">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="E39" s="3">
         <v>2</v>
@@ -6514,7 +6495,7 @@
         <v>0</v>
       </c>
       <c r="H39" s="3">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="I39" s="3">
         <v>0</v>
@@ -6535,7 +6516,7 @@
         <v>0</v>
       </c>
       <c r="O39" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P39" s="3">
         <v>0</v>
@@ -6649,7 +6630,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" ht="15.75" customHeight="1">
       <c r="A40" s="2" t="s">
         <v>39</v>
       </c>
@@ -6660,7 +6641,7 @@
         <v>0</v>
       </c>
       <c r="D40" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="E40" s="3">
         <v>-1</v>
@@ -6672,7 +6653,7 @@
         <v>0</v>
       </c>
       <c r="H40" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="I40" s="3">
         <v>-1</v>
@@ -6693,7 +6674,7 @@
         <v>0</v>
       </c>
       <c r="O40" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P40" s="3">
         <v>0</v>
@@ -6807,7 +6788,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" ht="15.75" customHeight="1">
       <c r="A41" s="2" t="s">
         <v>40</v>
       </c>
@@ -6830,7 +6811,7 @@
         <v>2</v>
       </c>
       <c r="H41" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I41" s="3">
         <v>1</v>
@@ -6851,7 +6832,7 @@
         <v>-1</v>
       </c>
       <c r="O41" s="3">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="P41" s="3">
         <v>-2</v>
@@ -6965,7 +6946,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" ht="15.75" customHeight="1">
       <c r="A42" s="2" t="s">
         <v>41</v>
       </c>
@@ -7009,7 +6990,7 @@
         <v>0</v>
       </c>
       <c r="O42" s="3">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="P42" s="3">
         <v>1</v>
@@ -7123,7 +7104,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="43" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" ht="15.75" customHeight="1">
       <c r="A43" s="2" t="s">
         <v>42</v>
       </c>
@@ -7134,7 +7115,7 @@
         <v>-1</v>
       </c>
       <c r="D43" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E43" s="3">
         <v>-1</v>
@@ -7146,7 +7127,7 @@
         <v>0</v>
       </c>
       <c r="H43" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I43" s="3">
         <v>1</v>
@@ -7281,7 +7262,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="44" ht="15.75" customHeight="1">
       <c r="A44" s="2" t="s">
         <v>43</v>
       </c>
@@ -7289,7 +7270,7 @@
         <v>0</v>
       </c>
       <c r="C44" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D44" s="3">
         <v>1</v>
@@ -7325,7 +7306,7 @@
         <v>0</v>
       </c>
       <c r="O44" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P44" s="3">
         <v>0</v>
@@ -7439,7 +7420,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="45" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" ht="15.75" customHeight="1">
       <c r="A45" s="2" t="s">
         <v>44</v>
       </c>
@@ -7450,7 +7431,7 @@
         <v>-1</v>
       </c>
       <c r="D45" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E45" s="3">
         <v>-1</v>
@@ -7483,7 +7464,7 @@
         <v>0</v>
       </c>
       <c r="O45" s="3">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="P45" s="3">
         <v>-1</v>
@@ -7597,7 +7578,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="46" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" ht="15.75" customHeight="1">
       <c r="A46" s="2" t="s">
         <v>45</v>
       </c>
@@ -7608,7 +7589,7 @@
         <v>1</v>
       </c>
       <c r="D46" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E46" s="3">
         <v>0</v>
@@ -7641,7 +7622,7 @@
         <v>0</v>
       </c>
       <c r="O46" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P46" s="3">
         <v>0</v>
@@ -7755,7 +7736,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" ht="15.75" customHeight="1">
       <c r="A47" s="2" t="s">
         <v>46</v>
       </c>
@@ -7766,7 +7747,7 @@
         <v>0</v>
       </c>
       <c r="D47" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="E47" s="3">
         <v>1</v>
@@ -7913,7 +7894,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" ht="15.75" customHeight="1">
       <c r="A48" s="2" t="s">
         <v>47</v>
       </c>
@@ -7924,7 +7905,7 @@
         <v>1</v>
       </c>
       <c r="D48" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="E48" s="3">
         <v>1</v>
@@ -8071,7 +8052,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" ht="15.75" customHeight="1">
       <c r="A49" s="2" t="s">
         <v>48</v>
       </c>
@@ -8082,7 +8063,7 @@
         <v>1</v>
       </c>
       <c r="D49" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="E49" s="3">
         <v>-1</v>
@@ -8094,7 +8075,7 @@
         <v>-2</v>
       </c>
       <c r="H49" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="I49" s="3">
         <v>1</v>
@@ -8229,7 +8210,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="50" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" ht="15.75" customHeight="1">
       <c r="A50" s="2" t="s">
         <v>49</v>
       </c>
@@ -8240,7 +8221,7 @@
         <v>-2</v>
       </c>
       <c r="D50" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="E50" s="3">
         <v>-1</v>
@@ -8252,7 +8233,7 @@
         <v>0</v>
       </c>
       <c r="H50" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="I50" s="3">
         <v>1</v>
@@ -8273,7 +8254,7 @@
         <v>2</v>
       </c>
       <c r="O50" s="3">
-        <v>-2</v>
+        <v>1</v>
       </c>
       <c r="P50" s="3">
         <v>0</v>
@@ -8387,7 +8368,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" ht="15.75" customHeight="1">
       <c r="A51" s="2" t="s">
         <v>50</v>
       </c>
@@ -8398,7 +8379,7 @@
         <v>1</v>
       </c>
       <c r="D51" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E51" s="3">
         <v>1</v>
@@ -8431,7 +8412,7 @@
         <v>0</v>
       </c>
       <c r="O51" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P51" s="3">
         <v>0</v>
@@ -8545,7 +8526,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="52" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="52" ht="15.75" customHeight="1">
       <c r="A52" s="2" t="s">
         <v>51</v>
       </c>
@@ -8556,7 +8537,7 @@
         <v>1</v>
       </c>
       <c r="D52" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E52" s="3">
         <v>2</v>
@@ -8703,964 +8684,964 @@
         <v>-11</v>
       </c>
     </row>
-    <row r="53" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="53" ht="15.75" customHeight="1">
       <c r="J53" s="3"/>
     </row>
-    <row r="54" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="55" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="56" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="57" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="58" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="59" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="60" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="61" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="62" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="63" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="64" spans="1:52" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="65" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="66" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="67" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="68" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="69" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="70" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="71" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="72" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="73" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="74" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="75" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="76" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="77" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="78" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="79" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="80" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="81" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="82" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="83" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="84" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="85" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="86" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="87" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="88" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="89" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="90" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="91" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="92" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="93" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="94" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="95" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="96" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="97" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="98" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="99" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="100" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="101" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="102" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="103" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="104" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="105" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="106" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="107" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="108" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="109" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="110" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="111" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="112" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="113" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="114" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="115" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="116" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="117" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="118" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="119" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="120" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="121" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="122" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="123" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="124" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="125" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="126" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="127" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="128" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="129" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="130" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="131" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="132" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="133" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="134" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="135" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="136" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="137" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="138" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="139" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="140" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="141" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="142" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="143" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="144" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="145" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="146" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="147" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="148" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="149" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="150" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="151" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="152" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="153" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="154" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="155" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="156" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="157" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="158" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="159" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="160" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="161" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="162" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="163" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="164" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="165" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="166" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="167" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="168" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="169" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="170" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="171" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="172" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="173" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="174" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="175" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="176" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="177" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="178" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="179" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="180" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="181" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="182" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="183" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="184" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="185" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="186" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="187" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="188" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="189" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="190" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="191" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="192" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="193" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="194" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="195" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="196" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="197" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="198" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="199" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="200" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="201" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="202" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="203" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="204" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="205" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="206" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="207" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="208" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="209" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="210" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="211" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="212" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="213" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="214" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="215" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="216" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="217" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="218" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="219" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="220" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="221" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="222" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="223" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="224" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="225" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="226" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="227" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="228" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="229" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="230" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="231" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="232" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="233" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="234" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="235" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="236" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="237" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="238" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="239" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="240" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="241" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="242" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="243" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="244" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="245" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="246" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="247" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="248" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="249" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="250" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="251" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="252" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="253" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="254" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="255" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="256" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="257" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="258" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="259" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="260" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="261" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="262" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="263" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="264" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="265" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="266" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="267" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="268" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="269" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="270" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="271" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="272" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="273" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="274" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="275" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="276" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="277" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="278" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="279" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="280" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="281" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="282" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="283" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="284" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="285" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="286" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="287" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="288" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="289" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="290" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="291" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="292" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="293" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="294" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="295" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="296" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="297" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="298" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="299" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="300" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="301" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="302" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="303" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="304" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="305" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="306" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="307" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="308" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="309" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="310" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="311" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="312" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="313" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="314" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="315" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="316" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="317" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="318" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="319" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="320" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="321" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="322" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="323" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="324" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="325" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="326" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="327" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="328" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="329" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="330" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="331" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="332" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="333" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="334" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="335" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="336" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="337" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="338" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="339" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="340" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="341" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="342" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="343" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="344" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="345" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="346" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="347" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="348" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="349" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="350" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="351" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="352" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="353" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="354" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="355" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="356" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="357" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="358" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="359" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="360" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="361" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="362" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="363" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="364" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="365" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="366" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="367" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="368" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="369" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="370" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="371" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="372" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="373" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="374" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="375" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="376" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="377" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="378" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="379" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="380" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="381" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="382" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="383" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="384" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="385" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="386" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="387" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="388" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="389" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="390" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="391" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="392" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="393" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="394" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="395" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="396" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="397" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="398" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="399" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="400" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="401" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="402" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="403" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="404" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="405" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="406" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="407" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="408" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="409" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="410" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="411" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="412" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="413" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="414" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="415" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="416" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="417" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="418" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="419" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="420" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="421" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="422" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="423" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="424" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="425" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="426" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="427" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="428" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="429" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="430" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="431" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="432" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="433" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="434" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="435" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="436" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="437" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="438" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="439" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="440" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="441" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="442" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="443" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="444" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="445" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="446" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="447" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="448" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="449" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="450" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="451" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="452" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="453" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="454" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="455" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="456" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="457" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="458" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="459" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="460" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="461" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="462" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="463" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="464" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="465" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="466" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="467" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="468" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="469" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="470" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="471" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="472" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="473" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="474" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="475" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="476" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="477" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="478" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="479" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="480" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="481" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="482" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="483" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="484" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="485" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="486" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="487" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="488" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="489" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="490" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="491" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="492" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="493" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="494" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="495" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="496" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="497" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="498" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="499" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="500" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="501" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="502" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="503" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="504" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="505" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="506" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="507" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="508" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="509" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="510" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="511" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="512" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="513" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="514" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="515" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="516" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="517" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="518" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="519" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="520" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="521" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="522" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="523" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="524" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="525" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="526" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="527" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="528" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="529" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="530" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="531" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="532" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="533" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="534" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="535" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="536" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="537" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="538" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="539" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="540" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="541" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="542" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="543" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="544" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="545" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="546" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="547" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="548" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="549" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="550" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="551" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="552" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="553" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="554" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="555" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="556" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="557" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="558" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="559" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="560" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="561" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="562" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="563" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="564" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="565" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="566" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="567" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="568" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="569" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="570" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="571" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="572" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="573" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="574" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="575" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="576" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="577" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="578" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="579" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="580" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="581" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="582" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="583" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="584" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="585" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="586" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="587" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="588" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="589" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="590" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="591" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="592" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="593" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="594" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="595" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="596" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="597" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="598" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="599" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="600" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="601" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="602" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="603" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="604" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="605" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="606" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="607" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="608" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="609" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="610" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="611" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="612" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="613" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="614" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="615" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="616" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="617" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="618" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="619" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="620" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="621" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="622" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="623" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="624" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="625" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="626" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="627" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="628" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="629" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="630" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="631" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="632" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="633" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="634" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="635" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="636" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="637" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="638" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="639" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="640" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="641" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="642" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="643" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="644" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="645" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="646" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="647" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="648" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="649" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="650" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="651" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="652" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="653" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="654" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="655" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="656" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="657" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="658" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="659" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="660" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="661" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="662" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="663" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="664" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="665" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="666" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="667" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="668" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="669" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="670" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="671" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="672" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="673" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="674" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="675" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="676" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="677" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="678" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="679" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="680" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="681" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="682" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="683" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="684" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="685" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="686" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="687" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="688" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="689" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="690" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="691" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="692" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="693" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="694" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="695" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="696" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="697" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="698" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="699" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="700" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="701" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="702" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="703" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="704" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="705" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="706" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="707" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="708" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="709" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="710" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="711" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="712" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="713" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="714" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="715" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="716" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="717" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="718" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="719" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="720" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="721" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="722" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="723" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="724" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="725" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="726" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="727" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="728" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="729" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="730" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="731" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="732" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="733" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="734" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="735" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="736" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="737" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="738" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="739" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="740" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="741" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="742" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="743" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="744" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="745" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="746" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="747" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="748" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="749" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="750" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="751" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="752" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="753" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="754" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="755" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="756" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="757" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="758" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="759" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="760" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="761" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="762" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="763" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="764" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="765" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="766" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="767" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="768" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="769" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="770" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="771" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="772" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="773" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="774" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="775" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="776" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="777" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="778" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="779" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="780" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="781" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="782" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="783" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="784" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="785" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="786" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="787" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="788" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="789" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="790" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="791" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="792" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="793" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="794" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="795" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="796" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="797" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="798" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="799" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="800" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="801" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="802" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="803" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="804" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="805" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="806" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="807" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="808" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="809" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="810" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="811" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="812" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="813" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="814" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="815" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="816" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="817" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="818" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="819" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="820" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="821" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="822" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="823" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="824" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="825" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="826" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="827" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="828" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="829" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="830" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="831" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="832" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="833" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="834" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="835" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="836" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="837" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="838" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="839" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="840" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="841" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="842" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="843" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="844" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="845" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="846" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="847" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="848" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="849" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="850" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="851" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="852" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="853" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="854" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="855" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="856" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="857" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="858" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="859" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="860" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="861" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="862" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="863" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="864" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="865" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="866" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="867" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="868" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="869" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="870" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="871" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="872" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="873" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="874" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="875" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="876" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="877" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="878" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="879" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="880" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="881" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="882" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="883" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="884" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="885" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="886" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="887" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="888" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="889" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="890" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="891" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="892" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="893" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="894" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="895" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="896" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="897" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="898" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="899" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="900" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="901" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="902" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="903" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="904" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="905" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="906" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="907" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="908" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="909" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="910" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="911" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="912" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="913" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="914" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="915" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="916" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="917" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="918" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="919" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="920" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="921" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="922" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="923" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="924" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="925" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="926" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="927" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="928" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="929" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="930" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="931" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="932" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="933" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="934" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="935" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="936" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="937" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="938" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="939" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="940" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="941" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="942" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="943" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="944" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="945" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="946" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="947" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="948" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="949" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="950" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="951" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="952" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="953" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="954" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="955" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="956" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="957" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="958" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="959" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="960" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="961" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="962" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="963" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="964" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="965" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="966" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="967" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="968" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="969" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="970" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="971" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="972" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="973" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="974" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="975" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="976" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="977" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="978" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="979" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="980" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="981" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="982" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="983" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="984" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="985" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="986" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="987" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="988" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="989" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="990" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="991" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="992" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="993" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="994" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="995" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="996" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="997" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="998" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="999" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="1001" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="54" ht="15.75" customHeight="1"/>
+    <row r="55" ht="15.75" customHeight="1"/>
+    <row r="56" ht="15.75" customHeight="1"/>
+    <row r="57" ht="15.75" customHeight="1"/>
+    <row r="58" ht="15.75" customHeight="1"/>
+    <row r="59" ht="15.75" customHeight="1"/>
+    <row r="60" ht="15.75" customHeight="1"/>
+    <row r="61" ht="15.75" customHeight="1"/>
+    <row r="62" ht="15.75" customHeight="1"/>
+    <row r="63" ht="15.75" customHeight="1"/>
+    <row r="64" ht="15.75" customHeight="1"/>
+    <row r="65" ht="15.75" customHeight="1"/>
+    <row r="66" ht="15.75" customHeight="1"/>
+    <row r="67" ht="15.75" customHeight="1"/>
+    <row r="68" ht="15.75" customHeight="1"/>
+    <row r="69" ht="15.75" customHeight="1"/>
+    <row r="70" ht="15.75" customHeight="1"/>
+    <row r="71" ht="15.75" customHeight="1"/>
+    <row r="72" ht="15.75" customHeight="1"/>
+    <row r="73" ht="15.75" customHeight="1"/>
+    <row r="74" ht="15.75" customHeight="1"/>
+    <row r="75" ht="15.75" customHeight="1"/>
+    <row r="76" ht="15.75" customHeight="1"/>
+    <row r="77" ht="15.75" customHeight="1"/>
+    <row r="78" ht="15.75" customHeight="1"/>
+    <row r="79" ht="15.75" customHeight="1"/>
+    <row r="80" ht="15.75" customHeight="1"/>
+    <row r="81" ht="15.75" customHeight="1"/>
+    <row r="82" ht="15.75" customHeight="1"/>
+    <row r="83" ht="15.75" customHeight="1"/>
+    <row r="84" ht="15.75" customHeight="1"/>
+    <row r="85" ht="15.75" customHeight="1"/>
+    <row r="86" ht="15.75" customHeight="1"/>
+    <row r="87" ht="15.75" customHeight="1"/>
+    <row r="88" ht="15.75" customHeight="1"/>
+    <row r="89" ht="15.75" customHeight="1"/>
+    <row r="90" ht="15.75" customHeight="1"/>
+    <row r="91" ht="15.75" customHeight="1"/>
+    <row r="92" ht="15.75" customHeight="1"/>
+    <row r="93" ht="15.75" customHeight="1"/>
+    <row r="94" ht="15.75" customHeight="1"/>
+    <row r="95" ht="15.75" customHeight="1"/>
+    <row r="96" ht="15.75" customHeight="1"/>
+    <row r="97" ht="15.75" customHeight="1"/>
+    <row r="98" ht="15.75" customHeight="1"/>
+    <row r="99" ht="15.75" customHeight="1"/>
+    <row r="100" ht="15.75" customHeight="1"/>
+    <row r="101" ht="15.75" customHeight="1"/>
+    <row r="102" ht="15.75" customHeight="1"/>
+    <row r="103" ht="15.75" customHeight="1"/>
+    <row r="104" ht="15.75" customHeight="1"/>
+    <row r="105" ht="15.75" customHeight="1"/>
+    <row r="106" ht="15.75" customHeight="1"/>
+    <row r="107" ht="15.75" customHeight="1"/>
+    <row r="108" ht="15.75" customHeight="1"/>
+    <row r="109" ht="15.75" customHeight="1"/>
+    <row r="110" ht="15.75" customHeight="1"/>
+    <row r="111" ht="15.75" customHeight="1"/>
+    <row r="112" ht="15.75" customHeight="1"/>
+    <row r="113" ht="15.75" customHeight="1"/>
+    <row r="114" ht="15.75" customHeight="1"/>
+    <row r="115" ht="15.75" customHeight="1"/>
+    <row r="116" ht="15.75" customHeight="1"/>
+    <row r="117" ht="15.75" customHeight="1"/>
+    <row r="118" ht="15.75" customHeight="1"/>
+    <row r="119" ht="15.75" customHeight="1"/>
+    <row r="120" ht="15.75" customHeight="1"/>
+    <row r="121" ht="15.75" customHeight="1"/>
+    <row r="122" ht="15.75" customHeight="1"/>
+    <row r="123" ht="15.75" customHeight="1"/>
+    <row r="124" ht="15.75" customHeight="1"/>
+    <row r="125" ht="15.75" customHeight="1"/>
+    <row r="126" ht="15.75" customHeight="1"/>
+    <row r="127" ht="15.75" customHeight="1"/>
+    <row r="128" ht="15.75" customHeight="1"/>
+    <row r="129" ht="15.75" customHeight="1"/>
+    <row r="130" ht="15.75" customHeight="1"/>
+    <row r="131" ht="15.75" customHeight="1"/>
+    <row r="132" ht="15.75" customHeight="1"/>
+    <row r="133" ht="15.75" customHeight="1"/>
+    <row r="134" ht="15.75" customHeight="1"/>
+    <row r="135" ht="15.75" customHeight="1"/>
+    <row r="136" ht="15.75" customHeight="1"/>
+    <row r="137" ht="15.75" customHeight="1"/>
+    <row r="138" ht="15.75" customHeight="1"/>
+    <row r="139" ht="15.75" customHeight="1"/>
+    <row r="140" ht="15.75" customHeight="1"/>
+    <row r="141" ht="15.75" customHeight="1"/>
+    <row r="142" ht="15.75" customHeight="1"/>
+    <row r="143" ht="15.75" customHeight="1"/>
+    <row r="144" ht="15.75" customHeight="1"/>
+    <row r="145" ht="15.75" customHeight="1"/>
+    <row r="146" ht="15.75" customHeight="1"/>
+    <row r="147" ht="15.75" customHeight="1"/>
+    <row r="148" ht="15.75" customHeight="1"/>
+    <row r="149" ht="15.75" customHeight="1"/>
+    <row r="150" ht="15.75" customHeight="1"/>
+    <row r="151" ht="15.75" customHeight="1"/>
+    <row r="152" ht="15.75" customHeight="1"/>
+    <row r="153" ht="15.75" customHeight="1"/>
+    <row r="154" ht="15.75" customHeight="1"/>
+    <row r="155" ht="15.75" customHeight="1"/>
+    <row r="156" ht="15.75" customHeight="1"/>
+    <row r="157" ht="15.75" customHeight="1"/>
+    <row r="158" ht="15.75" customHeight="1"/>
+    <row r="159" ht="15.75" customHeight="1"/>
+    <row r="160" ht="15.75" customHeight="1"/>
+    <row r="161" ht="15.75" customHeight="1"/>
+    <row r="162" ht="15.75" customHeight="1"/>
+    <row r="163" ht="15.75" customHeight="1"/>
+    <row r="164" ht="15.75" customHeight="1"/>
+    <row r="165" ht="15.75" customHeight="1"/>
+    <row r="166" ht="15.75" customHeight="1"/>
+    <row r="167" ht="15.75" customHeight="1"/>
+    <row r="168" ht="15.75" customHeight="1"/>
+    <row r="169" ht="15.75" customHeight="1"/>
+    <row r="170" ht="15.75" customHeight="1"/>
+    <row r="171" ht="15.75" customHeight="1"/>
+    <row r="172" ht="15.75" customHeight="1"/>
+    <row r="173" ht="15.75" customHeight="1"/>
+    <row r="174" ht="15.75" customHeight="1"/>
+    <row r="175" ht="15.75" customHeight="1"/>
+    <row r="176" ht="15.75" customHeight="1"/>
+    <row r="177" ht="15.75" customHeight="1"/>
+    <row r="178" ht="15.75" customHeight="1"/>
+    <row r="179" ht="15.75" customHeight="1"/>
+    <row r="180" ht="15.75" customHeight="1"/>
+    <row r="181" ht="15.75" customHeight="1"/>
+    <row r="182" ht="15.75" customHeight="1"/>
+    <row r="183" ht="15.75" customHeight="1"/>
+    <row r="184" ht="15.75" customHeight="1"/>
+    <row r="185" ht="15.75" customHeight="1"/>
+    <row r="186" ht="15.75" customHeight="1"/>
+    <row r="187" ht="15.75" customHeight="1"/>
+    <row r="188" ht="15.75" customHeight="1"/>
+    <row r="189" ht="15.75" customHeight="1"/>
+    <row r="190" ht="15.75" customHeight="1"/>
+    <row r="191" ht="15.75" customHeight="1"/>
+    <row r="192" ht="15.75" customHeight="1"/>
+    <row r="193" ht="15.75" customHeight="1"/>
+    <row r="194" ht="15.75" customHeight="1"/>
+    <row r="195" ht="15.75" customHeight="1"/>
+    <row r="196" ht="15.75" customHeight="1"/>
+    <row r="197" ht="15.75" customHeight="1"/>
+    <row r="198" ht="15.75" customHeight="1"/>
+    <row r="199" ht="15.75" customHeight="1"/>
+    <row r="200" ht="15.75" customHeight="1"/>
+    <row r="201" ht="15.75" customHeight="1"/>
+    <row r="202" ht="15.75" customHeight="1"/>
+    <row r="203" ht="15.75" customHeight="1"/>
+    <row r="204" ht="15.75" customHeight="1"/>
+    <row r="205" ht="15.75" customHeight="1"/>
+    <row r="206" ht="15.75" customHeight="1"/>
+    <row r="207" ht="15.75" customHeight="1"/>
+    <row r="208" ht="15.75" customHeight="1"/>
+    <row r="209" ht="15.75" customHeight="1"/>
+    <row r="210" ht="15.75" customHeight="1"/>
+    <row r="211" ht="15.75" customHeight="1"/>
+    <row r="212" ht="15.75" customHeight="1"/>
+    <row r="213" ht="15.75" customHeight="1"/>
+    <row r="214" ht="15.75" customHeight="1"/>
+    <row r="215" ht="15.75" customHeight="1"/>
+    <row r="216" ht="15.75" customHeight="1"/>
+    <row r="217" ht="15.75" customHeight="1"/>
+    <row r="218" ht="15.75" customHeight="1"/>
+    <row r="219" ht="15.75" customHeight="1"/>
+    <row r="220" ht="15.75" customHeight="1"/>
+    <row r="221" ht="15.75" customHeight="1"/>
+    <row r="222" ht="15.75" customHeight="1"/>
+    <row r="223" ht="15.75" customHeight="1"/>
+    <row r="224" ht="15.75" customHeight="1"/>
+    <row r="225" ht="15.75" customHeight="1"/>
+    <row r="226" ht="15.75" customHeight="1"/>
+    <row r="227" ht="15.75" customHeight="1"/>
+    <row r="228" ht="15.75" customHeight="1"/>
+    <row r="229" ht="15.75" customHeight="1"/>
+    <row r="230" ht="15.75" customHeight="1"/>
+    <row r="231" ht="15.75" customHeight="1"/>
+    <row r="232" ht="15.75" customHeight="1"/>
+    <row r="233" ht="15.75" customHeight="1"/>
+    <row r="234" ht="15.75" customHeight="1"/>
+    <row r="235" ht="15.75" customHeight="1"/>
+    <row r="236" ht="15.75" customHeight="1"/>
+    <row r="237" ht="15.75" customHeight="1"/>
+    <row r="238" ht="15.75" customHeight="1"/>
+    <row r="239" ht="15.75" customHeight="1"/>
+    <row r="240" ht="15.75" customHeight="1"/>
+    <row r="241" ht="15.75" customHeight="1"/>
+    <row r="242" ht="15.75" customHeight="1"/>
+    <row r="243" ht="15.75" customHeight="1"/>
+    <row r="244" ht="15.75" customHeight="1"/>
+    <row r="245" ht="15.75" customHeight="1"/>
+    <row r="246" ht="15.75" customHeight="1"/>
+    <row r="247" ht="15.75" customHeight="1"/>
+    <row r="248" ht="15.75" customHeight="1"/>
+    <row r="249" ht="15.75" customHeight="1"/>
+    <row r="250" ht="15.75" customHeight="1"/>
+    <row r="251" ht="15.75" customHeight="1"/>
+    <row r="252" ht="15.75" customHeight="1"/>
+    <row r="253" ht="15.75" customHeight="1"/>
+    <row r="254" ht="15.75" customHeight="1"/>
+    <row r="255" ht="15.75" customHeight="1"/>
+    <row r="256" ht="15.75" customHeight="1"/>
+    <row r="257" ht="15.75" customHeight="1"/>
+    <row r="258" ht="15.75" customHeight="1"/>
+    <row r="259" ht="15.75" customHeight="1"/>
+    <row r="260" ht="15.75" customHeight="1"/>
+    <row r="261" ht="15.75" customHeight="1"/>
+    <row r="262" ht="15.75" customHeight="1"/>
+    <row r="263" ht="15.75" customHeight="1"/>
+    <row r="264" ht="15.75" customHeight="1"/>
+    <row r="265" ht="15.75" customHeight="1"/>
+    <row r="266" ht="15.75" customHeight="1"/>
+    <row r="267" ht="15.75" customHeight="1"/>
+    <row r="268" ht="15.75" customHeight="1"/>
+    <row r="269" ht="15.75" customHeight="1"/>
+    <row r="270" ht="15.75" customHeight="1"/>
+    <row r="271" ht="15.75" customHeight="1"/>
+    <row r="272" ht="15.75" customHeight="1"/>
+    <row r="273" ht="15.75" customHeight="1"/>
+    <row r="274" ht="15.75" customHeight="1"/>
+    <row r="275" ht="15.75" customHeight="1"/>
+    <row r="276" ht="15.75" customHeight="1"/>
+    <row r="277" ht="15.75" customHeight="1"/>
+    <row r="278" ht="15.75" customHeight="1"/>
+    <row r="279" ht="15.75" customHeight="1"/>
+    <row r="280" ht="15.75" customHeight="1"/>
+    <row r="281" ht="15.75" customHeight="1"/>
+    <row r="282" ht="15.75" customHeight="1"/>
+    <row r="283" ht="15.75" customHeight="1"/>
+    <row r="284" ht="15.75" customHeight="1"/>
+    <row r="285" ht="15.75" customHeight="1"/>
+    <row r="286" ht="15.75" customHeight="1"/>
+    <row r="287" ht="15.75" customHeight="1"/>
+    <row r="288" ht="15.75" customHeight="1"/>
+    <row r="289" ht="15.75" customHeight="1"/>
+    <row r="290" ht="15.75" customHeight="1"/>
+    <row r="291" ht="15.75" customHeight="1"/>
+    <row r="292" ht="15.75" customHeight="1"/>
+    <row r="293" ht="15.75" customHeight="1"/>
+    <row r="294" ht="15.75" customHeight="1"/>
+    <row r="295" ht="15.75" customHeight="1"/>
+    <row r="296" ht="15.75" customHeight="1"/>
+    <row r="297" ht="15.75" customHeight="1"/>
+    <row r="298" ht="15.75" customHeight="1"/>
+    <row r="299" ht="15.75" customHeight="1"/>
+    <row r="300" ht="15.75" customHeight="1"/>
+    <row r="301" ht="15.75" customHeight="1"/>
+    <row r="302" ht="15.75" customHeight="1"/>
+    <row r="303" ht="15.75" customHeight="1"/>
+    <row r="304" ht="15.75" customHeight="1"/>
+    <row r="305" ht="15.75" customHeight="1"/>
+    <row r="306" ht="15.75" customHeight="1"/>
+    <row r="307" ht="15.75" customHeight="1"/>
+    <row r="308" ht="15.75" customHeight="1"/>
+    <row r="309" ht="15.75" customHeight="1"/>
+    <row r="310" ht="15.75" customHeight="1"/>
+    <row r="311" ht="15.75" customHeight="1"/>
+    <row r="312" ht="15.75" customHeight="1"/>
+    <row r="313" ht="15.75" customHeight="1"/>
+    <row r="314" ht="15.75" customHeight="1"/>
+    <row r="315" ht="15.75" customHeight="1"/>
+    <row r="316" ht="15.75" customHeight="1"/>
+    <row r="317" ht="15.75" customHeight="1"/>
+    <row r="318" ht="15.75" customHeight="1"/>
+    <row r="319" ht="15.75" customHeight="1"/>
+    <row r="320" ht="15.75" customHeight="1"/>
+    <row r="321" ht="15.75" customHeight="1"/>
+    <row r="322" ht="15.75" customHeight="1"/>
+    <row r="323" ht="15.75" customHeight="1"/>
+    <row r="324" ht="15.75" customHeight="1"/>
+    <row r="325" ht="15.75" customHeight="1"/>
+    <row r="326" ht="15.75" customHeight="1"/>
+    <row r="327" ht="15.75" customHeight="1"/>
+    <row r="328" ht="15.75" customHeight="1"/>
+    <row r="329" ht="15.75" customHeight="1"/>
+    <row r="330" ht="15.75" customHeight="1"/>
+    <row r="331" ht="15.75" customHeight="1"/>
+    <row r="332" ht="15.75" customHeight="1"/>
+    <row r="333" ht="15.75" customHeight="1"/>
+    <row r="334" ht="15.75" customHeight="1"/>
+    <row r="335" ht="15.75" customHeight="1"/>
+    <row r="336" ht="15.75" customHeight="1"/>
+    <row r="337" ht="15.75" customHeight="1"/>
+    <row r="338" ht="15.75" customHeight="1"/>
+    <row r="339" ht="15.75" customHeight="1"/>
+    <row r="340" ht="15.75" customHeight="1"/>
+    <row r="341" ht="15.75" customHeight="1"/>
+    <row r="342" ht="15.75" customHeight="1"/>
+    <row r="343" ht="15.75" customHeight="1"/>
+    <row r="344" ht="15.75" customHeight="1"/>
+    <row r="345" ht="15.75" customHeight="1"/>
+    <row r="346" ht="15.75" customHeight="1"/>
+    <row r="347" ht="15.75" customHeight="1"/>
+    <row r="348" ht="15.75" customHeight="1"/>
+    <row r="349" ht="15.75" customHeight="1"/>
+    <row r="350" ht="15.75" customHeight="1"/>
+    <row r="351" ht="15.75" customHeight="1"/>
+    <row r="352" ht="15.75" customHeight="1"/>
+    <row r="353" ht="15.75" customHeight="1"/>
+    <row r="354" ht="15.75" customHeight="1"/>
+    <row r="355" ht="15.75" customHeight="1"/>
+    <row r="356" ht="15.75" customHeight="1"/>
+    <row r="357" ht="15.75" customHeight="1"/>
+    <row r="358" ht="15.75" customHeight="1"/>
+    <row r="359" ht="15.75" customHeight="1"/>
+    <row r="360" ht="15.75" customHeight="1"/>
+    <row r="361" ht="15.75" customHeight="1"/>
+    <row r="362" ht="15.75" customHeight="1"/>
+    <row r="363" ht="15.75" customHeight="1"/>
+    <row r="364" ht="15.75" customHeight="1"/>
+    <row r="365" ht="15.75" customHeight="1"/>
+    <row r="366" ht="15.75" customHeight="1"/>
+    <row r="367" ht="15.75" customHeight="1"/>
+    <row r="368" ht="15.75" customHeight="1"/>
+    <row r="369" ht="15.75" customHeight="1"/>
+    <row r="370" ht="15.75" customHeight="1"/>
+    <row r="371" ht="15.75" customHeight="1"/>
+    <row r="372" ht="15.75" customHeight="1"/>
+    <row r="373" ht="15.75" customHeight="1"/>
+    <row r="374" ht="15.75" customHeight="1"/>
+    <row r="375" ht="15.75" customHeight="1"/>
+    <row r="376" ht="15.75" customHeight="1"/>
+    <row r="377" ht="15.75" customHeight="1"/>
+    <row r="378" ht="15.75" customHeight="1"/>
+    <row r="379" ht="15.75" customHeight="1"/>
+    <row r="380" ht="15.75" customHeight="1"/>
+    <row r="381" ht="15.75" customHeight="1"/>
+    <row r="382" ht="15.75" customHeight="1"/>
+    <row r="383" ht="15.75" customHeight="1"/>
+    <row r="384" ht="15.75" customHeight="1"/>
+    <row r="385" ht="15.75" customHeight="1"/>
+    <row r="386" ht="15.75" customHeight="1"/>
+    <row r="387" ht="15.75" customHeight="1"/>
+    <row r="388" ht="15.75" customHeight="1"/>
+    <row r="389" ht="15.75" customHeight="1"/>
+    <row r="390" ht="15.75" customHeight="1"/>
+    <row r="391" ht="15.75" customHeight="1"/>
+    <row r="392" ht="15.75" customHeight="1"/>
+    <row r="393" ht="15.75" customHeight="1"/>
+    <row r="394" ht="15.75" customHeight="1"/>
+    <row r="395" ht="15.75" customHeight="1"/>
+    <row r="396" ht="15.75" customHeight="1"/>
+    <row r="397" ht="15.75" customHeight="1"/>
+    <row r="398" ht="15.75" customHeight="1"/>
+    <row r="399" ht="15.75" customHeight="1"/>
+    <row r="400" ht="15.75" customHeight="1"/>
+    <row r="401" ht="15.75" customHeight="1"/>
+    <row r="402" ht="15.75" customHeight="1"/>
+    <row r="403" ht="15.75" customHeight="1"/>
+    <row r="404" ht="15.75" customHeight="1"/>
+    <row r="405" ht="15.75" customHeight="1"/>
+    <row r="406" ht="15.75" customHeight="1"/>
+    <row r="407" ht="15.75" customHeight="1"/>
+    <row r="408" ht="15.75" customHeight="1"/>
+    <row r="409" ht="15.75" customHeight="1"/>
+    <row r="410" ht="15.75" customHeight="1"/>
+    <row r="411" ht="15.75" customHeight="1"/>
+    <row r="412" ht="15.75" customHeight="1"/>
+    <row r="413" ht="15.75" customHeight="1"/>
+    <row r="414" ht="15.75" customHeight="1"/>
+    <row r="415" ht="15.75" customHeight="1"/>
+    <row r="416" ht="15.75" customHeight="1"/>
+    <row r="417" ht="15.75" customHeight="1"/>
+    <row r="418" ht="15.75" customHeight="1"/>
+    <row r="419" ht="15.75" customHeight="1"/>
+    <row r="420" ht="15.75" customHeight="1"/>
+    <row r="421" ht="15.75" customHeight="1"/>
+    <row r="422" ht="15.75" customHeight="1"/>
+    <row r="423" ht="15.75" customHeight="1"/>
+    <row r="424" ht="15.75" customHeight="1"/>
+    <row r="425" ht="15.75" customHeight="1"/>
+    <row r="426" ht="15.75" customHeight="1"/>
+    <row r="427" ht="15.75" customHeight="1"/>
+    <row r="428" ht="15.75" customHeight="1"/>
+    <row r="429" ht="15.75" customHeight="1"/>
+    <row r="430" ht="15.75" customHeight="1"/>
+    <row r="431" ht="15.75" customHeight="1"/>
+    <row r="432" ht="15.75" customHeight="1"/>
+    <row r="433" ht="15.75" customHeight="1"/>
+    <row r="434" ht="15.75" customHeight="1"/>
+    <row r="435" ht="15.75" customHeight="1"/>
+    <row r="436" ht="15.75" customHeight="1"/>
+    <row r="437" ht="15.75" customHeight="1"/>
+    <row r="438" ht="15.75" customHeight="1"/>
+    <row r="439" ht="15.75" customHeight="1"/>
+    <row r="440" ht="15.75" customHeight="1"/>
+    <row r="441" ht="15.75" customHeight="1"/>
+    <row r="442" ht="15.75" customHeight="1"/>
+    <row r="443" ht="15.75" customHeight="1"/>
+    <row r="444" ht="15.75" customHeight="1"/>
+    <row r="445" ht="15.75" customHeight="1"/>
+    <row r="446" ht="15.75" customHeight="1"/>
+    <row r="447" ht="15.75" customHeight="1"/>
+    <row r="448" ht="15.75" customHeight="1"/>
+    <row r="449" ht="15.75" customHeight="1"/>
+    <row r="450" ht="15.75" customHeight="1"/>
+    <row r="451" ht="15.75" customHeight="1"/>
+    <row r="452" ht="15.75" customHeight="1"/>
+    <row r="453" ht="15.75" customHeight="1"/>
+    <row r="454" ht="15.75" customHeight="1"/>
+    <row r="455" ht="15.75" customHeight="1"/>
+    <row r="456" ht="15.75" customHeight="1"/>
+    <row r="457" ht="15.75" customHeight="1"/>
+    <row r="458" ht="15.75" customHeight="1"/>
+    <row r="459" ht="15.75" customHeight="1"/>
+    <row r="460" ht="15.75" customHeight="1"/>
+    <row r="461" ht="15.75" customHeight="1"/>
+    <row r="462" ht="15.75" customHeight="1"/>
+    <row r="463" ht="15.75" customHeight="1"/>
+    <row r="464" ht="15.75" customHeight="1"/>
+    <row r="465" ht="15.75" customHeight="1"/>
+    <row r="466" ht="15.75" customHeight="1"/>
+    <row r="467" ht="15.75" customHeight="1"/>
+    <row r="468" ht="15.75" customHeight="1"/>
+    <row r="469" ht="15.75" customHeight="1"/>
+    <row r="470" ht="15.75" customHeight="1"/>
+    <row r="471" ht="15.75" customHeight="1"/>
+    <row r="472" ht="15.75" customHeight="1"/>
+    <row r="473" ht="15.75" customHeight="1"/>
+    <row r="474" ht="15.75" customHeight="1"/>
+    <row r="475" ht="15.75" customHeight="1"/>
+    <row r="476" ht="15.75" customHeight="1"/>
+    <row r="477" ht="15.75" customHeight="1"/>
+    <row r="478" ht="15.75" customHeight="1"/>
+    <row r="479" ht="15.75" customHeight="1"/>
+    <row r="480" ht="15.75" customHeight="1"/>
+    <row r="481" ht="15.75" customHeight="1"/>
+    <row r="482" ht="15.75" customHeight="1"/>
+    <row r="483" ht="15.75" customHeight="1"/>
+    <row r="484" ht="15.75" customHeight="1"/>
+    <row r="485" ht="15.75" customHeight="1"/>
+    <row r="486" ht="15.75" customHeight="1"/>
+    <row r="487" ht="15.75" customHeight="1"/>
+    <row r="488" ht="15.75" customHeight="1"/>
+    <row r="489" ht="15.75" customHeight="1"/>
+    <row r="490" ht="15.75" customHeight="1"/>
+    <row r="491" ht="15.75" customHeight="1"/>
+    <row r="492" ht="15.75" customHeight="1"/>
+    <row r="493" ht="15.75" customHeight="1"/>
+    <row r="494" ht="15.75" customHeight="1"/>
+    <row r="495" ht="15.75" customHeight="1"/>
+    <row r="496" ht="15.75" customHeight="1"/>
+    <row r="497" ht="15.75" customHeight="1"/>
+    <row r="498" ht="15.75" customHeight="1"/>
+    <row r="499" ht="15.75" customHeight="1"/>
+    <row r="500" ht="15.75" customHeight="1"/>
+    <row r="501" ht="15.75" customHeight="1"/>
+    <row r="502" ht="15.75" customHeight="1"/>
+    <row r="503" ht="15.75" customHeight="1"/>
+    <row r="504" ht="15.75" customHeight="1"/>
+    <row r="505" ht="15.75" customHeight="1"/>
+    <row r="506" ht="15.75" customHeight="1"/>
+    <row r="507" ht="15.75" customHeight="1"/>
+    <row r="508" ht="15.75" customHeight="1"/>
+    <row r="509" ht="15.75" customHeight="1"/>
+    <row r="510" ht="15.75" customHeight="1"/>
+    <row r="511" ht="15.75" customHeight="1"/>
+    <row r="512" ht="15.75" customHeight="1"/>
+    <row r="513" ht="15.75" customHeight="1"/>
+    <row r="514" ht="15.75" customHeight="1"/>
+    <row r="515" ht="15.75" customHeight="1"/>
+    <row r="516" ht="15.75" customHeight="1"/>
+    <row r="517" ht="15.75" customHeight="1"/>
+    <row r="518" ht="15.75" customHeight="1"/>
+    <row r="519" ht="15.75" customHeight="1"/>
+    <row r="520" ht="15.75" customHeight="1"/>
+    <row r="521" ht="15.75" customHeight="1"/>
+    <row r="522" ht="15.75" customHeight="1"/>
+    <row r="523" ht="15.75" customHeight="1"/>
+    <row r="524" ht="15.75" customHeight="1"/>
+    <row r="525" ht="15.75" customHeight="1"/>
+    <row r="526" ht="15.75" customHeight="1"/>
+    <row r="527" ht="15.75" customHeight="1"/>
+    <row r="528" ht="15.75" customHeight="1"/>
+    <row r="529" ht="15.75" customHeight="1"/>
+    <row r="530" ht="15.75" customHeight="1"/>
+    <row r="531" ht="15.75" customHeight="1"/>
+    <row r="532" ht="15.75" customHeight="1"/>
+    <row r="533" ht="15.75" customHeight="1"/>
+    <row r="534" ht="15.75" customHeight="1"/>
+    <row r="535" ht="15.75" customHeight="1"/>
+    <row r="536" ht="15.75" customHeight="1"/>
+    <row r="537" ht="15.75" customHeight="1"/>
+    <row r="538" ht="15.75" customHeight="1"/>
+    <row r="539" ht="15.75" customHeight="1"/>
+    <row r="540" ht="15.75" customHeight="1"/>
+    <row r="541" ht="15.75" customHeight="1"/>
+    <row r="542" ht="15.75" customHeight="1"/>
+    <row r="543" ht="15.75" customHeight="1"/>
+    <row r="544" ht="15.75" customHeight="1"/>
+    <row r="545" ht="15.75" customHeight="1"/>
+    <row r="546" ht="15.75" customHeight="1"/>
+    <row r="547" ht="15.75" customHeight="1"/>
+    <row r="548" ht="15.75" customHeight="1"/>
+    <row r="549" ht="15.75" customHeight="1"/>
+    <row r="550" ht="15.75" customHeight="1"/>
+    <row r="551" ht="15.75" customHeight="1"/>
+    <row r="552" ht="15.75" customHeight="1"/>
+    <row r="553" ht="15.75" customHeight="1"/>
+    <row r="554" ht="15.75" customHeight="1"/>
+    <row r="555" ht="15.75" customHeight="1"/>
+    <row r="556" ht="15.75" customHeight="1"/>
+    <row r="557" ht="15.75" customHeight="1"/>
+    <row r="558" ht="15.75" customHeight="1"/>
+    <row r="559" ht="15.75" customHeight="1"/>
+    <row r="560" ht="15.75" customHeight="1"/>
+    <row r="561" ht="15.75" customHeight="1"/>
+    <row r="562" ht="15.75" customHeight="1"/>
+    <row r="563" ht="15.75" customHeight="1"/>
+    <row r="564" ht="15.75" customHeight="1"/>
+    <row r="565" ht="15.75" customHeight="1"/>
+    <row r="566" ht="15.75" customHeight="1"/>
+    <row r="567" ht="15.75" customHeight="1"/>
+    <row r="568" ht="15.75" customHeight="1"/>
+    <row r="569" ht="15.75" customHeight="1"/>
+    <row r="570" ht="15.75" customHeight="1"/>
+    <row r="571" ht="15.75" customHeight="1"/>
+    <row r="572" ht="15.75" customHeight="1"/>
+    <row r="573" ht="15.75" customHeight="1"/>
+    <row r="574" ht="15.75" customHeight="1"/>
+    <row r="575" ht="15.75" customHeight="1"/>
+    <row r="576" ht="15.75" customHeight="1"/>
+    <row r="577" ht="15.75" customHeight="1"/>
+    <row r="578" ht="15.75" customHeight="1"/>
+    <row r="579" ht="15.75" customHeight="1"/>
+    <row r="580" ht="15.75" customHeight="1"/>
+    <row r="581" ht="15.75" customHeight="1"/>
+    <row r="582" ht="15.75" customHeight="1"/>
+    <row r="583" ht="15.75" customHeight="1"/>
+    <row r="584" ht="15.75" customHeight="1"/>
+    <row r="585" ht="15.75" customHeight="1"/>
+    <row r="586" ht="15.75" customHeight="1"/>
+    <row r="587" ht="15.75" customHeight="1"/>
+    <row r="588" ht="15.75" customHeight="1"/>
+    <row r="589" ht="15.75" customHeight="1"/>
+    <row r="590" ht="15.75" customHeight="1"/>
+    <row r="591" ht="15.75" customHeight="1"/>
+    <row r="592" ht="15.75" customHeight="1"/>
+    <row r="593" ht="15.75" customHeight="1"/>
+    <row r="594" ht="15.75" customHeight="1"/>
+    <row r="595" ht="15.75" customHeight="1"/>
+    <row r="596" ht="15.75" customHeight="1"/>
+    <row r="597" ht="15.75" customHeight="1"/>
+    <row r="598" ht="15.75" customHeight="1"/>
+    <row r="599" ht="15.75" customHeight="1"/>
+    <row r="600" ht="15.75" customHeight="1"/>
+    <row r="601" ht="15.75" customHeight="1"/>
+    <row r="602" ht="15.75" customHeight="1"/>
+    <row r="603" ht="15.75" customHeight="1"/>
+    <row r="604" ht="15.75" customHeight="1"/>
+    <row r="605" ht="15.75" customHeight="1"/>
+    <row r="606" ht="15.75" customHeight="1"/>
+    <row r="607" ht="15.75" customHeight="1"/>
+    <row r="608" ht="15.75" customHeight="1"/>
+    <row r="609" ht="15.75" customHeight="1"/>
+    <row r="610" ht="15.75" customHeight="1"/>
+    <row r="611" ht="15.75" customHeight="1"/>
+    <row r="612" ht="15.75" customHeight="1"/>
+    <row r="613" ht="15.75" customHeight="1"/>
+    <row r="614" ht="15.75" customHeight="1"/>
+    <row r="615" ht="15.75" customHeight="1"/>
+    <row r="616" ht="15.75" customHeight="1"/>
+    <row r="617" ht="15.75" customHeight="1"/>
+    <row r="618" ht="15.75" customHeight="1"/>
+    <row r="619" ht="15.75" customHeight="1"/>
+    <row r="620" ht="15.75" customHeight="1"/>
+    <row r="621" ht="15.75" customHeight="1"/>
+    <row r="622" ht="15.75" customHeight="1"/>
+    <row r="623" ht="15.75" customHeight="1"/>
+    <row r="624" ht="15.75" customHeight="1"/>
+    <row r="625" ht="15.75" customHeight="1"/>
+    <row r="626" ht="15.75" customHeight="1"/>
+    <row r="627" ht="15.75" customHeight="1"/>
+    <row r="628" ht="15.75" customHeight="1"/>
+    <row r="629" ht="15.75" customHeight="1"/>
+    <row r="630" ht="15.75" customHeight="1"/>
+    <row r="631" ht="15.75" customHeight="1"/>
+    <row r="632" ht="15.75" customHeight="1"/>
+    <row r="633" ht="15.75" customHeight="1"/>
+    <row r="634" ht="15.75" customHeight="1"/>
+    <row r="635" ht="15.75" customHeight="1"/>
+    <row r="636" ht="15.75" customHeight="1"/>
+    <row r="637" ht="15.75" customHeight="1"/>
+    <row r="638" ht="15.75" customHeight="1"/>
+    <row r="639" ht="15.75" customHeight="1"/>
+    <row r="640" ht="15.75" customHeight="1"/>
+    <row r="641" ht="15.75" customHeight="1"/>
+    <row r="642" ht="15.75" customHeight="1"/>
+    <row r="643" ht="15.75" customHeight="1"/>
+    <row r="644" ht="15.75" customHeight="1"/>
+    <row r="645" ht="15.75" customHeight="1"/>
+    <row r="646" ht="15.75" customHeight="1"/>
+    <row r="647" ht="15.75" customHeight="1"/>
+    <row r="648" ht="15.75" customHeight="1"/>
+    <row r="649" ht="15.75" customHeight="1"/>
+    <row r="650" ht="15.75" customHeight="1"/>
+    <row r="651" ht="15.75" customHeight="1"/>
+    <row r="652" ht="15.75" customHeight="1"/>
+    <row r="653" ht="15.75" customHeight="1"/>
+    <row r="654" ht="15.75" customHeight="1"/>
+    <row r="655" ht="15.75" customHeight="1"/>
+    <row r="656" ht="15.75" customHeight="1"/>
+    <row r="657" ht="15.75" customHeight="1"/>
+    <row r="658" ht="15.75" customHeight="1"/>
+    <row r="659" ht="15.75" customHeight="1"/>
+    <row r="660" ht="15.75" customHeight="1"/>
+    <row r="661" ht="15.75" customHeight="1"/>
+    <row r="662" ht="15.75" customHeight="1"/>
+    <row r="663" ht="15.75" customHeight="1"/>
+    <row r="664" ht="15.75" customHeight="1"/>
+    <row r="665" ht="15.75" customHeight="1"/>
+    <row r="666" ht="15.75" customHeight="1"/>
+    <row r="667" ht="15.75" customHeight="1"/>
+    <row r="668" ht="15.75" customHeight="1"/>
+    <row r="669" ht="15.75" customHeight="1"/>
+    <row r="670" ht="15.75" customHeight="1"/>
+    <row r="671" ht="15.75" customHeight="1"/>
+    <row r="672" ht="15.75" customHeight="1"/>
+    <row r="673" ht="15.75" customHeight="1"/>
+    <row r="674" ht="15.75" customHeight="1"/>
+    <row r="675" ht="15.75" customHeight="1"/>
+    <row r="676" ht="15.75" customHeight="1"/>
+    <row r="677" ht="15.75" customHeight="1"/>
+    <row r="678" ht="15.75" customHeight="1"/>
+    <row r="679" ht="15.75" customHeight="1"/>
+    <row r="680" ht="15.75" customHeight="1"/>
+    <row r="681" ht="15.75" customHeight="1"/>
+    <row r="682" ht="15.75" customHeight="1"/>
+    <row r="683" ht="15.75" customHeight="1"/>
+    <row r="684" ht="15.75" customHeight="1"/>
+    <row r="685" ht="15.75" customHeight="1"/>
+    <row r="686" ht="15.75" customHeight="1"/>
+    <row r="687" ht="15.75" customHeight="1"/>
+    <row r="688" ht="15.75" customHeight="1"/>
+    <row r="689" ht="15.75" customHeight="1"/>
+    <row r="690" ht="15.75" customHeight="1"/>
+    <row r="691" ht="15.75" customHeight="1"/>
+    <row r="692" ht="15.75" customHeight="1"/>
+    <row r="693" ht="15.75" customHeight="1"/>
+    <row r="694" ht="15.75" customHeight="1"/>
+    <row r="695" ht="15.75" customHeight="1"/>
+    <row r="696" ht="15.75" customHeight="1"/>
+    <row r="697" ht="15.75" customHeight="1"/>
+    <row r="698" ht="15.75" customHeight="1"/>
+    <row r="699" ht="15.75" customHeight="1"/>
+    <row r="700" ht="15.75" customHeight="1"/>
+    <row r="701" ht="15.75" customHeight="1"/>
+    <row r="702" ht="15.75" customHeight="1"/>
+    <row r="703" ht="15.75" customHeight="1"/>
+    <row r="704" ht="15.75" customHeight="1"/>
+    <row r="705" ht="15.75" customHeight="1"/>
+    <row r="706" ht="15.75" customHeight="1"/>
+    <row r="707" ht="15.75" customHeight="1"/>
+    <row r="708" ht="15.75" customHeight="1"/>
+    <row r="709" ht="15.75" customHeight="1"/>
+    <row r="710" ht="15.75" customHeight="1"/>
+    <row r="711" ht="15.75" customHeight="1"/>
+    <row r="712" ht="15.75" customHeight="1"/>
+    <row r="713" ht="15.75" customHeight="1"/>
+    <row r="714" ht="15.75" customHeight="1"/>
+    <row r="715" ht="15.75" customHeight="1"/>
+    <row r="716" ht="15.75" customHeight="1"/>
+    <row r="717" ht="15.75" customHeight="1"/>
+    <row r="718" ht="15.75" customHeight="1"/>
+    <row r="719" ht="15.75" customHeight="1"/>
+    <row r="720" ht="15.75" customHeight="1"/>
+    <row r="721" ht="15.75" customHeight="1"/>
+    <row r="722" ht="15.75" customHeight="1"/>
+    <row r="723" ht="15.75" customHeight="1"/>
+    <row r="724" ht="15.75" customHeight="1"/>
+    <row r="725" ht="15.75" customHeight="1"/>
+    <row r="726" ht="15.75" customHeight="1"/>
+    <row r="727" ht="15.75" customHeight="1"/>
+    <row r="728" ht="15.75" customHeight="1"/>
+    <row r="729" ht="15.75" customHeight="1"/>
+    <row r="730" ht="15.75" customHeight="1"/>
+    <row r="731" ht="15.75" customHeight="1"/>
+    <row r="732" ht="15.75" customHeight="1"/>
+    <row r="733" ht="15.75" customHeight="1"/>
+    <row r="734" ht="15.75" customHeight="1"/>
+    <row r="735" ht="15.75" customHeight="1"/>
+    <row r="736" ht="15.75" customHeight="1"/>
+    <row r="737" ht="15.75" customHeight="1"/>
+    <row r="738" ht="15.75" customHeight="1"/>
+    <row r="739" ht="15.75" customHeight="1"/>
+    <row r="740" ht="15.75" customHeight="1"/>
+    <row r="741" ht="15.75" customHeight="1"/>
+    <row r="742" ht="15.75" customHeight="1"/>
+    <row r="743" ht="15.75" customHeight="1"/>
+    <row r="744" ht="15.75" customHeight="1"/>
+    <row r="745" ht="15.75" customHeight="1"/>
+    <row r="746" ht="15.75" customHeight="1"/>
+    <row r="747" ht="15.75" customHeight="1"/>
+    <row r="748" ht="15.75" customHeight="1"/>
+    <row r="749" ht="15.75" customHeight="1"/>
+    <row r="750" ht="15.75" customHeight="1"/>
+    <row r="751" ht="15.75" customHeight="1"/>
+    <row r="752" ht="15.75" customHeight="1"/>
+    <row r="753" ht="15.75" customHeight="1"/>
+    <row r="754" ht="15.75" customHeight="1"/>
+    <row r="755" ht="15.75" customHeight="1"/>
+    <row r="756" ht="15.75" customHeight="1"/>
+    <row r="757" ht="15.75" customHeight="1"/>
+    <row r="758" ht="15.75" customHeight="1"/>
+    <row r="759" ht="15.75" customHeight="1"/>
+    <row r="760" ht="15.75" customHeight="1"/>
+    <row r="761" ht="15.75" customHeight="1"/>
+    <row r="762" ht="15.75" customHeight="1"/>
+    <row r="763" ht="15.75" customHeight="1"/>
+    <row r="764" ht="15.75" customHeight="1"/>
+    <row r="765" ht="15.75" customHeight="1"/>
+    <row r="766" ht="15.75" customHeight="1"/>
+    <row r="767" ht="15.75" customHeight="1"/>
+    <row r="768" ht="15.75" customHeight="1"/>
+    <row r="769" ht="15.75" customHeight="1"/>
+    <row r="770" ht="15.75" customHeight="1"/>
+    <row r="771" ht="15.75" customHeight="1"/>
+    <row r="772" ht="15.75" customHeight="1"/>
+    <row r="773" ht="15.75" customHeight="1"/>
+    <row r="774" ht="15.75" customHeight="1"/>
+    <row r="775" ht="15.75" customHeight="1"/>
+    <row r="776" ht="15.75" customHeight="1"/>
+    <row r="777" ht="15.75" customHeight="1"/>
+    <row r="778" ht="15.75" customHeight="1"/>
+    <row r="779" ht="15.75" customHeight="1"/>
+    <row r="780" ht="15.75" customHeight="1"/>
+    <row r="781" ht="15.75" customHeight="1"/>
+    <row r="782" ht="15.75" customHeight="1"/>
+    <row r="783" ht="15.75" customHeight="1"/>
+    <row r="784" ht="15.75" customHeight="1"/>
+    <row r="785" ht="15.75" customHeight="1"/>
+    <row r="786" ht="15.75" customHeight="1"/>
+    <row r="787" ht="15.75" customHeight="1"/>
+    <row r="788" ht="15.75" customHeight="1"/>
+    <row r="789" ht="15.75" customHeight="1"/>
+    <row r="790" ht="15.75" customHeight="1"/>
+    <row r="791" ht="15.75" customHeight="1"/>
+    <row r="792" ht="15.75" customHeight="1"/>
+    <row r="793" ht="15.75" customHeight="1"/>
+    <row r="794" ht="15.75" customHeight="1"/>
+    <row r="795" ht="15.75" customHeight="1"/>
+    <row r="796" ht="15.75" customHeight="1"/>
+    <row r="797" ht="15.75" customHeight="1"/>
+    <row r="798" ht="15.75" customHeight="1"/>
+    <row r="799" ht="15.75" customHeight="1"/>
+    <row r="800" ht="15.75" customHeight="1"/>
+    <row r="801" ht="15.75" customHeight="1"/>
+    <row r="802" ht="15.75" customHeight="1"/>
+    <row r="803" ht="15.75" customHeight="1"/>
+    <row r="804" ht="15.75" customHeight="1"/>
+    <row r="805" ht="15.75" customHeight="1"/>
+    <row r="806" ht="15.75" customHeight="1"/>
+    <row r="807" ht="15.75" customHeight="1"/>
+    <row r="808" ht="15.75" customHeight="1"/>
+    <row r="809" ht="15.75" customHeight="1"/>
+    <row r="810" ht="15.75" customHeight="1"/>
+    <row r="811" ht="15.75" customHeight="1"/>
+    <row r="812" ht="15.75" customHeight="1"/>
+    <row r="813" ht="15.75" customHeight="1"/>
+    <row r="814" ht="15.75" customHeight="1"/>
+    <row r="815" ht="15.75" customHeight="1"/>
+    <row r="816" ht="15.75" customHeight="1"/>
+    <row r="817" ht="15.75" customHeight="1"/>
+    <row r="818" ht="15.75" customHeight="1"/>
+    <row r="819" ht="15.75" customHeight="1"/>
+    <row r="820" ht="15.75" customHeight="1"/>
+    <row r="821" ht="15.75" customHeight="1"/>
+    <row r="822" ht="15.75" customHeight="1"/>
+    <row r="823" ht="15.75" customHeight="1"/>
+    <row r="824" ht="15.75" customHeight="1"/>
+    <row r="825" ht="15.75" customHeight="1"/>
+    <row r="826" ht="15.75" customHeight="1"/>
+    <row r="827" ht="15.75" customHeight="1"/>
+    <row r="828" ht="15.75" customHeight="1"/>
+    <row r="829" ht="15.75" customHeight="1"/>
+    <row r="830" ht="15.75" customHeight="1"/>
+    <row r="831" ht="15.75" customHeight="1"/>
+    <row r="832" ht="15.75" customHeight="1"/>
+    <row r="833" ht="15.75" customHeight="1"/>
+    <row r="834" ht="15.75" customHeight="1"/>
+    <row r="835" ht="15.75" customHeight="1"/>
+    <row r="836" ht="15.75" customHeight="1"/>
+    <row r="837" ht="15.75" customHeight="1"/>
+    <row r="838" ht="15.75" customHeight="1"/>
+    <row r="839" ht="15.75" customHeight="1"/>
+    <row r="840" ht="15.75" customHeight="1"/>
+    <row r="841" ht="15.75" customHeight="1"/>
+    <row r="842" ht="15.75" customHeight="1"/>
+    <row r="843" ht="15.75" customHeight="1"/>
+    <row r="844" ht="15.75" customHeight="1"/>
+    <row r="845" ht="15.75" customHeight="1"/>
+    <row r="846" ht="15.75" customHeight="1"/>
+    <row r="847" ht="15.75" customHeight="1"/>
+    <row r="848" ht="15.75" customHeight="1"/>
+    <row r="849" ht="15.75" customHeight="1"/>
+    <row r="850" ht="15.75" customHeight="1"/>
+    <row r="851" ht="15.75" customHeight="1"/>
+    <row r="852" ht="15.75" customHeight="1"/>
+    <row r="853" ht="15.75" customHeight="1"/>
+    <row r="854" ht="15.75" customHeight="1"/>
+    <row r="855" ht="15.75" customHeight="1"/>
+    <row r="856" ht="15.75" customHeight="1"/>
+    <row r="857" ht="15.75" customHeight="1"/>
+    <row r="858" ht="15.75" customHeight="1"/>
+    <row r="859" ht="15.75" customHeight="1"/>
+    <row r="860" ht="15.75" customHeight="1"/>
+    <row r="861" ht="15.75" customHeight="1"/>
+    <row r="862" ht="15.75" customHeight="1"/>
+    <row r="863" ht="15.75" customHeight="1"/>
+    <row r="864" ht="15.75" customHeight="1"/>
+    <row r="865" ht="15.75" customHeight="1"/>
+    <row r="866" ht="15.75" customHeight="1"/>
+    <row r="867" ht="15.75" customHeight="1"/>
+    <row r="868" ht="15.75" customHeight="1"/>
+    <row r="869" ht="15.75" customHeight="1"/>
+    <row r="870" ht="15.75" customHeight="1"/>
+    <row r="871" ht="15.75" customHeight="1"/>
+    <row r="872" ht="15.75" customHeight="1"/>
+    <row r="873" ht="15.75" customHeight="1"/>
+    <row r="874" ht="15.75" customHeight="1"/>
+    <row r="875" ht="15.75" customHeight="1"/>
+    <row r="876" ht="15.75" customHeight="1"/>
+    <row r="877" ht="15.75" customHeight="1"/>
+    <row r="878" ht="15.75" customHeight="1"/>
+    <row r="879" ht="15.75" customHeight="1"/>
+    <row r="880" ht="15.75" customHeight="1"/>
+    <row r="881" ht="15.75" customHeight="1"/>
+    <row r="882" ht="15.75" customHeight="1"/>
+    <row r="883" ht="15.75" customHeight="1"/>
+    <row r="884" ht="15.75" customHeight="1"/>
+    <row r="885" ht="15.75" customHeight="1"/>
+    <row r="886" ht="15.75" customHeight="1"/>
+    <row r="887" ht="15.75" customHeight="1"/>
+    <row r="888" ht="15.75" customHeight="1"/>
+    <row r="889" ht="15.75" customHeight="1"/>
+    <row r="890" ht="15.75" customHeight="1"/>
+    <row r="891" ht="15.75" customHeight="1"/>
+    <row r="892" ht="15.75" customHeight="1"/>
+    <row r="893" ht="15.75" customHeight="1"/>
+    <row r="894" ht="15.75" customHeight="1"/>
+    <row r="895" ht="15.75" customHeight="1"/>
+    <row r="896" ht="15.75" customHeight="1"/>
+    <row r="897" ht="15.75" customHeight="1"/>
+    <row r="898" ht="15.75" customHeight="1"/>
+    <row r="899" ht="15.75" customHeight="1"/>
+    <row r="900" ht="15.75" customHeight="1"/>
+    <row r="901" ht="15.75" customHeight="1"/>
+    <row r="902" ht="15.75" customHeight="1"/>
+    <row r="903" ht="15.75" customHeight="1"/>
+    <row r="904" ht="15.75" customHeight="1"/>
+    <row r="905" ht="15.75" customHeight="1"/>
+    <row r="906" ht="15.75" customHeight="1"/>
+    <row r="907" ht="15.75" customHeight="1"/>
+    <row r="908" ht="15.75" customHeight="1"/>
+    <row r="909" ht="15.75" customHeight="1"/>
+    <row r="910" ht="15.75" customHeight="1"/>
+    <row r="911" ht="15.75" customHeight="1"/>
+    <row r="912" ht="15.75" customHeight="1"/>
+    <row r="913" ht="15.75" customHeight="1"/>
+    <row r="914" ht="15.75" customHeight="1"/>
+    <row r="915" ht="15.75" customHeight="1"/>
+    <row r="916" ht="15.75" customHeight="1"/>
+    <row r="917" ht="15.75" customHeight="1"/>
+    <row r="918" ht="15.75" customHeight="1"/>
+    <row r="919" ht="15.75" customHeight="1"/>
+    <row r="920" ht="15.75" customHeight="1"/>
+    <row r="921" ht="15.75" customHeight="1"/>
+    <row r="922" ht="15.75" customHeight="1"/>
+    <row r="923" ht="15.75" customHeight="1"/>
+    <row r="924" ht="15.75" customHeight="1"/>
+    <row r="925" ht="15.75" customHeight="1"/>
+    <row r="926" ht="15.75" customHeight="1"/>
+    <row r="927" ht="15.75" customHeight="1"/>
+    <row r="928" ht="15.75" customHeight="1"/>
+    <row r="929" ht="15.75" customHeight="1"/>
+    <row r="930" ht="15.75" customHeight="1"/>
+    <row r="931" ht="15.75" customHeight="1"/>
+    <row r="932" ht="15.75" customHeight="1"/>
+    <row r="933" ht="15.75" customHeight="1"/>
+    <row r="934" ht="15.75" customHeight="1"/>
+    <row r="935" ht="15.75" customHeight="1"/>
+    <row r="936" ht="15.75" customHeight="1"/>
+    <row r="937" ht="15.75" customHeight="1"/>
+    <row r="938" ht="15.75" customHeight="1"/>
+    <row r="939" ht="15.75" customHeight="1"/>
+    <row r="940" ht="15.75" customHeight="1"/>
+    <row r="941" ht="15.75" customHeight="1"/>
+    <row r="942" ht="15.75" customHeight="1"/>
+    <row r="943" ht="15.75" customHeight="1"/>
+    <row r="944" ht="15.75" customHeight="1"/>
+    <row r="945" ht="15.75" customHeight="1"/>
+    <row r="946" ht="15.75" customHeight="1"/>
+    <row r="947" ht="15.75" customHeight="1"/>
+    <row r="948" ht="15.75" customHeight="1"/>
+    <row r="949" ht="15.75" customHeight="1"/>
+    <row r="950" ht="15.75" customHeight="1"/>
+    <row r="951" ht="15.75" customHeight="1"/>
+    <row r="952" ht="15.75" customHeight="1"/>
+    <row r="953" ht="15.75" customHeight="1"/>
+    <row r="954" ht="15.75" customHeight="1"/>
+    <row r="955" ht="15.75" customHeight="1"/>
+    <row r="956" ht="15.75" customHeight="1"/>
+    <row r="957" ht="15.75" customHeight="1"/>
+    <row r="958" ht="15.75" customHeight="1"/>
+    <row r="959" ht="15.75" customHeight="1"/>
+    <row r="960" ht="15.75" customHeight="1"/>
+    <row r="961" ht="15.75" customHeight="1"/>
+    <row r="962" ht="15.75" customHeight="1"/>
+    <row r="963" ht="15.75" customHeight="1"/>
+    <row r="964" ht="15.75" customHeight="1"/>
+    <row r="965" ht="15.75" customHeight="1"/>
+    <row r="966" ht="15.75" customHeight="1"/>
+    <row r="967" ht="15.75" customHeight="1"/>
+    <row r="968" ht="15.75" customHeight="1"/>
+    <row r="969" ht="15.75" customHeight="1"/>
+    <row r="970" ht="15.75" customHeight="1"/>
+    <row r="971" ht="15.75" customHeight="1"/>
+    <row r="972" ht="15.75" customHeight="1"/>
+    <row r="973" ht="15.75" customHeight="1"/>
+    <row r="974" ht="15.75" customHeight="1"/>
+    <row r="975" ht="15.75" customHeight="1"/>
+    <row r="976" ht="15.75" customHeight="1"/>
+    <row r="977" ht="15.75" customHeight="1"/>
+    <row r="978" ht="15.75" customHeight="1"/>
+    <row r="979" ht="15.75" customHeight="1"/>
+    <row r="980" ht="15.75" customHeight="1"/>
+    <row r="981" ht="15.75" customHeight="1"/>
+    <row r="982" ht="15.75" customHeight="1"/>
+    <row r="983" ht="15.75" customHeight="1"/>
+    <row r="984" ht="15.75" customHeight="1"/>
+    <row r="985" ht="15.75" customHeight="1"/>
+    <row r="986" ht="15.75" customHeight="1"/>
+    <row r="987" ht="15.75" customHeight="1"/>
+    <row r="988" ht="15.75" customHeight="1"/>
+    <row r="989" ht="15.75" customHeight="1"/>
+    <row r="990" ht="15.75" customHeight="1"/>
+    <row r="991" ht="15.75" customHeight="1"/>
+    <row r="992" ht="15.75" customHeight="1"/>
+    <row r="993" ht="15.75" customHeight="1"/>
+    <row r="994" ht="15.75" customHeight="1"/>
+    <row r="995" ht="15.75" customHeight="1"/>
+    <row r="996" ht="15.75" customHeight="1"/>
+    <row r="997" ht="15.75" customHeight="1"/>
+    <row r="998" ht="15.75" customHeight="1"/>
+    <row r="999" ht="15.75" customHeight="1"/>
+    <row r="1000" ht="15.75" customHeight="1"/>
+    <row r="1001" ht="15.75" customHeight="1"/>
   </sheetData>
   <conditionalFormatting sqref="B2:AZ53">
-    <cfRule type="expression" dxfId="0" priority="8">
+    <cfRule priority="1" dxfId="0" type="expression">
       <formula>B2&lt;&gt;INDIRECT(ADDRESS(MATCH(B$1,$A:$A,0),MATCH($A2,$1:$1,0)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <pageMargins left="0.51180550000000002" right="0.51180550000000002" top="0.78749999999999998" bottom="0.78749999999999998" header="0" footer="0"/>
+  <pageMargins left="0.5118055" right="0.5118055" top="0.7875" bottom="0.7875" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update to OWPick v1.1.2
Correção do modelo de scoring (Meta Strength e Threat Weighting). Meta Strength agora usa estatísticas por role (DPS/TANK/SUP), sigma da winrate bruta e confiança via pickrate (conf = pr/(pr+k0)), com escala final ALPHA = 2.25 - corrige mistura de roles, sigma encolhido e o antigo kappa que encolhia ~99% da winrate observada. Threat Weighting agora usa softplus (w_e = ln(1 + e^raw)) no lugar do piso, preservando a ordenação das ameaças baixas em vez de cravar todas no piso. Removidos o shrinkage antigo e a constante KAPPA_BASE.
</commit_message>
<xml_diff>
--- a/dist/OWPick/_internal/heroes ally.xlsx
+++ b/dist/OWPick/_internal/heroes ally.xlsx
@@ -1,7 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DAVI\Projetos\Overwatch-Best-Picks\"/>
@@ -640,22 +639,22 @@
         <v>-11</v>
       </c>
       <c r="C2" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D2" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="E2" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="F2" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="G2" s="3">
-        <v>-1</v>
+        <v>2</v>
       </c>
       <c r="H2" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I2" s="3">
         <v>-1</v>
@@ -742,10 +741,10 @@
         <v>2</v>
       </c>
       <c r="AK2" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AL2" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AM2" s="3">
         <v>0</v>
@@ -906,7 +905,7 @@
         <v>0</v>
       </c>
       <c r="AL3" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AM3" s="3">
         <v>0</v>
@@ -1386,10 +1385,10 @@
         <v>0</v>
       </c>
       <c r="AK6" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AL6" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AM6" s="3">
         <v>1</v>
@@ -1547,7 +1546,7 @@
         <v>-1</v>
       </c>
       <c r="AK7" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AL7" s="3">
         <v>0</v>
@@ -1711,7 +1710,7 @@
         <v>0</v>
       </c>
       <c r="AL8" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="AM8" s="3">
         <v>1</v>
@@ -1869,10 +1868,10 @@
         <v>0</v>
       </c>
       <c r="AK9" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AL9" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AM9" s="3">
         <v>0</v>
@@ -2191,10 +2190,10 @@
         <v>-1</v>
       </c>
       <c r="AK11" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AL11" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AM11" s="3">
         <v>0</v>
@@ -2355,7 +2354,7 @@
         <v>0</v>
       </c>
       <c r="AL12" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AM12" s="3">
         <v>1</v>
@@ -2516,7 +2515,7 @@
         <v>0</v>
       </c>
       <c r="AL13" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AM13" s="3">
         <v>1</v>
@@ -2677,7 +2676,7 @@
         <v>0</v>
       </c>
       <c r="AL14" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AM14" s="3">
         <v>-1</v>
@@ -2838,7 +2837,7 @@
         <v>0</v>
       </c>
       <c r="AL15" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AM15" s="3">
         <v>0</v>
@@ -2999,7 +2998,7 @@
         <v>0</v>
       </c>
       <c r="AL16" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AM16" s="3">
         <v>-1</v>
@@ -3321,7 +3320,7 @@
         <v>0</v>
       </c>
       <c r="AL18" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AM18" s="3">
         <v>0</v>
@@ -3482,7 +3481,7 @@
         <v>0</v>
       </c>
       <c r="AL19" s="3">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AM19" s="3">
         <v>-1</v>
@@ -3643,7 +3642,7 @@
         <v>0</v>
       </c>
       <c r="AL20" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AM20" s="3">
         <v>1</v>
@@ -3804,7 +3803,7 @@
         <v>0</v>
       </c>
       <c r="AL21" s="3">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AM21" s="3">
         <v>0</v>
@@ -4123,7 +4122,7 @@
         <v>1</v>
       </c>
       <c r="AK23" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AL23" s="3">
         <v>0</v>
@@ -4284,7 +4283,7 @@
         <v>-1</v>
       </c>
       <c r="AK24" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AL24" s="3">
         <v>0</v>
@@ -4445,10 +4444,10 @@
         <v>1</v>
       </c>
       <c r="AK25" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AL25" s="3">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AM25" s="3">
         <v>0</v>
@@ -4770,7 +4769,7 @@
         <v>0</v>
       </c>
       <c r="AL27" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AM27" s="3">
         <v>2</v>
@@ -5092,7 +5091,7 @@
         <v>0</v>
       </c>
       <c r="AL29" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AM29" s="3">
         <v>0</v>
@@ -5250,7 +5249,7 @@
         <v>0</v>
       </c>
       <c r="AK30" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AL30" s="3">
         <v>0</v>
@@ -5414,7 +5413,7 @@
         <v>0</v>
       </c>
       <c r="AL31" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AM31" s="3">
         <v>2</v>
@@ -5575,7 +5574,7 @@
         <v>0</v>
       </c>
       <c r="AL32" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AM32" s="3">
         <v>0</v>
@@ -5897,7 +5896,7 @@
         <v>0</v>
       </c>
       <c r="AL34" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AM34" s="3">
         <v>-1</v>
@@ -6055,7 +6054,7 @@
         <v>0</v>
       </c>
       <c r="AK35" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AL35" s="3">
         <v>0</v>
@@ -6272,7 +6271,7 @@
         <v>36</v>
       </c>
       <c r="B37" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C37" s="3">
         <v>0</v>
@@ -6284,22 +6283,22 @@
         <v>0</v>
       </c>
       <c r="F37" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G37" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H37" s="3">
         <v>0</v>
       </c>
       <c r="I37" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J37" s="3">
         <v>0</v>
       </c>
       <c r="K37" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="L37" s="3">
         <v>0</v>
@@ -6335,13 +6334,13 @@
         <v>0</v>
       </c>
       <c r="W37" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="X37" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y37" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z37" s="3">
         <v>0</v>
@@ -6356,13 +6355,13 @@
         <v>0</v>
       </c>
       <c r="AD37" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AE37" s="3">
         <v>0</v>
       </c>
       <c r="AF37" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AG37" s="3">
         <v>0</v>
@@ -6371,7 +6370,7 @@
         <v>0</v>
       </c>
       <c r="AI37" s="3">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AJ37" s="3">
         <v>0</v>
@@ -6383,13 +6382,13 @@
         <v>0</v>
       </c>
       <c r="AM37" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AN37" s="3">
         <v>0</v>
       </c>
       <c r="AO37" s="3">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AP37" s="3">
         <v>0</v>
@@ -6416,7 +6415,7 @@
         <v>0</v>
       </c>
       <c r="AX37" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AY37" s="3">
         <v>0</v>
@@ -6436,94 +6435,94 @@
         <v>0</v>
       </c>
       <c r="C38" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="D38" s="3">
         <v>-1</v>
       </c>
       <c r="E38" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F38" s="3">
         <v>0</v>
       </c>
       <c r="G38" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H38" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="I38" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="J38" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K38" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="L38" s="3">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="M38" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N38" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O38" s="3">
         <v>0</v>
       </c>
       <c r="P38" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q38" s="3">
         <v>0</v>
       </c>
       <c r="R38" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="S38" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="T38" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="U38" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="V38" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W38" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X38" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Y38" s="3">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="Z38" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA38" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AB38" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AC38" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AD38" s="3">
         <v>0</v>
       </c>
       <c r="AE38" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF38" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG38" s="3">
         <v>0</v>
@@ -6532,10 +6531,10 @@
         <v>0</v>
       </c>
       <c r="AI38" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AJ38" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AK38" s="3">
         <v>0</v>
@@ -6547,7 +6546,7 @@
         <v>0</v>
       </c>
       <c r="AN38" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AO38" s="3">
         <v>0</v>
@@ -6556,22 +6555,22 @@
         <v>0</v>
       </c>
       <c r="AQ38" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AR38" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS38" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AT38" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU38" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AV38" s="3">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AW38" s="3">
         <v>0</v>
@@ -6580,13 +6579,13 @@
         <v>0</v>
       </c>
       <c r="AY38" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AZ38" s="3">
         <v>0</v>
       </c>
       <c r="BA38" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="39" ht="15.75" customHeight="1">
@@ -6699,10 +6698,10 @@
         <v>1</v>
       </c>
       <c r="AK39" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AL39" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AM39" s="3">
         <v>-11</v>
@@ -6863,7 +6862,7 @@
         <v>0</v>
       </c>
       <c r="AL40" s="3">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="AM40" s="3">
         <v>1</v>
@@ -7021,10 +7020,10 @@
         <v>-1</v>
       </c>
       <c r="AK41" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AL41" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AM41" s="3">
         <v>2</v>
@@ -7185,7 +7184,7 @@
         <v>0</v>
       </c>
       <c r="AL42" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AM42" s="3">
         <v>1</v>
@@ -7507,7 +7506,7 @@
         <v>0</v>
       </c>
       <c r="AL44" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AM44" s="3">
         <v>0</v>
@@ -7668,7 +7667,7 @@
         <v>0</v>
       </c>
       <c r="AL45" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AM45" s="3">
         <v>0</v>
@@ -7829,7 +7828,7 @@
         <v>0</v>
       </c>
       <c r="AL46" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AM46" s="3">
         <v>0</v>
@@ -7990,7 +7989,7 @@
         <v>0</v>
       </c>
       <c r="AL47" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AM47" s="3">
         <v>0</v>
@@ -8470,7 +8469,7 @@
         <v>0</v>
       </c>
       <c r="AK50" s="3">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AL50" s="3">
         <v>0</v>
@@ -8634,7 +8633,7 @@
         <v>0</v>
       </c>
       <c r="AL51" s="3">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AM51" s="3">
         <v>0</v>
@@ -8956,7 +8955,7 @@
         <v>0</v>
       </c>
       <c r="AL53" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AM53" s="3">
         <v>2</v>

</xml_diff>